<commit_message>
Mark whether Zebra scanner prices include a USB cable
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0164u4m2HzVL7yDN6jZnxUBp
</commit_message>
<xml_diff>
--- a/output/지브라_스캐너_옵션추가.xlsx
+++ b/output/지브라_스캐너_옵션추가.xlsx
@@ -705,7 +705,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -766,6 +766,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="164" fontId="25" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment vertical="center"/>
@@ -9694,7 +9697,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P31"/>
+  <dimension ref="A1:Q31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="16.375" customWidth="1" style="16" min="2" max="2"/>
@@ -9706,6 +9709,7 @@
     <col width="18.125" customWidth="1" style="16" min="13" max="13"/>
     <col width="19.875" customWidth="1" style="16" min="14" max="14"/>
     <col width="48" customWidth="1" style="16" min="16" max="16"/>
+    <col width="20" customWidth="1" style="16" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1" ht="18.75" customHeight="1" s="16">
@@ -9781,6 +9785,11 @@
           <t>옵션(추가금액)</t>
         </is>
       </c>
+      <c r="Q1" s="4" t="inlineStr">
+        <is>
+          <t>USB케이블 포함(O/X)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="n">
@@ -9813,6 +9822,11 @@
 본체만(케이블없음) (+0원)</t>
         </is>
       </c>
+      <c r="Q2" s="21" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="n">
@@ -9844,7 +9858,7 @@
         <f>J3/110%</f>
         <v/>
       </c>
-      <c r="L3" s="21" t="inlineStr">
+      <c r="L3" s="22" t="inlineStr">
         <is>
           <t>제벡스코리아</t>
         </is>
@@ -9865,6 +9879,11 @@
 본체+크래들만(케이블없음) (+0원)</t>
         </is>
       </c>
+      <c r="Q3" s="21" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="n">
@@ -9896,7 +9915,7 @@
         <f>J4/110%</f>
         <v/>
       </c>
-      <c r="L4" s="21" t="inlineStr">
+      <c r="L4" s="22" t="inlineStr">
         <is>
           <t>마켓굿초이스</t>
         </is>
@@ -9921,6 +9940,11 @@
 본체만(케이블없음) / 스탠드거치대 (+55,000원)</t>
         </is>
       </c>
+      <c r="Q4" s="21" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="n">
@@ -9952,7 +9976,7 @@
         <f>J5/110%</f>
         <v/>
       </c>
-      <c r="L5" s="21" t="inlineStr">
+      <c r="L5" s="22" t="inlineStr">
         <is>
           <t>바코드다판다</t>
         </is>
@@ -9972,6 +9996,11 @@
 본체만 (+0원)</t>
         </is>
       </c>
+      <c r="Q5" s="21" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="n">
@@ -10003,7 +10032,7 @@
         <f>J6/110%</f>
         <v/>
       </c>
-      <c r="L6" s="21" t="inlineStr">
+      <c r="L6" s="22" t="inlineStr">
         <is>
           <t>에이치에스스토어(usb제외)</t>
         </is>
@@ -10028,6 +10057,11 @@
 본체만(케이블없음) / 스탠드거치대 (+55,000원)</t>
         </is>
       </c>
+      <c r="Q6" s="21" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="n">
@@ -10056,7 +10090,7 @@
         <f>J7/110%</f>
         <v/>
       </c>
-      <c r="L7" s="21" t="inlineStr">
+      <c r="L7" s="22" t="inlineStr">
         <is>
           <t>컴엔더</t>
         </is>
@@ -10073,6 +10107,11 @@
         <is>
           <t>정품직선형USB (+16,500원)
 RS232C (+24,200원)</t>
+        </is>
+      </c>
+      <c r="Q7" s="21" t="inlineStr">
+        <is>
+          <t>X</t>
         </is>
       </c>
     </row>
@@ -10106,7 +10145,7 @@
         <f>J8/110%</f>
         <v/>
       </c>
-      <c r="L8" s="21" t="inlineStr">
+      <c r="L8" s="22" t="inlineStr">
         <is>
           <t>유니정보</t>
         </is>
@@ -10122,6 +10161,11 @@
       <c r="P8" s="20" t="inlineStr">
         <is>
           <t>USB (+0원)</t>
+        </is>
+      </c>
+      <c r="Q8" s="21" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
     </row>
@@ -10155,7 +10199,7 @@
         <f>J9/110%</f>
         <v/>
       </c>
-      <c r="L9" s="21" t="inlineStr">
+      <c r="L9" s="22" t="inlineStr">
         <is>
           <t>더원시스</t>
         </is>
@@ -10172,6 +10216,11 @@
         <is>
           <t>USB (+0원)
 RS232C (+24,200원)</t>
+        </is>
+      </c>
+      <c r="Q9" s="21" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
     </row>
@@ -10202,7 +10251,7 @@
         <f>J10/110%</f>
         <v/>
       </c>
-      <c r="L10" s="21" t="inlineStr">
+      <c r="L10" s="22" t="inlineStr">
         <is>
           <t>착한라벨</t>
         </is>
@@ -10219,6 +10268,11 @@
         <is>
           <t>USB (+0원)
 RS232C (+33,000원)</t>
+        </is>
+      </c>
+      <c r="Q10" s="21" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
     </row>
@@ -10252,7 +10306,7 @@
         <f>J11/110%</f>
         <v/>
       </c>
-      <c r="L11" s="22" t="inlineStr">
+      <c r="L11" s="23" t="inlineStr">
         <is>
           <t>디앤에스테크(USB미포함)</t>
         </is>
@@ -10272,6 +10326,11 @@
 RS232C (+24,200원)</t>
         </is>
       </c>
+      <c r="Q11" s="21" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="0" t="n">
@@ -10303,7 +10362,7 @@
         <f>J12/110%</f>
         <v/>
       </c>
-      <c r="L12" s="21" t="inlineStr">
+      <c r="L12" s="22" t="inlineStr">
         <is>
           <t>유니정보</t>
         </is>
@@ -10319,6 +10378,11 @@
       <c r="P12" t="inlineStr">
         <is>
           <t>옵션 정보 없음(상품 엑셀에 미포함)</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>확인필요</t>
         </is>
       </c>
     </row>
@@ -10352,7 +10416,7 @@
         <f>J13/110%</f>
         <v/>
       </c>
-      <c r="L13" s="21" t="inlineStr">
+      <c r="L13" s="22" t="inlineStr">
         <is>
           <t>코스모스몰</t>
         </is>
@@ -10368,6 +10432,11 @@
       <c r="P13" s="20" t="inlineStr">
         <is>
           <t>2D (+0원)</t>
+        </is>
+      </c>
+      <c r="Q13" s="21" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -10401,7 +10470,7 @@
         <f>J14/110%</f>
         <v/>
       </c>
-      <c r="L14" s="21" t="inlineStr">
+      <c r="L14" s="22" t="inlineStr">
         <is>
           <t>더원시스</t>
         </is>
@@ -10422,6 +10491,11 @@
 HD버전+RS232C케이블 (+275,000원)</t>
         </is>
       </c>
+      <c r="Q14" s="21" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="0" t="n">
@@ -10453,7 +10527,7 @@
         <f>J15/110%</f>
         <v/>
       </c>
-      <c r="L15" s="21" t="inlineStr">
+      <c r="L15" s="22" t="inlineStr">
         <is>
           <t>더원시스</t>
         </is>
@@ -10478,6 +10552,11 @@
 본체만(케이블없음) / 스탠드거치대 (+55,000원)</t>
         </is>
       </c>
+      <c r="Q15" s="21" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="0" t="n">
@@ -10509,7 +10588,7 @@
         <f>J16/110%</f>
         <v/>
       </c>
-      <c r="L16" s="21" t="inlineStr">
+      <c r="L16" s="22" t="inlineStr">
         <is>
           <t>코스모스몰</t>
         </is>
@@ -10526,6 +10605,11 @@
         <is>
           <t>RS232C (+24,200원)
 USB (+0원)</t>
+        </is>
+      </c>
+      <c r="Q16" s="21" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
     </row>
@@ -10556,7 +10640,7 @@
         <f>J17/110%</f>
         <v/>
       </c>
-      <c r="L17" s="21" t="inlineStr">
+      <c r="L17" s="22" t="inlineStr">
         <is>
           <t>코스모스몰</t>
         </is>
@@ -10573,6 +10657,11 @@
         <is>
           <t>RS232C (+24,200원)
 USB (+0원)</t>
+        </is>
+      </c>
+      <c r="Q17" s="21" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
     </row>
@@ -10606,7 +10695,7 @@
         <f>J18/110%</f>
         <v/>
       </c>
-      <c r="L18" s="21" t="inlineStr">
+      <c r="L18" s="22" t="inlineStr">
         <is>
           <t>바코드랩</t>
         </is>
@@ -10622,6 +10711,11 @@
       <c r="P18" s="20" t="inlineStr">
         <is>
           <t>USB (+0원)</t>
+        </is>
+      </c>
+      <c r="Q18" s="21" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
     </row>
@@ -10655,7 +10749,7 @@
         <f>J19/110%</f>
         <v/>
       </c>
-      <c r="L19" s="21" t="inlineStr">
+      <c r="L19" s="22" t="inlineStr">
         <is>
           <t>바코드랩</t>
         </is>
@@ -10671,6 +10765,11 @@
       <c r="P19" s="20" t="inlineStr">
         <is>
           <t>USB (+0원)</t>
+        </is>
+      </c>
+      <c r="Q19" s="21" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
     </row>
@@ -10701,7 +10800,7 @@
         <f>J20/110%</f>
         <v/>
       </c>
-      <c r="L20" s="21" t="inlineStr">
+      <c r="L20" s="22" t="inlineStr">
         <is>
           <t>코스모스몰</t>
         </is>
@@ -10718,6 +10817,11 @@
         <is>
           <t>USB (+0원)
 RS232C (+24,200원)</t>
+        </is>
+      </c>
+      <c r="Q20" s="21" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
     </row>
@@ -10748,7 +10852,7 @@
         <f>J21/110%</f>
         <v/>
       </c>
-      <c r="L21" s="21" t="inlineStr">
+      <c r="L21" s="22" t="inlineStr">
         <is>
           <t>유니정보,착한라벨,우주사무기</t>
         </is>
@@ -10765,6 +10869,11 @@
         <is>
           <t>RS232C (+49,500원)
 USB (+0원)</t>
+        </is>
+      </c>
+      <c r="Q21" s="21" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
     </row>
@@ -10798,7 +10907,7 @@
         <f>J22/110%</f>
         <v/>
       </c>
-      <c r="L22" s="21" t="inlineStr">
+      <c r="L22" s="22" t="inlineStr">
         <is>
           <t>코스모스전문몰</t>
         </is>
@@ -10819,6 +10928,11 @@
 RS232C (+24,200원)</t>
         </is>
       </c>
+      <c r="Q22" s="21" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="0" t="n">
@@ -10850,7 +10964,7 @@
         <f>J23/110%</f>
         <v/>
       </c>
-      <c r="L23" s="21" t="inlineStr">
+      <c r="L23" s="22" t="inlineStr">
         <is>
           <t>코스모스몰,더원시스</t>
         </is>
@@ -10866,6 +10980,11 @@
       <c r="P23" s="20" t="inlineStr">
         <is>
           <t>USB (+0원)</t>
+        </is>
+      </c>
+      <c r="Q23" s="21" t="inlineStr">
+        <is>
+          <t>O</t>
         </is>
       </c>
     </row>
@@ -10892,7 +11011,7 @@
       </c>
       <c r="J24" s="19" t="n"/>
       <c r="K24" s="17" t="n"/>
-      <c r="L24" s="21" t="n"/>
+      <c r="L24" s="22" t="n"/>
       <c r="M24" s="3" t="n"/>
       <c r="N24" s="3" t="n"/>
       <c r="O24" t="inlineStr">
@@ -10908,6 +11027,11 @@
 본체만(케이블없음) (+0원)</t>
         </is>
       </c>
+      <c r="Q24" s="21" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="0" t="n">
@@ -10932,7 +11056,7 @@
       </c>
       <c r="J25" s="19" t="n"/>
       <c r="K25" s="17" t="n"/>
-      <c r="L25" s="21" t="n"/>
+      <c r="L25" s="22" t="n"/>
       <c r="M25" s="3" t="n"/>
       <c r="N25" s="3" t="n"/>
       <c r="O25" t="inlineStr">
@@ -10948,6 +11072,11 @@
 본체+크래들만(케이블없음) (+0원)</t>
         </is>
       </c>
+      <c r="Q25" s="21" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="0" t="n">
@@ -10972,7 +11101,7 @@
       </c>
       <c r="J26" s="19" t="n"/>
       <c r="K26" s="17" t="n"/>
-      <c r="L26" s="21" t="n"/>
+      <c r="L26" s="22" t="n"/>
       <c r="M26" s="3" t="n"/>
       <c r="N26" s="3" t="n"/>
       <c r="O26" t="inlineStr">
@@ -10988,6 +11117,11 @@
 본체+크래들만(케이블없음) (+0원)</t>
         </is>
       </c>
+      <c r="Q26" s="21" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="0" t="n">
@@ -11012,7 +11146,7 @@
       </c>
       <c r="J27" s="19" t="n"/>
       <c r="K27" s="17" t="n"/>
-      <c r="L27" s="21" t="n"/>
+      <c r="L27" s="22" t="n"/>
       <c r="M27" s="3" t="n"/>
       <c r="N27" s="3" t="n"/>
       <c r="O27" t="inlineStr">
@@ -11025,6 +11159,11 @@
           <t>링트리거 (+0원)</t>
         </is>
       </c>
+      <c r="Q27" s="21" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="0" t="n">
@@ -11049,7 +11188,7 @@
       </c>
       <c r="J28" s="19" t="n"/>
       <c r="K28" s="17" t="n"/>
-      <c r="L28" s="21" t="n"/>
+      <c r="L28" s="22" t="n"/>
       <c r="M28" s="3" t="n"/>
       <c r="N28" s="3" t="n"/>
       <c r="O28" t="inlineStr">
@@ -11062,6 +11201,11 @@
           <t>본체 (+0원)</t>
         </is>
       </c>
+      <c r="Q28" s="21" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="0" t="n">
@@ -11086,7 +11230,7 @@
       </c>
       <c r="J29" s="19" t="n"/>
       <c r="K29" s="17" t="n"/>
-      <c r="L29" s="21" t="n"/>
+      <c r="L29" s="22" t="n"/>
       <c r="M29" s="3" t="n"/>
       <c r="N29" s="3" t="n"/>
       <c r="O29" t="inlineStr">
@@ -11099,6 +11243,11 @@
           <t>본체 (+0원)</t>
         </is>
       </c>
+      <c r="Q29" s="21" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="0" t="n">
@@ -11123,7 +11272,7 @@
       </c>
       <c r="J30" s="19" t="n"/>
       <c r="K30" s="17" t="n"/>
-      <c r="L30" s="21" t="n"/>
+      <c r="L30" s="22" t="n"/>
       <c r="M30" s="3" t="n"/>
       <c r="N30" s="3" t="n"/>
       <c r="O30" t="inlineStr">
@@ -11136,6 +11285,11 @@
           <t>본체 (+0원)</t>
         </is>
       </c>
+      <c r="Q30" s="21" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="0" t="n">
@@ -11160,7 +11314,7 @@
       </c>
       <c r="J31" s="19" t="n"/>
       <c r="K31" s="17" t="n"/>
-      <c r="L31" s="21" t="n"/>
+      <c r="L31" s="22" t="n"/>
       <c r="M31" s="3" t="n"/>
       <c r="N31" s="3" t="n"/>
       <c r="O31" t="inlineStr">
@@ -11171,6 +11325,11 @@
       <c r="P31" s="20" t="inlineStr">
         <is>
           <t>본체 (+0원)</t>
+        </is>
+      </c>
+      <c r="Q31" s="21" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -11398,35 +11557,35 @@
           <t xml:space="preserve"> 키패드(핸드헬드)</t>
         </is>
       </c>
-      <c r="D4" s="23" t="n">
+      <c r="D4" s="24" t="n">
         <v>1840000</v>
       </c>
-      <c r="E4" s="23">
+      <c r="E4" s="24">
         <f>D4*1.1</f>
         <v/>
       </c>
-      <c r="F4" s="23" t="n">
+      <c r="F4" s="24" t="n">
         <v>2640000</v>
       </c>
-      <c r="G4" s="23">
+      <c r="G4" s="24">
         <f>F4/110%</f>
         <v/>
       </c>
-      <c r="H4" s="24" t="n">
+      <c r="H4" s="25" t="n">
         <v>2500000</v>
       </c>
-      <c r="I4" s="24">
+      <c r="I4" s="25">
         <f>ROUND(H4*1.1/0.95,-1)</f>
         <v/>
       </c>
-      <c r="J4" s="23" t="n">
+      <c r="J4" s="24" t="n">
         <v>2640000</v>
       </c>
-      <c r="K4" s="23">
+      <c r="K4" s="24">
         <f>J4/1.1</f>
         <v/>
       </c>
-      <c r="L4" s="23" t="inlineStr">
+      <c r="L4" s="24" t="inlineStr">
         <is>
           <t>코스모스몰</t>
         </is>
@@ -11613,32 +11772,32 @@
           <t xml:space="preserve"> 프리미엄풀터치</t>
         </is>
       </c>
-      <c r="D8" s="23" t="n">
+      <c r="D8" s="24" t="n">
         <v>2500000</v>
       </c>
-      <c r="E8" s="23">
+      <c r="E8" s="24">
         <f>D8*1.1</f>
         <v/>
       </c>
-      <c r="F8" s="23" t="n">
+      <c r="F8" s="24" t="n">
         <v>2640000</v>
       </c>
-      <c r="G8" s="24" t="n"/>
-      <c r="H8" s="24" t="n">
+      <c r="G8" s="25" t="n"/>
+      <c r="H8" s="25" t="n">
         <v>3000000</v>
       </c>
-      <c r="I8" s="24">
+      <c r="I8" s="25">
         <f>ROUND(H8*1.1/0.95,-1)</f>
         <v/>
       </c>
-      <c r="J8" s="23" t="n">
+      <c r="J8" s="24" t="n">
         <v>2577960</v>
       </c>
-      <c r="K8" s="23">
+      <c r="K8" s="24">
         <f>J8/1.1</f>
         <v/>
       </c>
-      <c r="L8" s="23" t="inlineStr">
+      <c r="L8" s="24" t="inlineStr">
         <is>
           <t>솔바텍지마켓</t>
         </is>
@@ -11717,30 +11876,30 @@
           <t xml:space="preserve"> 키패드(핸드헬드)</t>
         </is>
       </c>
-      <c r="D10" s="23" t="n">
+      <c r="D10" s="24" t="n">
         <v>1490000</v>
       </c>
-      <c r="E10" s="23">
+      <c r="E10" s="24">
         <f>D10*1.1</f>
         <v/>
       </c>
-      <c r="F10" s="23" t="n">
+      <c r="F10" s="24" t="n">
         <v>2750000</v>
       </c>
-      <c r="G10" s="23">
+      <c r="G10" s="24">
         <f>F10/110%</f>
         <v/>
       </c>
-      <c r="H10" s="23" t="n"/>
-      <c r="I10" s="23" t="n"/>
-      <c r="J10" s="23" t="n">
+      <c r="H10" s="24" t="n"/>
+      <c r="I10" s="24" t="n"/>
+      <c r="J10" s="24" t="n">
         <v>2750000</v>
       </c>
-      <c r="K10" s="23">
+      <c r="K10" s="24">
         <f>J10/1.1</f>
         <v/>
       </c>
-      <c r="L10" s="23" t="inlineStr">
+      <c r="L10" s="24" t="inlineStr">
         <is>
           <t>코스모스몰,더원시스</t>
         </is>
@@ -11911,7 +12070,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="I18" s="25" t="n"/>
+      <c r="I18" s="26" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -11989,7 +12148,7 @@
           <t>LS2208 SR</t>
         </is>
       </c>
-      <c r="C2" s="26">
+      <c r="C2" s="27">
         <f>'지브라-스캐너'!F2</f>
         <v/>
       </c>
@@ -12003,14 +12162,14 @@
           <t>정품직선형USB</t>
         </is>
       </c>
-      <c r="F2" s="26" t="n">
+      <c r="F2" s="27" t="n">
         <v>18000</v>
       </c>
-      <c r="G2" s="26">
+      <c r="G2" s="27">
         <f>C2+F2</f>
         <v/>
       </c>
-      <c r="H2" s="26">
+      <c r="H2" s="27">
         <f>G2/110%</f>
         <v/>
       </c>
@@ -12024,7 +12183,7 @@
           <t>LS2208 SR</t>
         </is>
       </c>
-      <c r="C3" s="26">
+      <c r="C3" s="27">
         <f>'지브라-스캐너'!F2</f>
         <v/>
       </c>
@@ -12038,14 +12197,14 @@
           <t>코일형USB</t>
         </is>
       </c>
-      <c r="F3" s="26" t="n">
+      <c r="F3" s="27" t="n">
         <v>18000</v>
       </c>
-      <c r="G3" s="26">
+      <c r="G3" s="27">
         <f>C3+F3</f>
         <v/>
       </c>
-      <c r="H3" s="26">
+      <c r="H3" s="27">
         <f>G3/110%</f>
         <v/>
       </c>
@@ -12059,7 +12218,7 @@
           <t>LS2208 SR</t>
         </is>
       </c>
-      <c r="C4" s="26">
+      <c r="C4" s="27">
         <f>'지브라-스캐너'!F2</f>
         <v/>
       </c>
@@ -12073,14 +12232,14 @@
           <t>RS232C</t>
         </is>
       </c>
-      <c r="F4" s="26" t="n">
+      <c r="F4" s="27" t="n">
         <v>24200</v>
       </c>
-      <c r="G4" s="26">
+      <c r="G4" s="27">
         <f>C4+F4</f>
         <v/>
       </c>
-      <c r="H4" s="26">
+      <c r="H4" s="27">
         <f>G4/110%</f>
         <v/>
       </c>
@@ -12094,7 +12253,7 @@
           <t>LS2208 SR</t>
         </is>
       </c>
-      <c r="C5" s="26">
+      <c r="C5" s="27">
         <f>'지브라-스캐너'!F2</f>
         <v/>
       </c>
@@ -12108,14 +12267,14 @@
           <t>본체만(케이블없음)</t>
         </is>
       </c>
-      <c r="F5" s="26" t="n">
+      <c r="F5" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="G5" s="26">
+      <c r="G5" s="27">
         <f>C5+F5</f>
         <v/>
       </c>
-      <c r="H5" s="26">
+      <c r="H5" s="27">
         <f>G5/110%</f>
         <v/>
       </c>
@@ -12129,7 +12288,7 @@
           <t>DS2278</t>
         </is>
       </c>
-      <c r="C6" s="26">
+      <c r="C6" s="27">
         <f>'지브라-스캐너'!F3</f>
         <v/>
       </c>
@@ -12143,14 +12302,14 @@
           <t>정품직선형USB</t>
         </is>
       </c>
-      <c r="F6" s="26" t="n">
+      <c r="F6" s="27" t="n">
         <v>18000</v>
       </c>
-      <c r="G6" s="26">
+      <c r="G6" s="27">
         <f>C6+F6</f>
         <v/>
       </c>
-      <c r="H6" s="26">
+      <c r="H6" s="27">
         <f>G6/110%</f>
         <v/>
       </c>
@@ -12164,7 +12323,7 @@
           <t>DS2278</t>
         </is>
       </c>
-      <c r="C7" s="26">
+      <c r="C7" s="27">
         <f>'지브라-스캐너'!F3</f>
         <v/>
       </c>
@@ -12178,14 +12337,14 @@
           <t>코일형USB</t>
         </is>
       </c>
-      <c r="F7" s="26" t="n">
+      <c r="F7" s="27" t="n">
         <v>18000</v>
       </c>
-      <c r="G7" s="26">
+      <c r="G7" s="27">
         <f>C7+F7</f>
         <v/>
       </c>
-      <c r="H7" s="26">
+      <c r="H7" s="27">
         <f>G7/110%</f>
         <v/>
       </c>
@@ -12199,7 +12358,7 @@
           <t>DS2278</t>
         </is>
       </c>
-      <c r="C8" s="26">
+      <c r="C8" s="27">
         <f>'지브라-스캐너'!F3</f>
         <v/>
       </c>
@@ -12213,14 +12372,14 @@
           <t>RS232C</t>
         </is>
       </c>
-      <c r="F8" s="26" t="n">
+      <c r="F8" s="27" t="n">
         <v>24200</v>
       </c>
-      <c r="G8" s="26">
+      <c r="G8" s="27">
         <f>C8+F8</f>
         <v/>
       </c>
-      <c r="H8" s="26">
+      <c r="H8" s="27">
         <f>G8/110%</f>
         <v/>
       </c>
@@ -12234,7 +12393,7 @@
           <t>DS2278</t>
         </is>
       </c>
-      <c r="C9" s="26">
+      <c r="C9" s="27">
         <f>'지브라-스캐너'!F3</f>
         <v/>
       </c>
@@ -12248,14 +12407,14 @@
           <t>본체+크래들만(케이블없음)</t>
         </is>
       </c>
-      <c r="F9" s="26" t="n">
+      <c r="F9" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="G9" s="26">
+      <c r="G9" s="27">
         <f>C9+F9</f>
         <v/>
       </c>
-      <c r="H9" s="26">
+      <c r="H9" s="27">
         <f>G9/110%</f>
         <v/>
       </c>
@@ -12269,7 +12428,7 @@
           <t>DS2208</t>
         </is>
       </c>
-      <c r="C10" s="26">
+      <c r="C10" s="27">
         <f>'지브라-스캐너'!F4</f>
         <v/>
       </c>
@@ -12283,14 +12442,14 @@
           <t>정품직선형USB / 선택안함</t>
         </is>
       </c>
-      <c r="F10" s="26" t="n">
+      <c r="F10" s="27" t="n">
         <v>18000</v>
       </c>
-      <c r="G10" s="26">
+      <c r="G10" s="27">
         <f>C10+F10</f>
         <v/>
       </c>
-      <c r="H10" s="26">
+      <c r="H10" s="27">
         <f>G10/110%</f>
         <v/>
       </c>
@@ -12304,7 +12463,7 @@
           <t>DS2208</t>
         </is>
       </c>
-      <c r="C11" s="26">
+      <c r="C11" s="27">
         <f>'지브라-스캐너'!F4</f>
         <v/>
       </c>
@@ -12318,14 +12477,14 @@
           <t>정품직선형USB / 스탠드거치대</t>
         </is>
       </c>
-      <c r="F11" s="26" t="n">
+      <c r="F11" s="27" t="n">
         <v>73000</v>
       </c>
-      <c r="G11" s="26">
+      <c r="G11" s="27">
         <f>C11+F11</f>
         <v/>
       </c>
-      <c r="H11" s="26">
+      <c r="H11" s="27">
         <f>G11/110%</f>
         <v/>
       </c>
@@ -12339,7 +12498,7 @@
           <t>DS2208</t>
         </is>
       </c>
-      <c r="C12" s="26">
+      <c r="C12" s="27">
         <f>'지브라-스캐너'!F4</f>
         <v/>
       </c>
@@ -12353,14 +12512,14 @@
           <t>RS232C / 선택안함</t>
         </is>
       </c>
-      <c r="F12" s="26" t="n">
+      <c r="F12" s="27" t="n">
         <v>24200</v>
       </c>
-      <c r="G12" s="26">
+      <c r="G12" s="27">
         <f>C12+F12</f>
         <v/>
       </c>
-      <c r="H12" s="26">
+      <c r="H12" s="27">
         <f>G12/110%</f>
         <v/>
       </c>
@@ -12374,7 +12533,7 @@
           <t>DS2208</t>
         </is>
       </c>
-      <c r="C13" s="26">
+      <c r="C13" s="27">
         <f>'지브라-스캐너'!F4</f>
         <v/>
       </c>
@@ -12388,14 +12547,14 @@
           <t>RS232C / 스탠드거치대</t>
         </is>
       </c>
-      <c r="F13" s="26" t="n">
+      <c r="F13" s="27" t="n">
         <v>79200</v>
       </c>
-      <c r="G13" s="26">
+      <c r="G13" s="27">
         <f>C13+F13</f>
         <v/>
       </c>
-      <c r="H13" s="26">
+      <c r="H13" s="27">
         <f>G13/110%</f>
         <v/>
       </c>
@@ -12409,7 +12568,7 @@
           <t>DS2208</t>
         </is>
       </c>
-      <c r="C14" s="26">
+      <c r="C14" s="27">
         <f>'지브라-스캐너'!F4</f>
         <v/>
       </c>
@@ -12423,14 +12582,14 @@
           <t>코일형USB / 선택안함</t>
         </is>
       </c>
-      <c r="F14" s="26" t="n">
+      <c r="F14" s="27" t="n">
         <v>18000</v>
       </c>
-      <c r="G14" s="26">
+      <c r="G14" s="27">
         <f>C14+F14</f>
         <v/>
       </c>
-      <c r="H14" s="26">
+      <c r="H14" s="27">
         <f>G14/110%</f>
         <v/>
       </c>
@@ -12444,7 +12603,7 @@
           <t>DS2208</t>
         </is>
       </c>
-      <c r="C15" s="26">
+      <c r="C15" s="27">
         <f>'지브라-스캐너'!F4</f>
         <v/>
       </c>
@@ -12458,14 +12617,14 @@
           <t>코일형USB / 스탠드거치대</t>
         </is>
       </c>
-      <c r="F15" s="26" t="n">
+      <c r="F15" s="27" t="n">
         <v>73000</v>
       </c>
-      <c r="G15" s="26">
+      <c r="G15" s="27">
         <f>C15+F15</f>
         <v/>
       </c>
-      <c r="H15" s="26">
+      <c r="H15" s="27">
         <f>G15/110%</f>
         <v/>
       </c>
@@ -12479,7 +12638,7 @@
           <t>DS2208</t>
         </is>
       </c>
-      <c r="C16" s="26">
+      <c r="C16" s="27">
         <f>'지브라-스캐너'!F4</f>
         <v/>
       </c>
@@ -12493,14 +12652,14 @@
           <t>본체만(케이블없음) / 선택안함</t>
         </is>
       </c>
-      <c r="F16" s="26" t="n">
+      <c r="F16" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="G16" s="26">
+      <c r="G16" s="27">
         <f>C16+F16</f>
         <v/>
       </c>
-      <c r="H16" s="26">
+      <c r="H16" s="27">
         <f>G16/110%</f>
         <v/>
       </c>
@@ -12514,7 +12673,7 @@
           <t>DS2208</t>
         </is>
       </c>
-      <c r="C17" s="26">
+      <c r="C17" s="27">
         <f>'지브라-스캐너'!F4</f>
         <v/>
       </c>
@@ -12528,14 +12687,14 @@
           <t>본체만(케이블없음) / 스탠드거치대</t>
         </is>
       </c>
-      <c r="F17" s="26" t="n">
+      <c r="F17" s="27" t="n">
         <v>55000</v>
       </c>
-      <c r="G17" s="26">
+      <c r="G17" s="27">
         <f>C17+F17</f>
         <v/>
       </c>
-      <c r="H17" s="26">
+      <c r="H17" s="27">
         <f>G17/110%</f>
         <v/>
       </c>
@@ -12549,7 +12708,7 @@
           <t>DS8108</t>
         </is>
       </c>
-      <c r="C18" s="26">
+      <c r="C18" s="27">
         <f>'지브라-스캐너'!F5</f>
         <v/>
       </c>
@@ -12563,14 +12722,14 @@
           <t>정품직선형USB</t>
         </is>
       </c>
-      <c r="F18" s="26" t="n">
+      <c r="F18" s="27" t="n">
         <v>16500</v>
       </c>
-      <c r="G18" s="26">
+      <c r="G18" s="27">
         <f>C18+F18</f>
         <v/>
       </c>
-      <c r="H18" s="26">
+      <c r="H18" s="27">
         <f>G18/110%</f>
         <v/>
       </c>
@@ -12584,7 +12743,7 @@
           <t>DS8108</t>
         </is>
       </c>
-      <c r="C19" s="26">
+      <c r="C19" s="27">
         <f>'지브라-스캐너'!F5</f>
         <v/>
       </c>
@@ -12598,14 +12757,14 @@
           <t>RS232C</t>
         </is>
       </c>
-      <c r="F19" s="26" t="n">
+      <c r="F19" s="27" t="n">
         <v>24200</v>
       </c>
-      <c r="G19" s="26">
+      <c r="G19" s="27">
         <f>C19+F19</f>
         <v/>
       </c>
-      <c r="H19" s="26">
+      <c r="H19" s="27">
         <f>G19/110%</f>
         <v/>
       </c>
@@ -12619,7 +12778,7 @@
           <t>DS8108</t>
         </is>
       </c>
-      <c r="C20" s="26">
+      <c r="C20" s="27">
         <f>'지브라-스캐너'!F5</f>
         <v/>
       </c>
@@ -12633,14 +12792,14 @@
           <t>본체만</t>
         </is>
       </c>
-      <c r="F20" s="26" t="n">
+      <c r="F20" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="G20" s="26">
+      <c r="G20" s="27">
         <f>C20+F20</f>
         <v/>
       </c>
-      <c r="H20" s="26">
+      <c r="H20" s="27">
         <f>G20/110%</f>
         <v/>
       </c>
@@ -12654,7 +12813,7 @@
           <t>DS4608 SR</t>
         </is>
       </c>
-      <c r="C21" s="26">
+      <c r="C21" s="27">
         <f>'지브라-스캐너'!F6</f>
         <v/>
       </c>
@@ -12668,14 +12827,14 @@
           <t>정품직선형USB / 선택안함</t>
         </is>
       </c>
-      <c r="F21" s="26" t="n">
+      <c r="F21" s="27" t="n">
         <v>18000</v>
       </c>
-      <c r="G21" s="26">
+      <c r="G21" s="27">
         <f>C21+F21</f>
         <v/>
       </c>
-      <c r="H21" s="26">
+      <c r="H21" s="27">
         <f>G21/110%</f>
         <v/>
       </c>
@@ -12689,7 +12848,7 @@
           <t>DS4608 SR</t>
         </is>
       </c>
-      <c r="C22" s="26">
+      <c r="C22" s="27">
         <f>'지브라-스캐너'!F6</f>
         <v/>
       </c>
@@ -12703,14 +12862,14 @@
           <t>정품직선형USB / 스탠드거치대</t>
         </is>
       </c>
-      <c r="F22" s="26" t="n">
+      <c r="F22" s="27" t="n">
         <v>73000</v>
       </c>
-      <c r="G22" s="26">
+      <c r="G22" s="27">
         <f>C22+F22</f>
         <v/>
       </c>
-      <c r="H22" s="26">
+      <c r="H22" s="27">
         <f>G22/110%</f>
         <v/>
       </c>
@@ -12724,7 +12883,7 @@
           <t>DS4608 SR</t>
         </is>
       </c>
-      <c r="C23" s="26">
+      <c r="C23" s="27">
         <f>'지브라-스캐너'!F6</f>
         <v/>
       </c>
@@ -12738,14 +12897,14 @@
           <t>RS232C / 선택안함</t>
         </is>
       </c>
-      <c r="F23" s="26" t="n">
+      <c r="F23" s="27" t="n">
         <v>24200</v>
       </c>
-      <c r="G23" s="26">
+      <c r="G23" s="27">
         <f>C23+F23</f>
         <v/>
       </c>
-      <c r="H23" s="26">
+      <c r="H23" s="27">
         <f>G23/110%</f>
         <v/>
       </c>
@@ -12759,7 +12918,7 @@
           <t>DS4608 SR</t>
         </is>
       </c>
-      <c r="C24" s="26">
+      <c r="C24" s="27">
         <f>'지브라-스캐너'!F6</f>
         <v/>
       </c>
@@ -12773,14 +12932,14 @@
           <t>RS232C / 스탠드거치대</t>
         </is>
       </c>
-      <c r="F24" s="26" t="n">
+      <c r="F24" s="27" t="n">
         <v>79200</v>
       </c>
-      <c r="G24" s="26">
+      <c r="G24" s="27">
         <f>C24+F24</f>
         <v/>
       </c>
-      <c r="H24" s="26">
+      <c r="H24" s="27">
         <f>G24/110%</f>
         <v/>
       </c>
@@ -12794,7 +12953,7 @@
           <t>DS4608 SR</t>
         </is>
       </c>
-      <c r="C25" s="26">
+      <c r="C25" s="27">
         <f>'지브라-스캐너'!F6</f>
         <v/>
       </c>
@@ -12808,14 +12967,14 @@
           <t>코일형USB / 선택안함</t>
         </is>
       </c>
-      <c r="F25" s="26" t="n">
+      <c r="F25" s="27" t="n">
         <v>18000</v>
       </c>
-      <c r="G25" s="26">
+      <c r="G25" s="27">
         <f>C25+F25</f>
         <v/>
       </c>
-      <c r="H25" s="26">
+      <c r="H25" s="27">
         <f>G25/110%</f>
         <v/>
       </c>
@@ -12829,7 +12988,7 @@
           <t>DS4608 SR</t>
         </is>
       </c>
-      <c r="C26" s="26">
+      <c r="C26" s="27">
         <f>'지브라-스캐너'!F6</f>
         <v/>
       </c>
@@ -12843,14 +13002,14 @@
           <t>코일형USB / 스탠드거치대</t>
         </is>
       </c>
-      <c r="F26" s="26" t="n">
+      <c r="F26" s="27" t="n">
         <v>73000</v>
       </c>
-      <c r="G26" s="26">
+      <c r="G26" s="27">
         <f>C26+F26</f>
         <v/>
       </c>
-      <c r="H26" s="26">
+      <c r="H26" s="27">
         <f>G26/110%</f>
         <v/>
       </c>
@@ -12864,7 +13023,7 @@
           <t>DS4608 SR</t>
         </is>
       </c>
-      <c r="C27" s="26">
+      <c r="C27" s="27">
         <f>'지브라-스캐너'!F6</f>
         <v/>
       </c>
@@ -12878,14 +13037,14 @@
           <t>본체만(케이블없음) / 선택안함</t>
         </is>
       </c>
-      <c r="F27" s="26" t="n">
+      <c r="F27" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="G27" s="26">
+      <c r="G27" s="27">
         <f>C27+F27</f>
         <v/>
       </c>
-      <c r="H27" s="26">
+      <c r="H27" s="27">
         <f>G27/110%</f>
         <v/>
       </c>
@@ -12899,7 +13058,7 @@
           <t>DS4608 SR</t>
         </is>
       </c>
-      <c r="C28" s="26">
+      <c r="C28" s="27">
         <f>'지브라-스캐너'!F6</f>
         <v/>
       </c>
@@ -12913,14 +13072,14 @@
           <t>본체만(케이블없음) / 스탠드거치대</t>
         </is>
       </c>
-      <c r="F28" s="26" t="n">
+      <c r="F28" s="27" t="n">
         <v>55000</v>
       </c>
-      <c r="G28" s="26">
+      <c r="G28" s="27">
         <f>C28+F28</f>
         <v/>
       </c>
-      <c r="H28" s="26">
+      <c r="H28" s="27">
         <f>G28/110%</f>
         <v/>
       </c>
@@ -12934,7 +13093,7 @@
           <t>LI2208</t>
         </is>
       </c>
-      <c r="C29" s="26">
+      <c r="C29" s="27">
         <f>'지브라-스캐너'!F7</f>
         <v/>
       </c>
@@ -12948,14 +13107,14 @@
           <t>정품직선형USB</t>
         </is>
       </c>
-      <c r="F29" s="26" t="n">
+      <c r="F29" s="27" t="n">
         <v>16500</v>
       </c>
-      <c r="G29" s="26">
+      <c r="G29" s="27">
         <f>C29+F29</f>
         <v/>
       </c>
-      <c r="H29" s="26">
+      <c r="H29" s="27">
         <f>G29/110%</f>
         <v/>
       </c>
@@ -12969,7 +13128,7 @@
           <t>LI2208</t>
         </is>
       </c>
-      <c r="C30" s="26">
+      <c r="C30" s="27">
         <f>'지브라-스캐너'!F7</f>
         <v/>
       </c>
@@ -12983,14 +13142,14 @@
           <t>RS232C</t>
         </is>
       </c>
-      <c r="F30" s="26" t="n">
+      <c r="F30" s="27" t="n">
         <v>24200</v>
       </c>
-      <c r="G30" s="26">
+      <c r="G30" s="27">
         <f>C30+F30</f>
         <v/>
       </c>
-      <c r="H30" s="26">
+      <c r="H30" s="27">
         <f>G30/110%</f>
         <v/>
       </c>
@@ -13004,7 +13163,7 @@
           <t>LI3608 SR</t>
         </is>
       </c>
-      <c r="C31" s="26">
+      <c r="C31" s="27">
         <f>'지브라-스캐너'!F8</f>
         <v/>
       </c>
@@ -13018,14 +13177,14 @@
           <t>USB</t>
         </is>
       </c>
-      <c r="F31" s="26" t="n">
+      <c r="F31" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="G31" s="26">
+      <c r="G31" s="27">
         <f>C31+F31</f>
         <v/>
       </c>
-      <c r="H31" s="26">
+      <c r="H31" s="27">
         <f>G31/110%</f>
         <v/>
       </c>
@@ -13039,7 +13198,7 @@
           <t>DS3608 SR</t>
         </is>
       </c>
-      <c r="C32" s="26">
+      <c r="C32" s="27">
         <f>'지브라-스캐너'!F9</f>
         <v/>
       </c>
@@ -13053,14 +13212,14 @@
           <t>USB</t>
         </is>
       </c>
-      <c r="F32" s="26" t="n">
+      <c r="F32" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="G32" s="26">
+      <c r="G32" s="27">
         <f>C32+F32</f>
         <v/>
       </c>
-      <c r="H32" s="26">
+      <c r="H32" s="27">
         <f>G32/110%</f>
         <v/>
       </c>
@@ -13074,7 +13233,7 @@
           <t>DS3608 SR</t>
         </is>
       </c>
-      <c r="C33" s="26">
+      <c r="C33" s="27">
         <f>'지브라-스캐너'!F9</f>
         <v/>
       </c>
@@ -13088,14 +13247,14 @@
           <t>RS232C</t>
         </is>
       </c>
-      <c r="F33" s="26" t="n">
+      <c r="F33" s="27" t="n">
         <v>24200</v>
       </c>
-      <c r="G33" s="26">
+      <c r="G33" s="27">
         <f>C33+F33</f>
         <v/>
       </c>
-      <c r="H33" s="26">
+      <c r="H33" s="27">
         <f>G33/110%</f>
         <v/>
       </c>
@@ -13109,7 +13268,7 @@
           <t>LI3678</t>
         </is>
       </c>
-      <c r="C34" s="26">
+      <c r="C34" s="27">
         <f>'지브라-스캐너'!F10</f>
         <v/>
       </c>
@@ -13123,14 +13282,14 @@
           <t>USB</t>
         </is>
       </c>
-      <c r="F34" s="26" t="n">
+      <c r="F34" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="G34" s="26">
+      <c r="G34" s="27">
         <f>C34+F34</f>
         <v/>
       </c>
-      <c r="H34" s="26">
+      <c r="H34" s="27">
         <f>G34/110%</f>
         <v/>
       </c>
@@ -13144,7 +13303,7 @@
           <t>LI3678</t>
         </is>
       </c>
-      <c r="C35" s="26">
+      <c r="C35" s="27">
         <f>'지브라-스캐너'!F10</f>
         <v/>
       </c>
@@ -13158,14 +13317,14 @@
           <t>RS232C</t>
         </is>
       </c>
-      <c r="F35" s="26" t="n">
+      <c r="F35" s="27" t="n">
         <v>33000</v>
       </c>
-      <c r="G35" s="26">
+      <c r="G35" s="27">
         <f>C35+F35</f>
         <v/>
       </c>
-      <c r="H35" s="26">
+      <c r="H35" s="27">
         <f>G35/110%</f>
         <v/>
       </c>
@@ -13179,7 +13338,7 @@
           <t>DS9908</t>
         </is>
       </c>
-      <c r="C36" s="26">
+      <c r="C36" s="27">
         <f>'지브라-스캐너'!F11</f>
         <v/>
       </c>
@@ -13193,14 +13352,14 @@
           <t>코일형USB</t>
         </is>
       </c>
-      <c r="F36" s="26" t="n">
+      <c r="F36" s="27" t="n">
         <v>18000</v>
       </c>
-      <c r="G36" s="26">
+      <c r="G36" s="27">
         <f>C36+F36</f>
         <v/>
       </c>
-      <c r="H36" s="26">
+      <c r="H36" s="27">
         <f>G36/110%</f>
         <v/>
       </c>
@@ -13214,7 +13373,7 @@
           <t>DS9908</t>
         </is>
       </c>
-      <c r="C37" s="26">
+      <c r="C37" s="27">
         <f>'지브라-스캐너'!F11</f>
         <v/>
       </c>
@@ -13228,14 +13387,14 @@
           <t>직선형USB케이블</t>
         </is>
       </c>
-      <c r="F37" s="26" t="n">
+      <c r="F37" s="27" t="n">
         <v>18000</v>
       </c>
-      <c r="G37" s="26">
+      <c r="G37" s="27">
         <f>C37+F37</f>
         <v/>
       </c>
-      <c r="H37" s="26">
+      <c r="H37" s="27">
         <f>G37/110%</f>
         <v/>
       </c>
@@ -13249,7 +13408,7 @@
           <t>DS9908</t>
         </is>
       </c>
-      <c r="C38" s="26">
+      <c r="C38" s="27">
         <f>'지브라-스캐너'!F11</f>
         <v/>
       </c>
@@ -13263,14 +13422,14 @@
           <t>RS232C</t>
         </is>
       </c>
-      <c r="F38" s="26" t="n">
+      <c r="F38" s="27" t="n">
         <v>24200</v>
       </c>
-      <c r="G38" s="26">
+      <c r="G38" s="27">
         <f>C38+F38</f>
         <v/>
       </c>
-      <c r="H38" s="26">
+      <c r="H38" s="27">
         <f>G38/110%</f>
         <v/>
       </c>
@@ -13284,7 +13443,7 @@
           <t>CS6080</t>
         </is>
       </c>
-      <c r="C39" s="26">
+      <c r="C39" s="27">
         <f>'지브라-스캐너'!F13</f>
         <v/>
       </c>
@@ -13298,14 +13457,14 @@
           <t>2D</t>
         </is>
       </c>
-      <c r="F39" s="26" t="n">
+      <c r="F39" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="G39" s="26">
+      <c r="G39" s="27">
         <f>C39+F39</f>
         <v/>
       </c>
-      <c r="H39" s="26">
+      <c r="H39" s="27">
         <f>G39/110%</f>
         <v/>
       </c>
@@ -13319,7 +13478,7 @@
           <t>DS3678 SR</t>
         </is>
       </c>
-      <c r="C40" s="26">
+      <c r="C40" s="27">
         <f>'지브라-스캐너'!F14</f>
         <v/>
       </c>
@@ -13333,14 +13492,14 @@
           <t>SR버전+USB케이블</t>
         </is>
       </c>
-      <c r="F40" s="26" t="n">
+      <c r="F40" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="G40" s="26">
+      <c r="G40" s="27">
         <f>C40+F40</f>
         <v/>
       </c>
-      <c r="H40" s="26">
+      <c r="H40" s="27">
         <f>G40/110%</f>
         <v/>
       </c>
@@ -13354,7 +13513,7 @@
           <t>DS3678 SR</t>
         </is>
       </c>
-      <c r="C41" s="26">
+      <c r="C41" s="27">
         <f>'지브라-스캐너'!F14</f>
         <v/>
       </c>
@@ -13368,14 +13527,14 @@
           <t>HD버전+USB케이블</t>
         </is>
       </c>
-      <c r="F41" s="26" t="n">
+      <c r="F41" s="27" t="n">
         <v>220000</v>
       </c>
-      <c r="G41" s="26">
+      <c r="G41" s="27">
         <f>C41+F41</f>
         <v/>
       </c>
-      <c r="H41" s="26">
+      <c r="H41" s="27">
         <f>G41/110%</f>
         <v/>
       </c>
@@ -13389,7 +13548,7 @@
           <t>DS3678 SR</t>
         </is>
       </c>
-      <c r="C42" s="26">
+      <c r="C42" s="27">
         <f>'지브라-스캐너'!F14</f>
         <v/>
       </c>
@@ -13403,14 +13562,14 @@
           <t>SR버전+RS232C케이블</t>
         </is>
       </c>
-      <c r="F42" s="26" t="n">
+      <c r="F42" s="27" t="n">
         <v>33000</v>
       </c>
-      <c r="G42" s="26">
+      <c r="G42" s="27">
         <f>C42+F42</f>
         <v/>
       </c>
-      <c r="H42" s="26">
+      <c r="H42" s="27">
         <f>G42/110%</f>
         <v/>
       </c>
@@ -13424,7 +13583,7 @@
           <t>DS3678 SR</t>
         </is>
       </c>
-      <c r="C43" s="26">
+      <c r="C43" s="27">
         <f>'지브라-스캐너'!F14</f>
         <v/>
       </c>
@@ -13438,14 +13597,14 @@
           <t>HD버전+RS232C케이블</t>
         </is>
       </c>
-      <c r="F43" s="26" t="n">
+      <c r="F43" s="27" t="n">
         <v>275000</v>
       </c>
-      <c r="G43" s="26">
+      <c r="G43" s="27">
         <f>C43+F43</f>
         <v/>
       </c>
-      <c r="H43" s="26">
+      <c r="H43" s="27">
         <f>G43/110%</f>
         <v/>
       </c>
@@ -13459,7 +13618,7 @@
           <t>DS4608 XD</t>
         </is>
       </c>
-      <c r="C44" s="26">
+      <c r="C44" s="27">
         <f>'지브라-스캐너'!F15</f>
         <v/>
       </c>
@@ -13473,14 +13632,14 @@
           <t>정품직선형USB / 선택안함</t>
         </is>
       </c>
-      <c r="F44" s="26" t="n">
+      <c r="F44" s="27" t="n">
         <v>18000</v>
       </c>
-      <c r="G44" s="26">
+      <c r="G44" s="27">
         <f>C44+F44</f>
         <v/>
       </c>
-      <c r="H44" s="26">
+      <c r="H44" s="27">
         <f>G44/110%</f>
         <v/>
       </c>
@@ -13494,7 +13653,7 @@
           <t>DS4608 XD</t>
         </is>
       </c>
-      <c r="C45" s="26">
+      <c r="C45" s="27">
         <f>'지브라-스캐너'!F15</f>
         <v/>
       </c>
@@ -13508,14 +13667,14 @@
           <t>정품직선형USB / 스탠드거치대</t>
         </is>
       </c>
-      <c r="F45" s="26" t="n">
+      <c r="F45" s="27" t="n">
         <v>73000</v>
       </c>
-      <c r="G45" s="26">
+      <c r="G45" s="27">
         <f>C45+F45</f>
         <v/>
       </c>
-      <c r="H45" s="26">
+      <c r="H45" s="27">
         <f>G45/110%</f>
         <v/>
       </c>
@@ -13529,7 +13688,7 @@
           <t>DS4608 XD</t>
         </is>
       </c>
-      <c r="C46" s="26">
+      <c r="C46" s="27">
         <f>'지브라-스캐너'!F15</f>
         <v/>
       </c>
@@ -13543,14 +13702,14 @@
           <t>RS232C / 선택안함</t>
         </is>
       </c>
-      <c r="F46" s="26" t="n">
+      <c r="F46" s="27" t="n">
         <v>24200</v>
       </c>
-      <c r="G46" s="26">
+      <c r="G46" s="27">
         <f>C46+F46</f>
         <v/>
       </c>
-      <c r="H46" s="26">
+      <c r="H46" s="27">
         <f>G46/110%</f>
         <v/>
       </c>
@@ -13564,7 +13723,7 @@
           <t>DS4608 XD</t>
         </is>
       </c>
-      <c r="C47" s="26">
+      <c r="C47" s="27">
         <f>'지브라-스캐너'!F15</f>
         <v/>
       </c>
@@ -13578,14 +13737,14 @@
           <t>RS232C / 스탠드거치대</t>
         </is>
       </c>
-      <c r="F47" s="26" t="n">
+      <c r="F47" s="27" t="n">
         <v>79200</v>
       </c>
-      <c r="G47" s="26">
+      <c r="G47" s="27">
         <f>C47+F47</f>
         <v/>
       </c>
-      <c r="H47" s="26">
+      <c r="H47" s="27">
         <f>G47/110%</f>
         <v/>
       </c>
@@ -13599,7 +13758,7 @@
           <t>DS4608 XD</t>
         </is>
       </c>
-      <c r="C48" s="26">
+      <c r="C48" s="27">
         <f>'지브라-스캐너'!F15</f>
         <v/>
       </c>
@@ -13613,14 +13772,14 @@
           <t>코일형USB / 선택안함</t>
         </is>
       </c>
-      <c r="F48" s="26" t="n">
+      <c r="F48" s="27" t="n">
         <v>18000</v>
       </c>
-      <c r="G48" s="26">
+      <c r="G48" s="27">
         <f>C48+F48</f>
         <v/>
       </c>
-      <c r="H48" s="26">
+      <c r="H48" s="27">
         <f>G48/110%</f>
         <v/>
       </c>
@@ -13634,7 +13793,7 @@
           <t>DS4608 XD</t>
         </is>
       </c>
-      <c r="C49" s="26">
+      <c r="C49" s="27">
         <f>'지브라-스캐너'!F15</f>
         <v/>
       </c>
@@ -13648,14 +13807,14 @@
           <t>코일형USB / 스탠드거치대</t>
         </is>
       </c>
-      <c r="F49" s="26" t="n">
+      <c r="F49" s="27" t="n">
         <v>73000</v>
       </c>
-      <c r="G49" s="26">
+      <c r="G49" s="27">
         <f>C49+F49</f>
         <v/>
       </c>
-      <c r="H49" s="26">
+      <c r="H49" s="27">
         <f>G49/110%</f>
         <v/>
       </c>
@@ -13669,7 +13828,7 @@
           <t>DS4608 XD</t>
         </is>
       </c>
-      <c r="C50" s="26">
+      <c r="C50" s="27">
         <f>'지브라-스캐너'!F15</f>
         <v/>
       </c>
@@ -13683,14 +13842,14 @@
           <t>본체만(케이블없음) / 선택안함</t>
         </is>
       </c>
-      <c r="F50" s="26" t="n">
+      <c r="F50" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="G50" s="26">
+      <c r="G50" s="27">
         <f>C50+F50</f>
         <v/>
       </c>
-      <c r="H50" s="26">
+      <c r="H50" s="27">
         <f>G50/110%</f>
         <v/>
       </c>
@@ -13704,7 +13863,7 @@
           <t>DS4608 XD</t>
         </is>
       </c>
-      <c r="C51" s="26">
+      <c r="C51" s="27">
         <f>'지브라-스캐너'!F15</f>
         <v/>
       </c>
@@ -13718,14 +13877,14 @@
           <t>본체만(케이블없음) / 스탠드거치대</t>
         </is>
       </c>
-      <c r="F51" s="26" t="n">
+      <c r="F51" s="27" t="n">
         <v>55000</v>
       </c>
-      <c r="G51" s="26">
+      <c r="G51" s="27">
         <f>C51+F51</f>
         <v/>
       </c>
-      <c r="H51" s="26">
+      <c r="H51" s="27">
         <f>G51/110%</f>
         <v/>
       </c>
@@ -13739,7 +13898,7 @@
           <t>DS8288</t>
         </is>
       </c>
-      <c r="C52" s="26">
+      <c r="C52" s="27">
         <f>'지브라-스캐너'!F16</f>
         <v/>
       </c>
@@ -13753,14 +13912,14 @@
           <t>RS232C</t>
         </is>
       </c>
-      <c r="F52" s="26" t="n">
+      <c r="F52" s="27" t="n">
         <v>24200</v>
       </c>
-      <c r="G52" s="26">
+      <c r="G52" s="27">
         <f>C52+F52</f>
         <v/>
       </c>
-      <c r="H52" s="26">
+      <c r="H52" s="27">
         <f>G52/110%</f>
         <v/>
       </c>
@@ -13774,7 +13933,7 @@
           <t>DS8288</t>
         </is>
       </c>
-      <c r="C53" s="26">
+      <c r="C53" s="27">
         <f>'지브라-스캐너'!F16</f>
         <v/>
       </c>
@@ -13788,14 +13947,14 @@
           <t>USB</t>
         </is>
       </c>
-      <c r="F53" s="26" t="n">
+      <c r="F53" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="G53" s="26">
+      <c r="G53" s="27">
         <f>C53+F53</f>
         <v/>
       </c>
-      <c r="H53" s="26">
+      <c r="H53" s="27">
         <f>G53/110%</f>
         <v/>
       </c>
@@ -13809,7 +13968,7 @@
           <t>DS8208</t>
         </is>
       </c>
-      <c r="C54" s="26">
+      <c r="C54" s="27">
         <f>'지브라-스캐너'!F17</f>
         <v/>
       </c>
@@ -13823,14 +13982,14 @@
           <t>RS232C</t>
         </is>
       </c>
-      <c r="F54" s="26" t="n">
+      <c r="F54" s="27" t="n">
         <v>24200</v>
       </c>
-      <c r="G54" s="26">
+      <c r="G54" s="27">
         <f>C54+F54</f>
         <v/>
       </c>
-      <c r="H54" s="26">
+      <c r="H54" s="27">
         <f>G54/110%</f>
         <v/>
       </c>
@@ -13844,7 +14003,7 @@
           <t>DS8208</t>
         </is>
       </c>
-      <c r="C55" s="26">
+      <c r="C55" s="27">
         <f>'지브라-스캐너'!F17</f>
         <v/>
       </c>
@@ -13858,14 +14017,14 @@
           <t>USB</t>
         </is>
       </c>
-      <c r="F55" s="26" t="n">
+      <c r="F55" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="G55" s="26">
+      <c r="G55" s="27">
         <f>C55+F55</f>
         <v/>
       </c>
-      <c r="H55" s="26">
+      <c r="H55" s="27">
         <f>G55/110%</f>
         <v/>
       </c>
@@ -13879,7 +14038,7 @@
           <t>DS3608 ER</t>
         </is>
       </c>
-      <c r="C56" s="26">
+      <c r="C56" s="27">
         <f>'지브라-스캐너'!F18</f>
         <v/>
       </c>
@@ -13893,14 +14052,14 @@
           <t>USB</t>
         </is>
       </c>
-      <c r="F56" s="26" t="n">
+      <c r="F56" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="G56" s="26">
+      <c r="G56" s="27">
         <f>C56+F56</f>
         <v/>
       </c>
-      <c r="H56" s="26">
+      <c r="H56" s="27">
         <f>G56/110%</f>
         <v/>
       </c>
@@ -13914,7 +14073,7 @@
           <t>LI3608 ER</t>
         </is>
       </c>
-      <c r="C57" s="26">
+      <c r="C57" s="27">
         <f>'지브라-스캐너'!F19</f>
         <v/>
       </c>
@@ -13928,14 +14087,14 @@
           <t>USB</t>
         </is>
       </c>
-      <c r="F57" s="26" t="n">
+      <c r="F57" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="G57" s="26">
+      <c r="G57" s="27">
         <f>C57+F57</f>
         <v/>
       </c>
-      <c r="H57" s="26">
+      <c r="H57" s="27">
         <f>G57/110%</f>
         <v/>
       </c>
@@ -13949,7 +14108,7 @@
           <t>DS3678 XR</t>
         </is>
       </c>
-      <c r="C58" s="26">
+      <c r="C58" s="27">
         <f>'지브라-스캐너'!F20</f>
         <v/>
       </c>
@@ -13963,14 +14122,14 @@
           <t>USB</t>
         </is>
       </c>
-      <c r="F58" s="26" t="n">
+      <c r="F58" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="G58" s="26">
+      <c r="G58" s="27">
         <f>C58+F58</f>
         <v/>
       </c>
-      <c r="H58" s="26">
+      <c r="H58" s="27">
         <f>G58/110%</f>
         <v/>
       </c>
@@ -13984,7 +14143,7 @@
           <t>DS3678 XR</t>
         </is>
       </c>
-      <c r="C59" s="26">
+      <c r="C59" s="27">
         <f>'지브라-스캐너'!F20</f>
         <v/>
       </c>
@@ -13998,14 +14157,14 @@
           <t>RS232C</t>
         </is>
       </c>
-      <c r="F59" s="26" t="n">
+      <c r="F59" s="27" t="n">
         <v>24200</v>
       </c>
-      <c r="G59" s="26">
+      <c r="G59" s="27">
         <f>C59+F59</f>
         <v/>
       </c>
-      <c r="H59" s="26">
+      <c r="H59" s="27">
         <f>G59/110%</f>
         <v/>
       </c>
@@ -14019,7 +14178,7 @@
           <t>DS5502</t>
         </is>
       </c>
-      <c r="C60" s="26">
+      <c r="C60" s="27">
         <f>'지브라-스캐너'!F21</f>
         <v/>
       </c>
@@ -14033,14 +14192,14 @@
           <t>RS232C</t>
         </is>
       </c>
-      <c r="F60" s="26" t="n">
+      <c r="F60" s="27" t="n">
         <v>49500</v>
       </c>
-      <c r="G60" s="26">
+      <c r="G60" s="27">
         <f>C60+F60</f>
         <v/>
       </c>
-      <c r="H60" s="26">
+      <c r="H60" s="27">
         <f>G60/110%</f>
         <v/>
       </c>
@@ -14054,7 +14213,7 @@
           <t>DS5502</t>
         </is>
       </c>
-      <c r="C61" s="26">
+      <c r="C61" s="27">
         <f>'지브라-스캐너'!F21</f>
         <v/>
       </c>
@@ -14068,14 +14227,14 @@
           <t>USB</t>
         </is>
       </c>
-      <c r="F61" s="26" t="n">
+      <c r="F61" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="G61" s="26">
+      <c r="G61" s="27">
         <f>C61+F61</f>
         <v/>
       </c>
-      <c r="H61" s="26">
+      <c r="H61" s="27">
         <f>G61/110%</f>
         <v/>
       </c>
@@ -14089,7 +14248,7 @@
           <t>DS4678</t>
         </is>
       </c>
-      <c r="C62" s="26">
+      <c r="C62" s="27">
         <f>'지브라-스캐너'!F22</f>
         <v/>
       </c>
@@ -14103,14 +14262,14 @@
           <t>본체+크래들만(케이블없음)</t>
         </is>
       </c>
-      <c r="F62" s="26" t="n">
+      <c r="F62" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="G62" s="26">
+      <c r="G62" s="27">
         <f>C62+F62</f>
         <v/>
       </c>
-      <c r="H62" s="26">
+      <c r="H62" s="27">
         <f>G62/110%</f>
         <v/>
       </c>
@@ -14124,7 +14283,7 @@
           <t>DS4678</t>
         </is>
       </c>
-      <c r="C63" s="26">
+      <c r="C63" s="27">
         <f>'지브라-스캐너'!F22</f>
         <v/>
       </c>
@@ -14138,14 +14297,14 @@
           <t>정품직선형USB</t>
         </is>
       </c>
-      <c r="F63" s="26" t="n">
+      <c r="F63" s="27" t="n">
         <v>18000</v>
       </c>
-      <c r="G63" s="26">
+      <c r="G63" s="27">
         <f>C63+F63</f>
         <v/>
       </c>
-      <c r="H63" s="26">
+      <c r="H63" s="27">
         <f>G63/110%</f>
         <v/>
       </c>
@@ -14159,7 +14318,7 @@
           <t>DS4678</t>
         </is>
       </c>
-      <c r="C64" s="26">
+      <c r="C64" s="27">
         <f>'지브라-스캐너'!F22</f>
         <v/>
       </c>
@@ -14173,14 +14332,14 @@
           <t>코일형USB</t>
         </is>
       </c>
-      <c r="F64" s="26" t="n">
+      <c r="F64" s="27" t="n">
         <v>18000</v>
       </c>
-      <c r="G64" s="26">
+      <c r="G64" s="27">
         <f>C64+F64</f>
         <v/>
       </c>
-      <c r="H64" s="26">
+      <c r="H64" s="27">
         <f>G64/110%</f>
         <v/>
       </c>
@@ -14194,7 +14353,7 @@
           <t>DS4678</t>
         </is>
       </c>
-      <c r="C65" s="26">
+      <c r="C65" s="27">
         <f>'지브라-스캐너'!F22</f>
         <v/>
       </c>
@@ -14208,14 +14367,14 @@
           <t>RS232C</t>
         </is>
       </c>
-      <c r="F65" s="26" t="n">
+      <c r="F65" s="27" t="n">
         <v>24200</v>
       </c>
-      <c r="G65" s="26">
+      <c r="G65" s="27">
         <f>C65+F65</f>
         <v/>
       </c>
-      <c r="H65" s="26">
+      <c r="H65" s="27">
         <f>G65/110%</f>
         <v/>
       </c>
@@ -14229,7 +14388,7 @@
           <t>SP72</t>
         </is>
       </c>
-      <c r="C66" s="26">
+      <c r="C66" s="27">
         <f>'지브라-스캐너'!F23</f>
         <v/>
       </c>
@@ -14243,14 +14402,14 @@
           <t>USB</t>
         </is>
       </c>
-      <c r="F66" s="26" t="n">
+      <c r="F66" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="G66" s="26">
+      <c r="G66" s="27">
         <f>C66+F66</f>
         <v/>
       </c>
-      <c r="H66" s="26">
+      <c r="H66" s="27">
         <f>G66/110%</f>
         <v/>
       </c>
@@ -14264,7 +14423,7 @@
           <t>DS9308</t>
         </is>
       </c>
-      <c r="C67" s="26">
+      <c r="C67" s="27">
         <f>'지브라-스캐너'!F24</f>
         <v/>
       </c>
@@ -14278,14 +14437,14 @@
           <t>직선형USB케이블</t>
         </is>
       </c>
-      <c r="F67" s="26" t="n">
+      <c r="F67" s="27" t="n">
         <v>18000</v>
       </c>
-      <c r="G67" s="26">
+      <c r="G67" s="27">
         <f>C67+F67</f>
         <v/>
       </c>
-      <c r="H67" s="26">
+      <c r="H67" s="27">
         <f>G67/110%</f>
         <v/>
       </c>
@@ -14299,7 +14458,7 @@
           <t>DS9308</t>
         </is>
       </c>
-      <c r="C68" s="26">
+      <c r="C68" s="27">
         <f>'지브라-스캐너'!F24</f>
         <v/>
       </c>
@@ -14313,14 +14472,14 @@
           <t>RS232C</t>
         </is>
       </c>
-      <c r="F68" s="26" t="n">
+      <c r="F68" s="27" t="n">
         <v>24200</v>
       </c>
-      <c r="G68" s="26">
+      <c r="G68" s="27">
         <f>C68+F68</f>
         <v/>
       </c>
-      <c r="H68" s="26">
+      <c r="H68" s="27">
         <f>G68/110%</f>
         <v/>
       </c>
@@ -14334,7 +14493,7 @@
           <t>DS9308</t>
         </is>
       </c>
-      <c r="C69" s="26">
+      <c r="C69" s="27">
         <f>'지브라-스캐너'!F24</f>
         <v/>
       </c>
@@ -14348,14 +14507,14 @@
           <t>코일형USB</t>
         </is>
       </c>
-      <c r="F69" s="26" t="n">
+      <c r="F69" s="27" t="n">
         <v>18000</v>
       </c>
-      <c r="G69" s="26">
+      <c r="G69" s="27">
         <f>C69+F69</f>
         <v/>
       </c>
-      <c r="H69" s="26">
+      <c r="H69" s="27">
         <f>G69/110%</f>
         <v/>
       </c>
@@ -14369,7 +14528,7 @@
           <t>DS9308</t>
         </is>
       </c>
-      <c r="C70" s="26">
+      <c r="C70" s="27">
         <f>'지브라-스캐너'!F24</f>
         <v/>
       </c>
@@ -14383,14 +14542,14 @@
           <t>본체만(케이블없음)</t>
         </is>
       </c>
-      <c r="F70" s="26" t="n">
+      <c r="F70" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="G70" s="26">
+      <c r="G70" s="27">
         <f>C70+F70</f>
         <v/>
       </c>
-      <c r="H70" s="26">
+      <c r="H70" s="27">
         <f>G70/110%</f>
         <v/>
       </c>
@@ -14404,7 +14563,7 @@
           <t>DS8178</t>
         </is>
       </c>
-      <c r="C71" s="26">
+      <c r="C71" s="27">
         <f>'지브라-스캐너'!F25</f>
         <v/>
       </c>
@@ -14418,14 +14577,14 @@
           <t>정품직선형USB</t>
         </is>
       </c>
-      <c r="F71" s="26" t="n">
+      <c r="F71" s="27" t="n">
         <v>18000</v>
       </c>
-      <c r="G71" s="26">
+      <c r="G71" s="27">
         <f>C71+F71</f>
         <v/>
       </c>
-      <c r="H71" s="26">
+      <c r="H71" s="27">
         <f>G71/110%</f>
         <v/>
       </c>
@@ -14439,7 +14598,7 @@
           <t>DS8178</t>
         </is>
       </c>
-      <c r="C72" s="26">
+      <c r="C72" s="27">
         <f>'지브라-스캐너'!F25</f>
         <v/>
       </c>
@@ -14453,14 +14612,14 @@
           <t>RS232C</t>
         </is>
       </c>
-      <c r="F72" s="26" t="n">
+      <c r="F72" s="27" t="n">
         <v>24200</v>
       </c>
-      <c r="G72" s="26">
+      <c r="G72" s="27">
         <f>C72+F72</f>
         <v/>
       </c>
-      <c r="H72" s="26">
+      <c r="H72" s="27">
         <f>G72/110%</f>
         <v/>
       </c>
@@ -14474,7 +14633,7 @@
           <t>DS8178</t>
         </is>
       </c>
-      <c r="C73" s="26">
+      <c r="C73" s="27">
         <f>'지브라-스캐너'!F25</f>
         <v/>
       </c>
@@ -14488,14 +14647,14 @@
           <t>코일형USB</t>
         </is>
       </c>
-      <c r="F73" s="26" t="n">
+      <c r="F73" s="27" t="n">
         <v>18000</v>
       </c>
-      <c r="G73" s="26">
+      <c r="G73" s="27">
         <f>C73+F73</f>
         <v/>
       </c>
-      <c r="H73" s="26">
+      <c r="H73" s="27">
         <f>G73/110%</f>
         <v/>
       </c>
@@ -14509,7 +14668,7 @@
           <t>DS8178</t>
         </is>
       </c>
-      <c r="C74" s="26">
+      <c r="C74" s="27">
         <f>'지브라-스캐너'!F25</f>
         <v/>
       </c>
@@ -14523,14 +14682,14 @@
           <t>본체+크래들만(케이블없음)</t>
         </is>
       </c>
-      <c r="F74" s="26" t="n">
+      <c r="F74" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="G74" s="26">
+      <c r="G74" s="27">
         <f>C74+F74</f>
         <v/>
       </c>
-      <c r="H74" s="26">
+      <c r="H74" s="27">
         <f>G74/110%</f>
         <v/>
       </c>
@@ -14544,7 +14703,7 @@
           <t>LI4278</t>
         </is>
       </c>
-      <c r="C75" s="26">
+      <c r="C75" s="27">
         <f>'지브라-스캐너'!F26</f>
         <v/>
       </c>
@@ -14558,14 +14717,14 @@
           <t>정품직선형USB</t>
         </is>
       </c>
-      <c r="F75" s="26" t="n">
+      <c r="F75" s="27" t="n">
         <v>18000</v>
       </c>
-      <c r="G75" s="26">
+      <c r="G75" s="27">
         <f>C75+F75</f>
         <v/>
       </c>
-      <c r="H75" s="26">
+      <c r="H75" s="27">
         <f>G75/110%</f>
         <v/>
       </c>
@@ -14579,7 +14738,7 @@
           <t>LI4278</t>
         </is>
       </c>
-      <c r="C76" s="26">
+      <c r="C76" s="27">
         <f>'지브라-스캐너'!F26</f>
         <v/>
       </c>
@@ -14593,14 +14752,14 @@
           <t>RS232C</t>
         </is>
       </c>
-      <c r="F76" s="26" t="n">
+      <c r="F76" s="27" t="n">
         <v>24200</v>
       </c>
-      <c r="G76" s="26">
+      <c r="G76" s="27">
         <f>C76+F76</f>
         <v/>
       </c>
-      <c r="H76" s="26">
+      <c r="H76" s="27">
         <f>G76/110%</f>
         <v/>
       </c>
@@ -14614,7 +14773,7 @@
           <t>LI4278</t>
         </is>
       </c>
-      <c r="C77" s="26">
+      <c r="C77" s="27">
         <f>'지브라-스캐너'!F26</f>
         <v/>
       </c>
@@ -14628,14 +14787,14 @@
           <t>코일형USB</t>
         </is>
       </c>
-      <c r="F77" s="26" t="n">
+      <c r="F77" s="27" t="n">
         <v>18000</v>
       </c>
-      <c r="G77" s="26">
+      <c r="G77" s="27">
         <f>C77+F77</f>
         <v/>
       </c>
-      <c r="H77" s="26">
+      <c r="H77" s="27">
         <f>G77/110%</f>
         <v/>
       </c>
@@ -14649,7 +14808,7 @@
           <t>LI4278</t>
         </is>
       </c>
-      <c r="C78" s="26">
+      <c r="C78" s="27">
         <f>'지브라-스캐너'!F26</f>
         <v/>
       </c>
@@ -14663,14 +14822,14 @@
           <t>본체+크래들만(케이블없음)</t>
         </is>
       </c>
-      <c r="F78" s="26" t="n">
+      <c r="F78" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="G78" s="26">
+      <c r="G78" s="27">
         <f>C78+F78</f>
         <v/>
       </c>
-      <c r="H78" s="26">
+      <c r="H78" s="27">
         <f>G78/110%</f>
         <v/>
       </c>
@@ -14684,7 +14843,7 @@
           <t>RS6100</t>
         </is>
       </c>
-      <c r="C79" s="26">
+      <c r="C79" s="27">
         <f>'지브라-스캐너'!F27</f>
         <v/>
       </c>
@@ -14698,14 +14857,14 @@
           <t>링트리거</t>
         </is>
       </c>
-      <c r="F79" s="26" t="n">
+      <c r="F79" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="G79" s="26">
+      <c r="G79" s="27">
         <f>C79+F79</f>
         <v/>
       </c>
-      <c r="H79" s="26">
+      <c r="H79" s="27">
         <f>G79/110%</f>
         <v/>
       </c>
@@ -14719,7 +14878,7 @@
           <t>FS10</t>
         </is>
       </c>
-      <c r="C80" s="26">
+      <c r="C80" s="27">
         <f>'지브라-스캐너'!F28</f>
         <v/>
       </c>
@@ -14733,14 +14892,14 @@
           <t>본체</t>
         </is>
       </c>
-      <c r="F80" s="26" t="n">
+      <c r="F80" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="G80" s="26">
+      <c r="G80" s="27">
         <f>C80+F80</f>
         <v/>
       </c>
-      <c r="H80" s="26">
+      <c r="H80" s="27">
         <f>G80/110%</f>
         <v/>
       </c>
@@ -14754,7 +14913,7 @@
           <t>FS20</t>
         </is>
       </c>
-      <c r="C81" s="26">
+      <c r="C81" s="27">
         <f>'지브라-스캐너'!F29</f>
         <v/>
       </c>
@@ -14768,14 +14927,14 @@
           <t>본체</t>
         </is>
       </c>
-      <c r="F81" s="26" t="n">
+      <c r="F81" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="G81" s="26">
+      <c r="G81" s="27">
         <f>C81+F81</f>
         <v/>
       </c>
-      <c r="H81" s="26">
+      <c r="H81" s="27">
         <f>G81/110%</f>
         <v/>
       </c>
@@ -14789,7 +14948,7 @@
           <t>FS40</t>
         </is>
       </c>
-      <c r="C82" s="26">
+      <c r="C82" s="27">
         <f>'지브라-스캐너'!F30</f>
         <v/>
       </c>
@@ -14803,14 +14962,14 @@
           <t>본체</t>
         </is>
       </c>
-      <c r="F82" s="26" t="n">
+      <c r="F82" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="G82" s="26">
+      <c r="G82" s="27">
         <f>C82+F82</f>
         <v/>
       </c>
-      <c r="H82" s="26">
+      <c r="H82" s="27">
         <f>G82/110%</f>
         <v/>
       </c>
@@ -14824,7 +14983,7 @@
           <t>FS70</t>
         </is>
       </c>
-      <c r="C83" s="26">
+      <c r="C83" s="27">
         <f>'지브라-스캐너'!F31</f>
         <v/>
       </c>
@@ -14838,14 +14997,14 @@
           <t>본체</t>
         </is>
       </c>
-      <c r="F83" s="26" t="n">
+      <c r="F83" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="G83" s="26">
+      <c r="G83" s="27">
         <f>C83+F83</f>
         <v/>
       </c>
-      <c r="H83" s="26">
+      <c r="H83" s="27">
         <f>G83/110%</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Drop USB variants from option list; add USB-included price at 18,000 KRW
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0164u4m2HzVL7yDN6jZnxUBp
</commit_message>
<xml_diff>
--- a/output/지브라_스캐너_옵션추가.xlsx
+++ b/output/지브라_스캐너_옵션추가.xlsx
@@ -770,6 +770,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="25" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment vertical="center"/>
     </xf>
@@ -785,7 +786,6 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="44">
     <cellStyle name="표준" xfId="0" builtinId="0"/>
@@ -9697,7 +9697,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q31"/>
+  <dimension ref="A1:R31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="16.375" customWidth="1" style="16" min="2" max="2"/>
@@ -9710,6 +9710,7 @@
     <col width="19.875" customWidth="1" style="16" min="14" max="14"/>
     <col width="48" customWidth="1" style="16" min="16" max="16"/>
     <col width="20" customWidth="1" style="16" min="17" max="17"/>
+    <col width="22" customWidth="1" style="16" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1" ht="18.75" customHeight="1" s="16">
@@ -9782,12 +9783,17 @@
       </c>
       <c r="P1" s="4" t="inlineStr">
         <is>
-          <t>옵션(추가금액)</t>
+          <t>옵션(USB 제외, 추가금액)</t>
         </is>
       </c>
       <c r="Q1" s="4" t="inlineStr">
         <is>
           <t>USB케이블 포함(O/X)</t>
+        </is>
+      </c>
+      <c r="R1" s="4" t="inlineStr">
+        <is>
+          <t>USB포함가(18,000원 기준)</t>
         </is>
       </c>
     </row>
@@ -9816,9 +9822,7 @@
       </c>
       <c r="P2" s="20" t="inlineStr">
         <is>
-          <t>정품직선형USB (+18,000원)
-코일형USB (+18,000원)
-RS232C (+24,200원)
+          <t>RS232C (+24,200원)
 본체만(케이블없음) (+0원)</t>
         </is>
       </c>
@@ -9826,6 +9830,10 @@
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="R2" s="22">
+        <f>IF(Q2="X",F2+18000,F2)</f>
+        <v/>
       </c>
     </row>
     <row r="3">
@@ -9858,7 +9866,7 @@
         <f>J3/110%</f>
         <v/>
       </c>
-      <c r="L3" s="22" t="inlineStr">
+      <c r="L3" s="23" t="inlineStr">
         <is>
           <t>제벡스코리아</t>
         </is>
@@ -9873,9 +9881,7 @@
       </c>
       <c r="P3" s="20" t="inlineStr">
         <is>
-          <t>정품직선형USB (+18,000원)
-코일형USB (+18,000원)
-RS232C (+24,200원)
+          <t>RS232C (+24,200원)
 본체+크래들만(케이블없음) (+0원)</t>
         </is>
       </c>
@@ -9883,6 +9889,10 @@
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="R3" s="22">
+        <f>IF(Q3="X",F3+18000,F3)</f>
+        <v/>
       </c>
     </row>
     <row r="4">
@@ -9915,7 +9925,7 @@
         <f>J4/110%</f>
         <v/>
       </c>
-      <c r="L4" s="22" t="inlineStr">
+      <c r="L4" s="23" t="inlineStr">
         <is>
           <t>마켓굿초이스</t>
         </is>
@@ -9930,12 +9940,8 @@
       </c>
       <c r="P4" s="20" t="inlineStr">
         <is>
-          <t>정품직선형USB / 선택안함 (+18,000원)
-정품직선형USB / 스탠드거치대 (+73,000원)
-RS232C / 선택안함 (+24,200원)
+          <t>RS232C / 선택안함 (+24,200원)
 RS232C / 스탠드거치대 (+79,200원)
-코일형USB / 선택안함 (+18,000원)
-코일형USB / 스탠드거치대 (+73,000원)
 본체만(케이블없음) / 선택안함 (+0원)
 본체만(케이블없음) / 스탠드거치대 (+55,000원)</t>
         </is>
@@ -9944,6 +9950,10 @@
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="R4" s="22">
+        <f>IF(Q4="X",F4+18000,F4)</f>
+        <v/>
       </c>
     </row>
     <row r="5">
@@ -9976,7 +9986,7 @@
         <f>J5/110%</f>
         <v/>
       </c>
-      <c r="L5" s="22" t="inlineStr">
+      <c r="L5" s="23" t="inlineStr">
         <is>
           <t>바코드다판다</t>
         </is>
@@ -9991,8 +10001,7 @@
       </c>
       <c r="P5" s="20" t="inlineStr">
         <is>
-          <t>정품직선형USB (+16,500원)
-RS232C (+24,200원)
+          <t>RS232C (+24,200원)
 본체만 (+0원)</t>
         </is>
       </c>
@@ -10000,6 +10009,10 @@
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="R5" s="22">
+        <f>IF(Q5="X",F5+18000,F5)</f>
+        <v/>
       </c>
     </row>
     <row r="6">
@@ -10032,7 +10045,7 @@
         <f>J6/110%</f>
         <v/>
       </c>
-      <c r="L6" s="22" t="inlineStr">
+      <c r="L6" s="23" t="inlineStr">
         <is>
           <t>에이치에스스토어(usb제외)</t>
         </is>
@@ -10047,12 +10060,8 @@
       </c>
       <c r="P6" s="20" t="inlineStr">
         <is>
-          <t>정품직선형USB / 선택안함 (+18,000원)
-정품직선형USB / 스탠드거치대 (+73,000원)
-RS232C / 선택안함 (+24,200원)
+          <t>RS232C / 선택안함 (+24,200원)
 RS232C / 스탠드거치대 (+79,200원)
-코일형USB / 선택안함 (+18,000원)
-코일형USB / 스탠드거치대 (+73,000원)
 본체만(케이블없음) / 선택안함 (+0원)
 본체만(케이블없음) / 스탠드거치대 (+55,000원)</t>
         </is>
@@ -10061,6 +10070,10 @@
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="R6" s="22">
+        <f>IF(Q6="X",F6+18000,F6)</f>
+        <v/>
       </c>
     </row>
     <row r="7">
@@ -10090,7 +10103,7 @@
         <f>J7/110%</f>
         <v/>
       </c>
-      <c r="L7" s="22" t="inlineStr">
+      <c r="L7" s="23" t="inlineStr">
         <is>
           <t>컴엔더</t>
         </is>
@@ -10105,14 +10118,17 @@
       </c>
       <c r="P7" s="20" t="inlineStr">
         <is>
-          <t>정품직선형USB (+16,500원)
-RS232C (+24,200원)</t>
+          <t>RS232C (+24,200원)</t>
         </is>
       </c>
       <c r="Q7" s="21" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="R7" s="22">
+        <f>IF(Q7="X",F7+18000,F7)</f>
+        <v/>
       </c>
     </row>
     <row r="8">
@@ -10145,7 +10161,7 @@
         <f>J8/110%</f>
         <v/>
       </c>
-      <c r="L8" s="22" t="inlineStr">
+      <c r="L8" s="23" t="inlineStr">
         <is>
           <t>유니정보</t>
         </is>
@@ -10160,13 +10176,17 @@
       </c>
       <c r="P8" s="20" t="inlineStr">
         <is>
-          <t>USB (+0원)</t>
+          <t>없음</t>
         </is>
       </c>
       <c r="Q8" s="21" t="inlineStr">
         <is>
           <t>O</t>
         </is>
+      </c>
+      <c r="R8" s="22">
+        <f>IF(Q8="X",F8+18000,F8)</f>
+        <v/>
       </c>
     </row>
     <row r="9">
@@ -10199,7 +10219,7 @@
         <f>J9/110%</f>
         <v/>
       </c>
-      <c r="L9" s="22" t="inlineStr">
+      <c r="L9" s="23" t="inlineStr">
         <is>
           <t>더원시스</t>
         </is>
@@ -10214,14 +10234,17 @@
       </c>
       <c r="P9" s="20" t="inlineStr">
         <is>
-          <t>USB (+0원)
-RS232C (+24,200원)</t>
+          <t>RS232C (+24,200원)</t>
         </is>
       </c>
       <c r="Q9" s="21" t="inlineStr">
         <is>
           <t>O</t>
         </is>
+      </c>
+      <c r="R9" s="22">
+        <f>IF(Q9="X",F9+18000,F9)</f>
+        <v/>
       </c>
     </row>
     <row r="10">
@@ -10251,7 +10274,7 @@
         <f>J10/110%</f>
         <v/>
       </c>
-      <c r="L10" s="22" t="inlineStr">
+      <c r="L10" s="23" t="inlineStr">
         <is>
           <t>착한라벨</t>
         </is>
@@ -10266,14 +10289,17 @@
       </c>
       <c r="P10" s="20" t="inlineStr">
         <is>
-          <t>USB (+0원)
-RS232C (+33,000원)</t>
+          <t>RS232C (+33,000원)</t>
         </is>
       </c>
       <c r="Q10" s="21" t="inlineStr">
         <is>
           <t>O</t>
         </is>
+      </c>
+      <c r="R10" s="22">
+        <f>IF(Q10="X",F10+18000,F10)</f>
+        <v/>
       </c>
     </row>
     <row r="11">
@@ -10306,7 +10332,7 @@
         <f>J11/110%</f>
         <v/>
       </c>
-      <c r="L11" s="23" t="inlineStr">
+      <c r="L11" s="24" t="inlineStr">
         <is>
           <t>디앤에스테크(USB미포함)</t>
         </is>
@@ -10321,15 +10347,17 @@
       </c>
       <c r="P11" s="20" t="inlineStr">
         <is>
-          <t>코일형USB (+18,000원)
-직선형USB케이블 (+18,000원)
-RS232C (+24,200원)</t>
+          <t>RS232C (+24,200원)</t>
         </is>
       </c>
       <c r="Q11" s="21" t="inlineStr">
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="R11" s="22">
+        <f>IF(Q11="X",F11+18000,F11)</f>
+        <v/>
       </c>
     </row>
     <row r="12">
@@ -10362,7 +10390,7 @@
         <f>J12/110%</f>
         <v/>
       </c>
-      <c r="L12" s="22" t="inlineStr">
+      <c r="L12" s="23" t="inlineStr">
         <is>
           <t>유니정보</t>
         </is>
@@ -10416,7 +10444,7 @@
         <f>J13/110%</f>
         <v/>
       </c>
-      <c r="L13" s="22" t="inlineStr">
+      <c r="L13" s="23" t="inlineStr">
         <is>
           <t>코스모스몰</t>
         </is>
@@ -10470,7 +10498,7 @@
         <f>J14/110%</f>
         <v/>
       </c>
-      <c r="L14" s="22" t="inlineStr">
+      <c r="L14" s="23" t="inlineStr">
         <is>
           <t>더원시스</t>
         </is>
@@ -10496,6 +10524,10 @@
           <t>O</t>
         </is>
       </c>
+      <c r="R14" s="22">
+        <f>IF(Q14="X",F14+18000,F14)</f>
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="0" t="n">
@@ -10527,7 +10559,7 @@
         <f>J15/110%</f>
         <v/>
       </c>
-      <c r="L15" s="22" t="inlineStr">
+      <c r="L15" s="23" t="inlineStr">
         <is>
           <t>더원시스</t>
         </is>
@@ -10542,12 +10574,8 @@
       </c>
       <c r="P15" s="20" t="inlineStr">
         <is>
-          <t>정품직선형USB / 선택안함 (+18,000원)
-정품직선형USB / 스탠드거치대 (+73,000원)
-RS232C / 선택안함 (+24,200원)
+          <t>RS232C / 선택안함 (+24,200원)
 RS232C / 스탠드거치대 (+79,200원)
-코일형USB / 선택안함 (+18,000원)
-코일형USB / 스탠드거치대 (+73,000원)
 본체만(케이블없음) / 선택안함 (+0원)
 본체만(케이블없음) / 스탠드거치대 (+55,000원)</t>
         </is>
@@ -10556,6 +10584,10 @@
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="R15" s="22">
+        <f>IF(Q15="X",F15+18000,F15)</f>
+        <v/>
       </c>
     </row>
     <row r="16">
@@ -10588,7 +10620,7 @@
         <f>J16/110%</f>
         <v/>
       </c>
-      <c r="L16" s="22" t="inlineStr">
+      <c r="L16" s="23" t="inlineStr">
         <is>
           <t>코스모스몰</t>
         </is>
@@ -10603,14 +10635,17 @@
       </c>
       <c r="P16" s="20" t="inlineStr">
         <is>
-          <t>RS232C (+24,200원)
-USB (+0원)</t>
+          <t>RS232C (+24,200원)</t>
         </is>
       </c>
       <c r="Q16" s="21" t="inlineStr">
         <is>
           <t>O</t>
         </is>
+      </c>
+      <c r="R16" s="22">
+        <f>IF(Q16="X",F16+18000,F16)</f>
+        <v/>
       </c>
     </row>
     <row r="17">
@@ -10640,7 +10675,7 @@
         <f>J17/110%</f>
         <v/>
       </c>
-      <c r="L17" s="22" t="inlineStr">
+      <c r="L17" s="23" t="inlineStr">
         <is>
           <t>코스모스몰</t>
         </is>
@@ -10655,14 +10690,17 @@
       </c>
       <c r="P17" s="20" t="inlineStr">
         <is>
-          <t>RS232C (+24,200원)
-USB (+0원)</t>
+          <t>RS232C (+24,200원)</t>
         </is>
       </c>
       <c r="Q17" s="21" t="inlineStr">
         <is>
           <t>O</t>
         </is>
+      </c>
+      <c r="R17" s="22">
+        <f>IF(Q17="X",F17+18000,F17)</f>
+        <v/>
       </c>
     </row>
     <row r="18">
@@ -10695,7 +10733,7 @@
         <f>J18/110%</f>
         <v/>
       </c>
-      <c r="L18" s="22" t="inlineStr">
+      <c r="L18" s="23" t="inlineStr">
         <is>
           <t>바코드랩</t>
         </is>
@@ -10710,13 +10748,17 @@
       </c>
       <c r="P18" s="20" t="inlineStr">
         <is>
-          <t>USB (+0원)</t>
+          <t>없음</t>
         </is>
       </c>
       <c r="Q18" s="21" t="inlineStr">
         <is>
           <t>O</t>
         </is>
+      </c>
+      <c r="R18" s="22">
+        <f>IF(Q18="X",F18+18000,F18)</f>
+        <v/>
       </c>
     </row>
     <row r="19">
@@ -10749,7 +10791,7 @@
         <f>J19/110%</f>
         <v/>
       </c>
-      <c r="L19" s="22" t="inlineStr">
+      <c r="L19" s="23" t="inlineStr">
         <is>
           <t>바코드랩</t>
         </is>
@@ -10764,13 +10806,17 @@
       </c>
       <c r="P19" s="20" t="inlineStr">
         <is>
-          <t>USB (+0원)</t>
+          <t>없음</t>
         </is>
       </c>
       <c r="Q19" s="21" t="inlineStr">
         <is>
           <t>O</t>
         </is>
+      </c>
+      <c r="R19" s="22">
+        <f>IF(Q19="X",F19+18000,F19)</f>
+        <v/>
       </c>
     </row>
     <row r="20">
@@ -10800,7 +10846,7 @@
         <f>J20/110%</f>
         <v/>
       </c>
-      <c r="L20" s="22" t="inlineStr">
+      <c r="L20" s="23" t="inlineStr">
         <is>
           <t>코스모스몰</t>
         </is>
@@ -10815,14 +10861,17 @@
       </c>
       <c r="P20" s="20" t="inlineStr">
         <is>
-          <t>USB (+0원)
-RS232C (+24,200원)</t>
+          <t>RS232C (+24,200원)</t>
         </is>
       </c>
       <c r="Q20" s="21" t="inlineStr">
         <is>
           <t>O</t>
         </is>
+      </c>
+      <c r="R20" s="22">
+        <f>IF(Q20="X",F20+18000,F20)</f>
+        <v/>
       </c>
     </row>
     <row r="21">
@@ -10852,7 +10901,7 @@
         <f>J21/110%</f>
         <v/>
       </c>
-      <c r="L21" s="22" t="inlineStr">
+      <c r="L21" s="23" t="inlineStr">
         <is>
           <t>유니정보,착한라벨,우주사무기</t>
         </is>
@@ -10867,14 +10916,17 @@
       </c>
       <c r="P21" s="20" t="inlineStr">
         <is>
-          <t>RS232C (+49,500원)
-USB (+0원)</t>
+          <t>RS232C (+49,500원)</t>
         </is>
       </c>
       <c r="Q21" s="21" t="inlineStr">
         <is>
           <t>O</t>
         </is>
+      </c>
+      <c r="R21" s="22">
+        <f>IF(Q21="X",F21+18000,F21)</f>
+        <v/>
       </c>
     </row>
     <row r="22">
@@ -10907,7 +10959,7 @@
         <f>J22/110%</f>
         <v/>
       </c>
-      <c r="L22" s="22" t="inlineStr">
+      <c r="L22" s="23" t="inlineStr">
         <is>
           <t>코스모스전문몰</t>
         </is>
@@ -10923,8 +10975,6 @@
       <c r="P22" s="20" t="inlineStr">
         <is>
           <t>본체+크래들만(케이블없음) (+0원)
-정품직선형USB (+18,000원)
-코일형USB (+18,000원)
 RS232C (+24,200원)</t>
         </is>
       </c>
@@ -10932,6 +10982,10 @@
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="R22" s="22">
+        <f>IF(Q22="X",F22+18000,F22)</f>
+        <v/>
       </c>
     </row>
     <row r="23">
@@ -10964,7 +11018,7 @@
         <f>J23/110%</f>
         <v/>
       </c>
-      <c r="L23" s="22" t="inlineStr">
+      <c r="L23" s="23" t="inlineStr">
         <is>
           <t>코스모스몰,더원시스</t>
         </is>
@@ -10979,13 +11033,17 @@
       </c>
       <c r="P23" s="20" t="inlineStr">
         <is>
-          <t>USB (+0원)</t>
+          <t>없음</t>
         </is>
       </c>
       <c r="Q23" s="21" t="inlineStr">
         <is>
           <t>O</t>
         </is>
+      </c>
+      <c r="R23" s="22">
+        <f>IF(Q23="X",F23+18000,F23)</f>
+        <v/>
       </c>
     </row>
     <row r="24">
@@ -11011,7 +11069,7 @@
       </c>
       <c r="J24" s="19" t="n"/>
       <c r="K24" s="17" t="n"/>
-      <c r="L24" s="22" t="n"/>
+      <c r="L24" s="23" t="n"/>
       <c r="M24" s="3" t="n"/>
       <c r="N24" s="3" t="n"/>
       <c r="O24" t="inlineStr">
@@ -11021,9 +11079,7 @@
       </c>
       <c r="P24" s="20" t="inlineStr">
         <is>
-          <t>직선형USB케이블 (+18,000원)
-RS232C (+24,200원)
-코일형USB (+18,000원)
+          <t>RS232C (+24,200원)
 본체만(케이블없음) (+0원)</t>
         </is>
       </c>
@@ -11031,6 +11087,10 @@
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="R24" s="22">
+        <f>IF(Q24="X",F24+18000,F24)</f>
+        <v/>
       </c>
     </row>
     <row r="25">
@@ -11056,7 +11116,7 @@
       </c>
       <c r="J25" s="19" t="n"/>
       <c r="K25" s="17" t="n"/>
-      <c r="L25" s="22" t="n"/>
+      <c r="L25" s="23" t="n"/>
       <c r="M25" s="3" t="n"/>
       <c r="N25" s="3" t="n"/>
       <c r="O25" t="inlineStr">
@@ -11066,9 +11126,7 @@
       </c>
       <c r="P25" s="20" t="inlineStr">
         <is>
-          <t>정품직선형USB (+18,000원)
-RS232C (+24,200원)
-코일형USB (+18,000원)
+          <t>RS232C (+24,200원)
 본체+크래들만(케이블없음) (+0원)</t>
         </is>
       </c>
@@ -11076,6 +11134,10 @@
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="R25" s="22">
+        <f>IF(Q25="X",F25+18000,F25)</f>
+        <v/>
       </c>
     </row>
     <row r="26">
@@ -11101,7 +11163,7 @@
       </c>
       <c r="J26" s="19" t="n"/>
       <c r="K26" s="17" t="n"/>
-      <c r="L26" s="22" t="n"/>
+      <c r="L26" s="23" t="n"/>
       <c r="M26" s="3" t="n"/>
       <c r="N26" s="3" t="n"/>
       <c r="O26" t="inlineStr">
@@ -11111,9 +11173,7 @@
       </c>
       <c r="P26" s="20" t="inlineStr">
         <is>
-          <t>정품직선형USB (+18,000원)
-RS232C (+24,200원)
-코일형USB (+18,000원)
+          <t>RS232C (+24,200원)
 본체+크래들만(케이블없음) (+0원)</t>
         </is>
       </c>
@@ -11121,6 +11181,10 @@
         <is>
           <t>X</t>
         </is>
+      </c>
+      <c r="R26" s="22">
+        <f>IF(Q26="X",F26+18000,F26)</f>
+        <v/>
       </c>
     </row>
     <row r="27">
@@ -11146,7 +11210,7 @@
       </c>
       <c r="J27" s="19" t="n"/>
       <c r="K27" s="17" t="n"/>
-      <c r="L27" s="22" t="n"/>
+      <c r="L27" s="23" t="n"/>
       <c r="M27" s="3" t="n"/>
       <c r="N27" s="3" t="n"/>
       <c r="O27" t="inlineStr">
@@ -11188,7 +11252,7 @@
       </c>
       <c r="J28" s="19" t="n"/>
       <c r="K28" s="17" t="n"/>
-      <c r="L28" s="22" t="n"/>
+      <c r="L28" s="23" t="n"/>
       <c r="M28" s="3" t="n"/>
       <c r="N28" s="3" t="n"/>
       <c r="O28" t="inlineStr">
@@ -11230,7 +11294,7 @@
       </c>
       <c r="J29" s="19" t="n"/>
       <c r="K29" s="17" t="n"/>
-      <c r="L29" s="22" t="n"/>
+      <c r="L29" s="23" t="n"/>
       <c r="M29" s="3" t="n"/>
       <c r="N29" s="3" t="n"/>
       <c r="O29" t="inlineStr">
@@ -11272,7 +11336,7 @@
       </c>
       <c r="J30" s="19" t="n"/>
       <c r="K30" s="17" t="n"/>
-      <c r="L30" s="22" t="n"/>
+      <c r="L30" s="23" t="n"/>
       <c r="M30" s="3" t="n"/>
       <c r="N30" s="3" t="n"/>
       <c r="O30" t="inlineStr">
@@ -11314,7 +11378,7 @@
       </c>
       <c r="J31" s="19" t="n"/>
       <c r="K31" s="17" t="n"/>
-      <c r="L31" s="22" t="n"/>
+      <c r="L31" s="23" t="n"/>
       <c r="M31" s="3" t="n"/>
       <c r="N31" s="3" t="n"/>
       <c r="O31" t="inlineStr">
@@ -11557,35 +11621,35 @@
           <t xml:space="preserve"> 키패드(핸드헬드)</t>
         </is>
       </c>
-      <c r="D4" s="24" t="n">
+      <c r="D4" s="25" t="n">
         <v>1840000</v>
       </c>
-      <c r="E4" s="24">
+      <c r="E4" s="25">
         <f>D4*1.1</f>
         <v/>
       </c>
-      <c r="F4" s="24" t="n">
+      <c r="F4" s="25" t="n">
         <v>2640000</v>
       </c>
-      <c r="G4" s="24">
+      <c r="G4" s="25">
         <f>F4/110%</f>
         <v/>
       </c>
-      <c r="H4" s="25" t="n">
+      <c r="H4" s="26" t="n">
         <v>2500000</v>
       </c>
-      <c r="I4" s="25">
+      <c r="I4" s="26">
         <f>ROUND(H4*1.1/0.95,-1)</f>
         <v/>
       </c>
-      <c r="J4" s="24" t="n">
+      <c r="J4" s="25" t="n">
         <v>2640000</v>
       </c>
-      <c r="K4" s="24">
+      <c r="K4" s="25">
         <f>J4/1.1</f>
         <v/>
       </c>
-      <c r="L4" s="24" t="inlineStr">
+      <c r="L4" s="25" t="inlineStr">
         <is>
           <t>코스모스몰</t>
         </is>
@@ -11772,32 +11836,32 @@
           <t xml:space="preserve"> 프리미엄풀터치</t>
         </is>
       </c>
-      <c r="D8" s="24" t="n">
+      <c r="D8" s="25" t="n">
         <v>2500000</v>
       </c>
-      <c r="E8" s="24">
+      <c r="E8" s="25">
         <f>D8*1.1</f>
         <v/>
       </c>
-      <c r="F8" s="24" t="n">
+      <c r="F8" s="25" t="n">
         <v>2640000</v>
       </c>
-      <c r="G8" s="25" t="n"/>
-      <c r="H8" s="25" t="n">
+      <c r="G8" s="26" t="n"/>
+      <c r="H8" s="26" t="n">
         <v>3000000</v>
       </c>
-      <c r="I8" s="25">
+      <c r="I8" s="26">
         <f>ROUND(H8*1.1/0.95,-1)</f>
         <v/>
       </c>
-      <c r="J8" s="24" t="n">
+      <c r="J8" s="25" t="n">
         <v>2577960</v>
       </c>
-      <c r="K8" s="24">
+      <c r="K8" s="25">
         <f>J8/1.1</f>
         <v/>
       </c>
-      <c r="L8" s="24" t="inlineStr">
+      <c r="L8" s="25" t="inlineStr">
         <is>
           <t>솔바텍지마켓</t>
         </is>
@@ -11876,30 +11940,30 @@
           <t xml:space="preserve"> 키패드(핸드헬드)</t>
         </is>
       </c>
-      <c r="D10" s="24" t="n">
+      <c r="D10" s="25" t="n">
         <v>1490000</v>
       </c>
-      <c r="E10" s="24">
+      <c r="E10" s="25">
         <f>D10*1.1</f>
         <v/>
       </c>
-      <c r="F10" s="24" t="n">
+      <c r="F10" s="25" t="n">
         <v>2750000</v>
       </c>
-      <c r="G10" s="24">
+      <c r="G10" s="25">
         <f>F10/110%</f>
         <v/>
       </c>
-      <c r="H10" s="24" t="n"/>
-      <c r="I10" s="24" t="n"/>
-      <c r="J10" s="24" t="n">
+      <c r="H10" s="25" t="n"/>
+      <c r="I10" s="25" t="n"/>
+      <c r="J10" s="25" t="n">
         <v>2750000</v>
       </c>
-      <c r="K10" s="24">
+      <c r="K10" s="25">
         <f>J10/1.1</f>
         <v/>
       </c>
-      <c r="L10" s="24" t="inlineStr">
+      <c r="L10" s="25" t="inlineStr">
         <is>
           <t>코스모스몰,더원시스</t>
         </is>
@@ -12070,7 +12134,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="I18" s="26" t="n"/>
+      <c r="I18" s="27" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -12084,7 +12148,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H83"/>
+  <dimension ref="A1:H45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" style="16" min="1" max="1"/>
@@ -12148,7 +12212,7 @@
           <t>LS2208 SR</t>
         </is>
       </c>
-      <c r="C2" s="27">
+      <c r="C2" s="22">
         <f>'지브라-스캐너'!F2</f>
         <v/>
       </c>
@@ -12159,17 +12223,17 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>정품직선형USB</t>
-        </is>
-      </c>
-      <c r="F2" s="27" t="n">
-        <v>18000</v>
-      </c>
-      <c r="G2" s="27">
+          <t>RS232C</t>
+        </is>
+      </c>
+      <c r="F2" s="22" t="n">
+        <v>24200</v>
+      </c>
+      <c r="G2" s="22">
         <f>C2+F2</f>
         <v/>
       </c>
-      <c r="H2" s="27">
+      <c r="H2" s="22">
         <f>G2/110%</f>
         <v/>
       </c>
@@ -12183,7 +12247,7 @@
           <t>LS2208 SR</t>
         </is>
       </c>
-      <c r="C3" s="27">
+      <c r="C3" s="22">
         <f>'지브라-스캐너'!F2</f>
         <v/>
       </c>
@@ -12194,17 +12258,17 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>코일형USB</t>
-        </is>
-      </c>
-      <c r="F3" s="27" t="n">
-        <v>18000</v>
-      </c>
-      <c r="G3" s="27">
+          <t>본체만(케이블없음)</t>
+        </is>
+      </c>
+      <c r="F3" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" s="22">
         <f>C3+F3</f>
         <v/>
       </c>
-      <c r="H3" s="27">
+      <c r="H3" s="22">
         <f>G3/110%</f>
         <v/>
       </c>
@@ -12215,11 +12279,11 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>LS2208 SR</t>
-        </is>
-      </c>
-      <c r="C4" s="27">
-        <f>'지브라-스캐너'!F2</f>
+          <t>DS2278</t>
+        </is>
+      </c>
+      <c r="C4" s="22">
+        <f>'지브라-스캐너'!F3</f>
         <v/>
       </c>
       <c r="D4" t="inlineStr">
@@ -12232,14 +12296,14 @@
           <t>RS232C</t>
         </is>
       </c>
-      <c r="F4" s="27" t="n">
+      <c r="F4" s="22" t="n">
         <v>24200</v>
       </c>
-      <c r="G4" s="27">
+      <c r="G4" s="22">
         <f>C4+F4</f>
         <v/>
       </c>
-      <c r="H4" s="27">
+      <c r="H4" s="22">
         <f>G4/110%</f>
         <v/>
       </c>
@@ -12250,11 +12314,11 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>LS2208 SR</t>
-        </is>
-      </c>
-      <c r="C5" s="27">
-        <f>'지브라-스캐너'!F2</f>
+          <t>DS2278</t>
+        </is>
+      </c>
+      <c r="C5" s="22">
+        <f>'지브라-스캐너'!F3</f>
         <v/>
       </c>
       <c r="D5" t="inlineStr">
@@ -12264,17 +12328,17 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>본체만(케이블없음)</t>
-        </is>
-      </c>
-      <c r="F5" s="27" t="n">
+          <t>본체+크래들만(케이블없음)</t>
+        </is>
+      </c>
+      <c r="F5" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="G5" s="27">
+      <c r="G5" s="22">
         <f>C5+F5</f>
         <v/>
       </c>
-      <c r="H5" s="27">
+      <c r="H5" s="22">
         <f>G5/110%</f>
         <v/>
       </c>
@@ -12285,31 +12349,31 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>DS2278</t>
-        </is>
-      </c>
-      <c r="C6" s="27">
-        <f>'지브라-스캐너'!F3</f>
+          <t>DS2208</t>
+        </is>
+      </c>
+      <c r="C6" s="22">
+        <f>'지브라-스캐너'!F4</f>
         <v/>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>인터페이스</t>
+          <t>인터페이스 / 악세사리</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>정품직선형USB</t>
-        </is>
-      </c>
-      <c r="F6" s="27" t="n">
-        <v>18000</v>
-      </c>
-      <c r="G6" s="27">
+          <t>RS232C / 선택안함</t>
+        </is>
+      </c>
+      <c r="F6" s="22" t="n">
+        <v>24200</v>
+      </c>
+      <c r="G6" s="22">
         <f>C6+F6</f>
         <v/>
       </c>
-      <c r="H6" s="27">
+      <c r="H6" s="22">
         <f>G6/110%</f>
         <v/>
       </c>
@@ -12320,31 +12384,31 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>DS2278</t>
-        </is>
-      </c>
-      <c r="C7" s="27">
-        <f>'지브라-스캐너'!F3</f>
+          <t>DS2208</t>
+        </is>
+      </c>
+      <c r="C7" s="22">
+        <f>'지브라-스캐너'!F4</f>
         <v/>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>인터페이스</t>
+          <t>인터페이스 / 악세사리</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>코일형USB</t>
-        </is>
-      </c>
-      <c r="F7" s="27" t="n">
-        <v>18000</v>
-      </c>
-      <c r="G7" s="27">
+          <t>RS232C / 스탠드거치대</t>
+        </is>
+      </c>
+      <c r="F7" s="22" t="n">
+        <v>79200</v>
+      </c>
+      <c r="G7" s="22">
         <f>C7+F7</f>
         <v/>
       </c>
-      <c r="H7" s="27">
+      <c r="H7" s="22">
         <f>G7/110%</f>
         <v/>
       </c>
@@ -12355,31 +12419,31 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>DS2278</t>
-        </is>
-      </c>
-      <c r="C8" s="27">
-        <f>'지브라-스캐너'!F3</f>
+          <t>DS2208</t>
+        </is>
+      </c>
+      <c r="C8" s="22">
+        <f>'지브라-스캐너'!F4</f>
         <v/>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>인터페이스</t>
+          <t>인터페이스 / 악세사리</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>RS232C</t>
-        </is>
-      </c>
-      <c r="F8" s="27" t="n">
-        <v>24200</v>
-      </c>
-      <c r="G8" s="27">
+          <t>본체만(케이블없음) / 선택안함</t>
+        </is>
+      </c>
+      <c r="F8" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="22">
         <f>C8+F8</f>
         <v/>
       </c>
-      <c r="H8" s="27">
+      <c r="H8" s="22">
         <f>G8/110%</f>
         <v/>
       </c>
@@ -12390,31 +12454,31 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>DS2278</t>
-        </is>
-      </c>
-      <c r="C9" s="27">
-        <f>'지브라-스캐너'!F3</f>
+          <t>DS2208</t>
+        </is>
+      </c>
+      <c r="C9" s="22">
+        <f>'지브라-스캐너'!F4</f>
         <v/>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>인터페이스</t>
+          <t>인터페이스 / 악세사리</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>본체+크래들만(케이블없음)</t>
-        </is>
-      </c>
-      <c r="F9" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="G9" s="27">
+          <t>본체만(케이블없음) / 스탠드거치대</t>
+        </is>
+      </c>
+      <c r="F9" s="22" t="n">
+        <v>55000</v>
+      </c>
+      <c r="G9" s="22">
         <f>C9+F9</f>
         <v/>
       </c>
-      <c r="H9" s="27">
+      <c r="H9" s="22">
         <f>G9/110%</f>
         <v/>
       </c>
@@ -12425,31 +12489,31 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>DS2208</t>
-        </is>
-      </c>
-      <c r="C10" s="27">
-        <f>'지브라-스캐너'!F4</f>
+          <t>DS8108</t>
+        </is>
+      </c>
+      <c r="C10" s="22">
+        <f>'지브라-스캐너'!F5</f>
         <v/>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>인터페이스 / 악세사리</t>
+          <t>인터페이스</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>정품직선형USB / 선택안함</t>
-        </is>
-      </c>
-      <c r="F10" s="27" t="n">
-        <v>18000</v>
-      </c>
-      <c r="G10" s="27">
+          <t>RS232C</t>
+        </is>
+      </c>
+      <c r="F10" s="22" t="n">
+        <v>24200</v>
+      </c>
+      <c r="G10" s="22">
         <f>C10+F10</f>
         <v/>
       </c>
-      <c r="H10" s="27">
+      <c r="H10" s="22">
         <f>G10/110%</f>
         <v/>
       </c>
@@ -12460,31 +12524,31 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>DS2208</t>
-        </is>
-      </c>
-      <c r="C11" s="27">
-        <f>'지브라-스캐너'!F4</f>
+          <t>DS8108</t>
+        </is>
+      </c>
+      <c r="C11" s="22">
+        <f>'지브라-스캐너'!F5</f>
         <v/>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>인터페이스 / 악세사리</t>
+          <t>인터페이스</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>정품직선형USB / 스탠드거치대</t>
-        </is>
-      </c>
-      <c r="F11" s="27" t="n">
-        <v>73000</v>
-      </c>
-      <c r="G11" s="27">
+          <t>본체만</t>
+        </is>
+      </c>
+      <c r="F11" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" s="22">
         <f>C11+F11</f>
         <v/>
       </c>
-      <c r="H11" s="27">
+      <c r="H11" s="22">
         <f>G11/110%</f>
         <v/>
       </c>
@@ -12495,11 +12559,11 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>DS2208</t>
-        </is>
-      </c>
-      <c r="C12" s="27">
-        <f>'지브라-스캐너'!F4</f>
+          <t>DS4608 SR</t>
+        </is>
+      </c>
+      <c r="C12" s="22">
+        <f>'지브라-스캐너'!F6</f>
         <v/>
       </c>
       <c r="D12" t="inlineStr">
@@ -12512,14 +12576,14 @@
           <t>RS232C / 선택안함</t>
         </is>
       </c>
-      <c r="F12" s="27" t="n">
+      <c r="F12" s="22" t="n">
         <v>24200</v>
       </c>
-      <c r="G12" s="27">
+      <c r="G12" s="22">
         <f>C12+F12</f>
         <v/>
       </c>
-      <c r="H12" s="27">
+      <c r="H12" s="22">
         <f>G12/110%</f>
         <v/>
       </c>
@@ -12530,11 +12594,11 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>DS2208</t>
-        </is>
-      </c>
-      <c r="C13" s="27">
-        <f>'지브라-스캐너'!F4</f>
+          <t>DS4608 SR</t>
+        </is>
+      </c>
+      <c r="C13" s="22">
+        <f>'지브라-스캐너'!F6</f>
         <v/>
       </c>
       <c r="D13" t="inlineStr">
@@ -12547,14 +12611,14 @@
           <t>RS232C / 스탠드거치대</t>
         </is>
       </c>
-      <c r="F13" s="27" t="n">
+      <c r="F13" s="22" t="n">
         <v>79200</v>
       </c>
-      <c r="G13" s="27">
+      <c r="G13" s="22">
         <f>C13+F13</f>
         <v/>
       </c>
-      <c r="H13" s="27">
+      <c r="H13" s="22">
         <f>G13/110%</f>
         <v/>
       </c>
@@ -12565,11 +12629,11 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>DS2208</t>
-        </is>
-      </c>
-      <c r="C14" s="27">
-        <f>'지브라-스캐너'!F4</f>
+          <t>DS4608 SR</t>
+        </is>
+      </c>
+      <c r="C14" s="22">
+        <f>'지브라-스캐너'!F6</f>
         <v/>
       </c>
       <c r="D14" t="inlineStr">
@@ -12579,17 +12643,17 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>코일형USB / 선택안함</t>
-        </is>
-      </c>
-      <c r="F14" s="27" t="n">
-        <v>18000</v>
-      </c>
-      <c r="G14" s="27">
+          <t>본체만(케이블없음) / 선택안함</t>
+        </is>
+      </c>
+      <c r="F14" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" s="22">
         <f>C14+F14</f>
         <v/>
       </c>
-      <c r="H14" s="27">
+      <c r="H14" s="22">
         <f>G14/110%</f>
         <v/>
       </c>
@@ -12600,11 +12664,11 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>DS2208</t>
-        </is>
-      </c>
-      <c r="C15" s="27">
-        <f>'지브라-스캐너'!F4</f>
+          <t>DS4608 SR</t>
+        </is>
+      </c>
+      <c r="C15" s="22">
+        <f>'지브라-스캐너'!F6</f>
         <v/>
       </c>
       <c r="D15" t="inlineStr">
@@ -12614,17 +12678,17 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>코일형USB / 스탠드거치대</t>
-        </is>
-      </c>
-      <c r="F15" s="27" t="n">
-        <v>73000</v>
-      </c>
-      <c r="G15" s="27">
+          <t>본체만(케이블없음) / 스탠드거치대</t>
+        </is>
+      </c>
+      <c r="F15" s="22" t="n">
+        <v>55000</v>
+      </c>
+      <c r="G15" s="22">
         <f>C15+F15</f>
         <v/>
       </c>
-      <c r="H15" s="27">
+      <c r="H15" s="22">
         <f>G15/110%</f>
         <v/>
       </c>
@@ -12635,31 +12699,31 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>DS2208</t>
-        </is>
-      </c>
-      <c r="C16" s="27">
-        <f>'지브라-스캐너'!F4</f>
+          <t>LI2208</t>
+        </is>
+      </c>
+      <c r="C16" s="22">
+        <f>'지브라-스캐너'!F7</f>
         <v/>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>인터페이스 / 악세사리</t>
+          <t>인터페이스</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>본체만(케이블없음) / 선택안함</t>
-        </is>
-      </c>
-      <c r="F16" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="G16" s="27">
+          <t>RS232C</t>
+        </is>
+      </c>
+      <c r="F16" s="22" t="n">
+        <v>24200</v>
+      </c>
+      <c r="G16" s="22">
         <f>C16+F16</f>
         <v/>
       </c>
-      <c r="H16" s="27">
+      <c r="H16" s="22">
         <f>G16/110%</f>
         <v/>
       </c>
@@ -12670,31 +12734,31 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>DS2208</t>
-        </is>
-      </c>
-      <c r="C17" s="27">
-        <f>'지브라-스캐너'!F4</f>
+          <t>DS3608 SR</t>
+        </is>
+      </c>
+      <c r="C17" s="22">
+        <f>'지브라-스캐너'!F9</f>
         <v/>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>인터페이스 / 악세사리</t>
+          <t>인터페이스</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>본체만(케이블없음) / 스탠드거치대</t>
-        </is>
-      </c>
-      <c r="F17" s="27" t="n">
-        <v>55000</v>
-      </c>
-      <c r="G17" s="27">
+          <t>RS232C</t>
+        </is>
+      </c>
+      <c r="F17" s="22" t="n">
+        <v>24200</v>
+      </c>
+      <c r="G17" s="22">
         <f>C17+F17</f>
         <v/>
       </c>
-      <c r="H17" s="27">
+      <c r="H17" s="22">
         <f>G17/110%</f>
         <v/>
       </c>
@@ -12705,11 +12769,11 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>DS8108</t>
-        </is>
-      </c>
-      <c r="C18" s="27">
-        <f>'지브라-스캐너'!F5</f>
+          <t>LI3678</t>
+        </is>
+      </c>
+      <c r="C18" s="22">
+        <f>'지브라-스캐너'!F10</f>
         <v/>
       </c>
       <c r="D18" t="inlineStr">
@@ -12719,17 +12783,17 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>정품직선형USB</t>
-        </is>
-      </c>
-      <c r="F18" s="27" t="n">
-        <v>16500</v>
-      </c>
-      <c r="G18" s="27">
+          <t>RS232C</t>
+        </is>
+      </c>
+      <c r="F18" s="22" t="n">
+        <v>33000</v>
+      </c>
+      <c r="G18" s="22">
         <f>C18+F18</f>
         <v/>
       </c>
-      <c r="H18" s="27">
+      <c r="H18" s="22">
         <f>G18/110%</f>
         <v/>
       </c>
@@ -12740,11 +12804,11 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>DS8108</t>
-        </is>
-      </c>
-      <c r="C19" s="27">
-        <f>'지브라-스캐너'!F5</f>
+          <t>DS9908</t>
+        </is>
+      </c>
+      <c r="C19" s="22">
+        <f>'지브라-스캐너'!F11</f>
         <v/>
       </c>
       <c r="D19" t="inlineStr">
@@ -12757,14 +12821,14 @@
           <t>RS232C</t>
         </is>
       </c>
-      <c r="F19" s="27" t="n">
+      <c r="F19" s="22" t="n">
         <v>24200</v>
       </c>
-      <c r="G19" s="27">
+      <c r="G19" s="22">
         <f>C19+F19</f>
         <v/>
       </c>
-      <c r="H19" s="27">
+      <c r="H19" s="22">
         <f>G19/110%</f>
         <v/>
       </c>
@@ -12775,31 +12839,31 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>DS8108</t>
-        </is>
-      </c>
-      <c r="C20" s="27">
-        <f>'지브라-스캐너'!F5</f>
+          <t>CS6080</t>
+        </is>
+      </c>
+      <c r="C20" s="22">
+        <f>'지브라-스캐너'!F13</f>
         <v/>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>인터페이스</t>
+          <t>스캔엔진</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>본체만</t>
-        </is>
-      </c>
-      <c r="F20" s="27" t="n">
+          <t>2D</t>
+        </is>
+      </c>
+      <c r="F20" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="G20" s="27">
+      <c r="G20" s="22">
         <f>C20+F20</f>
         <v/>
       </c>
-      <c r="H20" s="27">
+      <c r="H20" s="22">
         <f>G20/110%</f>
         <v/>
       </c>
@@ -12810,31 +12874,31 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>DS4608 SR</t>
-        </is>
-      </c>
-      <c r="C21" s="27">
-        <f>'지브라-스캐너'!F6</f>
+          <t>DS3678 SR</t>
+        </is>
+      </c>
+      <c r="C21" s="22">
+        <f>'지브라-스캐너'!F14</f>
         <v/>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>인터페이스 / 악세사리</t>
+          <t>인터페이스</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>정품직선형USB / 선택안함</t>
-        </is>
-      </c>
-      <c r="F21" s="27" t="n">
-        <v>18000</v>
-      </c>
-      <c r="G21" s="27">
+          <t>SR버전+USB케이블</t>
+        </is>
+      </c>
+      <c r="F21" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" s="22">
         <f>C21+F21</f>
         <v/>
       </c>
-      <c r="H21" s="27">
+      <c r="H21" s="22">
         <f>G21/110%</f>
         <v/>
       </c>
@@ -12845,31 +12909,31 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>DS4608 SR</t>
-        </is>
-      </c>
-      <c r="C22" s="27">
-        <f>'지브라-스캐너'!F6</f>
+          <t>DS3678 SR</t>
+        </is>
+      </c>
+      <c r="C22" s="22">
+        <f>'지브라-스캐너'!F14</f>
         <v/>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>인터페이스 / 악세사리</t>
+          <t>인터페이스</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>정품직선형USB / 스탠드거치대</t>
-        </is>
-      </c>
-      <c r="F22" s="27" t="n">
-        <v>73000</v>
-      </c>
-      <c r="G22" s="27">
+          <t>HD버전+USB케이블</t>
+        </is>
+      </c>
+      <c r="F22" s="22" t="n">
+        <v>220000</v>
+      </c>
+      <c r="G22" s="22">
         <f>C22+F22</f>
         <v/>
       </c>
-      <c r="H22" s="27">
+      <c r="H22" s="22">
         <f>G22/110%</f>
         <v/>
       </c>
@@ -12880,31 +12944,31 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>DS4608 SR</t>
-        </is>
-      </c>
-      <c r="C23" s="27">
-        <f>'지브라-스캐너'!F6</f>
+          <t>DS3678 SR</t>
+        </is>
+      </c>
+      <c r="C23" s="22">
+        <f>'지브라-스캐너'!F14</f>
         <v/>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>인터페이스 / 악세사리</t>
+          <t>인터페이스</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>RS232C / 선택안함</t>
-        </is>
-      </c>
-      <c r="F23" s="27" t="n">
-        <v>24200</v>
-      </c>
-      <c r="G23" s="27">
+          <t>SR버전+RS232C케이블</t>
+        </is>
+      </c>
+      <c r="F23" s="22" t="n">
+        <v>33000</v>
+      </c>
+      <c r="G23" s="22">
         <f>C23+F23</f>
         <v/>
       </c>
-      <c r="H23" s="27">
+      <c r="H23" s="22">
         <f>G23/110%</f>
         <v/>
       </c>
@@ -12915,31 +12979,31 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>DS4608 SR</t>
-        </is>
-      </c>
-      <c r="C24" s="27">
-        <f>'지브라-스캐너'!F6</f>
+          <t>DS3678 SR</t>
+        </is>
+      </c>
+      <c r="C24" s="22">
+        <f>'지브라-스캐너'!F14</f>
         <v/>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>인터페이스 / 악세사리</t>
+          <t>인터페이스</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>RS232C / 스탠드거치대</t>
-        </is>
-      </c>
-      <c r="F24" s="27" t="n">
-        <v>79200</v>
-      </c>
-      <c r="G24" s="27">
+          <t>HD버전+RS232C케이블</t>
+        </is>
+      </c>
+      <c r="F24" s="22" t="n">
+        <v>275000</v>
+      </c>
+      <c r="G24" s="22">
         <f>C24+F24</f>
         <v/>
       </c>
-      <c r="H24" s="27">
+      <c r="H24" s="22">
         <f>G24/110%</f>
         <v/>
       </c>
@@ -12950,11 +13014,11 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>DS4608 SR</t>
-        </is>
-      </c>
-      <c r="C25" s="27">
-        <f>'지브라-스캐너'!F6</f>
+          <t>DS4608 XD</t>
+        </is>
+      </c>
+      <c r="C25" s="22">
+        <f>'지브라-스캐너'!F15</f>
         <v/>
       </c>
       <c r="D25" t="inlineStr">
@@ -12964,17 +13028,17 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>코일형USB / 선택안함</t>
-        </is>
-      </c>
-      <c r="F25" s="27" t="n">
-        <v>18000</v>
-      </c>
-      <c r="G25" s="27">
+          <t>RS232C / 선택안함</t>
+        </is>
+      </c>
+      <c r="F25" s="22" t="n">
+        <v>24200</v>
+      </c>
+      <c r="G25" s="22">
         <f>C25+F25</f>
         <v/>
       </c>
-      <c r="H25" s="27">
+      <c r="H25" s="22">
         <f>G25/110%</f>
         <v/>
       </c>
@@ -12985,11 +13049,11 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>DS4608 SR</t>
-        </is>
-      </c>
-      <c r="C26" s="27">
-        <f>'지브라-스캐너'!F6</f>
+          <t>DS4608 XD</t>
+        </is>
+      </c>
+      <c r="C26" s="22">
+        <f>'지브라-스캐너'!F15</f>
         <v/>
       </c>
       <c r="D26" t="inlineStr">
@@ -12999,17 +13063,17 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>코일형USB / 스탠드거치대</t>
-        </is>
-      </c>
-      <c r="F26" s="27" t="n">
-        <v>73000</v>
-      </c>
-      <c r="G26" s="27">
+          <t>RS232C / 스탠드거치대</t>
+        </is>
+      </c>
+      <c r="F26" s="22" t="n">
+        <v>79200</v>
+      </c>
+      <c r="G26" s="22">
         <f>C26+F26</f>
         <v/>
       </c>
-      <c r="H26" s="27">
+      <c r="H26" s="22">
         <f>G26/110%</f>
         <v/>
       </c>
@@ -13020,11 +13084,11 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>DS4608 SR</t>
-        </is>
-      </c>
-      <c r="C27" s="27">
-        <f>'지브라-스캐너'!F6</f>
+          <t>DS4608 XD</t>
+        </is>
+      </c>
+      <c r="C27" s="22">
+        <f>'지브라-스캐너'!F15</f>
         <v/>
       </c>
       <c r="D27" t="inlineStr">
@@ -13037,14 +13101,14 @@
           <t>본체만(케이블없음) / 선택안함</t>
         </is>
       </c>
-      <c r="F27" s="27" t="n">
+      <c r="F27" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="G27" s="27">
+      <c r="G27" s="22">
         <f>C27+F27</f>
         <v/>
       </c>
-      <c r="H27" s="27">
+      <c r="H27" s="22">
         <f>G27/110%</f>
         <v/>
       </c>
@@ -13055,11 +13119,11 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>DS4608 SR</t>
-        </is>
-      </c>
-      <c r="C28" s="27">
-        <f>'지브라-스캐너'!F6</f>
+          <t>DS4608 XD</t>
+        </is>
+      </c>
+      <c r="C28" s="22">
+        <f>'지브라-스캐너'!F15</f>
         <v/>
       </c>
       <c r="D28" t="inlineStr">
@@ -13072,14 +13136,14 @@
           <t>본체만(케이블없음) / 스탠드거치대</t>
         </is>
       </c>
-      <c r="F28" s="27" t="n">
+      <c r="F28" s="22" t="n">
         <v>55000</v>
       </c>
-      <c r="G28" s="27">
+      <c r="G28" s="22">
         <f>C28+F28</f>
         <v/>
       </c>
-      <c r="H28" s="27">
+      <c r="H28" s="22">
         <f>G28/110%</f>
         <v/>
       </c>
@@ -13090,11 +13154,11 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>LI2208</t>
-        </is>
-      </c>
-      <c r="C29" s="27">
-        <f>'지브라-스캐너'!F7</f>
+          <t>DS8288</t>
+        </is>
+      </c>
+      <c r="C29" s="22">
+        <f>'지브라-스캐너'!F16</f>
         <v/>
       </c>
       <c r="D29" t="inlineStr">
@@ -13104,17 +13168,17 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>정품직선형USB</t>
-        </is>
-      </c>
-      <c r="F29" s="27" t="n">
-        <v>16500</v>
-      </c>
-      <c r="G29" s="27">
+          <t>RS232C</t>
+        </is>
+      </c>
+      <c r="F29" s="22" t="n">
+        <v>24200</v>
+      </c>
+      <c r="G29" s="22">
         <f>C29+F29</f>
         <v/>
       </c>
-      <c r="H29" s="27">
+      <c r="H29" s="22">
         <f>G29/110%</f>
         <v/>
       </c>
@@ -13125,11 +13189,11 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>LI2208</t>
-        </is>
-      </c>
-      <c r="C30" s="27">
-        <f>'지브라-스캐너'!F7</f>
+          <t>DS8208</t>
+        </is>
+      </c>
+      <c r="C30" s="22">
+        <f>'지브라-스캐너'!F17</f>
         <v/>
       </c>
       <c r="D30" t="inlineStr">
@@ -13142,14 +13206,14 @@
           <t>RS232C</t>
         </is>
       </c>
-      <c r="F30" s="27" t="n">
+      <c r="F30" s="22" t="n">
         <v>24200</v>
       </c>
-      <c r="G30" s="27">
+      <c r="G30" s="22">
         <f>C30+F30</f>
         <v/>
       </c>
-      <c r="H30" s="27">
+      <c r="H30" s="22">
         <f>G30/110%</f>
         <v/>
       </c>
@@ -13160,11 +13224,11 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>LI3608 SR</t>
-        </is>
-      </c>
-      <c r="C31" s="27">
-        <f>'지브라-스캐너'!F8</f>
+          <t>DS3678 XR</t>
+        </is>
+      </c>
+      <c r="C31" s="22">
+        <f>'지브라-스캐너'!F20</f>
         <v/>
       </c>
       <c r="D31" t="inlineStr">
@@ -13174,17 +13238,17 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>USB</t>
-        </is>
-      </c>
-      <c r="F31" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="G31" s="27">
+          <t>RS232C</t>
+        </is>
+      </c>
+      <c r="F31" s="22" t="n">
+        <v>24200</v>
+      </c>
+      <c r="G31" s="22">
         <f>C31+F31</f>
         <v/>
       </c>
-      <c r="H31" s="27">
+      <c r="H31" s="22">
         <f>G31/110%</f>
         <v/>
       </c>
@@ -13195,11 +13259,11 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>DS3608 SR</t>
-        </is>
-      </c>
-      <c r="C32" s="27">
-        <f>'지브라-스캐너'!F9</f>
+          <t>DS5502</t>
+        </is>
+      </c>
+      <c r="C32" s="22">
+        <f>'지브라-스캐너'!F21</f>
         <v/>
       </c>
       <c r="D32" t="inlineStr">
@@ -13209,17 +13273,17 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>USB</t>
-        </is>
-      </c>
-      <c r="F32" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="G32" s="27">
+          <t>RS232C</t>
+        </is>
+      </c>
+      <c r="F32" s="22" t="n">
+        <v>49500</v>
+      </c>
+      <c r="G32" s="22">
         <f>C32+F32</f>
         <v/>
       </c>
-      <c r="H32" s="27">
+      <c r="H32" s="22">
         <f>G32/110%</f>
         <v/>
       </c>
@@ -13230,11 +13294,11 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>DS3608 SR</t>
-        </is>
-      </c>
-      <c r="C33" s="27">
-        <f>'지브라-스캐너'!F9</f>
+          <t>DS4678</t>
+        </is>
+      </c>
+      <c r="C33" s="22">
+        <f>'지브라-스캐너'!F22</f>
         <v/>
       </c>
       <c r="D33" t="inlineStr">
@@ -13244,17 +13308,17 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>RS232C</t>
-        </is>
-      </c>
-      <c r="F33" s="27" t="n">
-        <v>24200</v>
-      </c>
-      <c r="G33" s="27">
+          <t>본체+크래들만(케이블없음)</t>
+        </is>
+      </c>
+      <c r="F33" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G33" s="22">
         <f>C33+F33</f>
         <v/>
       </c>
-      <c r="H33" s="27">
+      <c r="H33" s="22">
         <f>G33/110%</f>
         <v/>
       </c>
@@ -13265,11 +13329,11 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>LI3678</t>
-        </is>
-      </c>
-      <c r="C34" s="27">
-        <f>'지브라-스캐너'!F10</f>
+          <t>DS4678</t>
+        </is>
+      </c>
+      <c r="C34" s="22">
+        <f>'지브라-스캐너'!F22</f>
         <v/>
       </c>
       <c r="D34" t="inlineStr">
@@ -13279,17 +13343,17 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>USB</t>
-        </is>
-      </c>
-      <c r="F34" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="G34" s="27">
+          <t>RS232C</t>
+        </is>
+      </c>
+      <c r="F34" s="22" t="n">
+        <v>24200</v>
+      </c>
+      <c r="G34" s="22">
         <f>C34+F34</f>
         <v/>
       </c>
-      <c r="H34" s="27">
+      <c r="H34" s="22">
         <f>G34/110%</f>
         <v/>
       </c>
@@ -13300,11 +13364,11 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>LI3678</t>
-        </is>
-      </c>
-      <c r="C35" s="27">
-        <f>'지브라-스캐너'!F10</f>
+          <t>DS9308</t>
+        </is>
+      </c>
+      <c r="C35" s="22">
+        <f>'지브라-스캐너'!F24</f>
         <v/>
       </c>
       <c r="D35" t="inlineStr">
@@ -13317,14 +13381,14 @@
           <t>RS232C</t>
         </is>
       </c>
-      <c r="F35" s="27" t="n">
-        <v>33000</v>
-      </c>
-      <c r="G35" s="27">
+      <c r="F35" s="22" t="n">
+        <v>24200</v>
+      </c>
+      <c r="G35" s="22">
         <f>C35+F35</f>
         <v/>
       </c>
-      <c r="H35" s="27">
+      <c r="H35" s="22">
         <f>G35/110%</f>
         <v/>
       </c>
@@ -13335,11 +13399,11 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>DS9908</t>
-        </is>
-      </c>
-      <c r="C36" s="27">
-        <f>'지브라-스캐너'!F11</f>
+          <t>DS9308</t>
+        </is>
+      </c>
+      <c r="C36" s="22">
+        <f>'지브라-스캐너'!F24</f>
         <v/>
       </c>
       <c r="D36" t="inlineStr">
@@ -13349,17 +13413,17 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>코일형USB</t>
-        </is>
-      </c>
-      <c r="F36" s="27" t="n">
-        <v>18000</v>
-      </c>
-      <c r="G36" s="27">
+          <t>본체만(케이블없음)</t>
+        </is>
+      </c>
+      <c r="F36" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G36" s="22">
         <f>C36+F36</f>
         <v/>
       </c>
-      <c r="H36" s="27">
+      <c r="H36" s="22">
         <f>G36/110%</f>
         <v/>
       </c>
@@ -13370,11 +13434,11 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>DS9908</t>
-        </is>
-      </c>
-      <c r="C37" s="27">
-        <f>'지브라-스캐너'!F11</f>
+          <t>DS8178</t>
+        </is>
+      </c>
+      <c r="C37" s="22">
+        <f>'지브라-스캐너'!F25</f>
         <v/>
       </c>
       <c r="D37" t="inlineStr">
@@ -13384,17 +13448,17 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>직선형USB케이블</t>
-        </is>
-      </c>
-      <c r="F37" s="27" t="n">
-        <v>18000</v>
-      </c>
-      <c r="G37" s="27">
+          <t>RS232C</t>
+        </is>
+      </c>
+      <c r="F37" s="22" t="n">
+        <v>24200</v>
+      </c>
+      <c r="G37" s="22">
         <f>C37+F37</f>
         <v/>
       </c>
-      <c r="H37" s="27">
+      <c r="H37" s="22">
         <f>G37/110%</f>
         <v/>
       </c>
@@ -13405,11 +13469,11 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>DS9908</t>
-        </is>
-      </c>
-      <c r="C38" s="27">
-        <f>'지브라-스캐너'!F11</f>
+          <t>DS8178</t>
+        </is>
+      </c>
+      <c r="C38" s="22">
+        <f>'지브라-스캐너'!F25</f>
         <v/>
       </c>
       <c r="D38" t="inlineStr">
@@ -13419,17 +13483,17 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>RS232C</t>
-        </is>
-      </c>
-      <c r="F38" s="27" t="n">
-        <v>24200</v>
-      </c>
-      <c r="G38" s="27">
+          <t>본체+크래들만(케이블없음)</t>
+        </is>
+      </c>
+      <c r="F38" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G38" s="22">
         <f>C38+F38</f>
         <v/>
       </c>
-      <c r="H38" s="27">
+      <c r="H38" s="22">
         <f>G38/110%</f>
         <v/>
       </c>
@@ -13440,31 +13504,31 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>CS6080</t>
-        </is>
-      </c>
-      <c r="C39" s="27">
-        <f>'지브라-스캐너'!F13</f>
+          <t>LI4278</t>
+        </is>
+      </c>
+      <c r="C39" s="22">
+        <f>'지브라-스캐너'!F26</f>
         <v/>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>스캔엔진</t>
+          <t>인터페이스</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>2D</t>
-        </is>
-      </c>
-      <c r="F39" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="G39" s="27">
+          <t>RS232C</t>
+        </is>
+      </c>
+      <c r="F39" s="22" t="n">
+        <v>24200</v>
+      </c>
+      <c r="G39" s="22">
         <f>C39+F39</f>
         <v/>
       </c>
-      <c r="H39" s="27">
+      <c r="H39" s="22">
         <f>G39/110%</f>
         <v/>
       </c>
@@ -13475,11 +13539,11 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>DS3678 SR</t>
-        </is>
-      </c>
-      <c r="C40" s="27">
-        <f>'지브라-스캐너'!F14</f>
+          <t>LI4278</t>
+        </is>
+      </c>
+      <c r="C40" s="22">
+        <f>'지브라-스캐너'!F26</f>
         <v/>
       </c>
       <c r="D40" t="inlineStr">
@@ -13489,17 +13553,17 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>SR버전+USB케이블</t>
-        </is>
-      </c>
-      <c r="F40" s="27" t="n">
+          <t>본체+크래들만(케이블없음)</t>
+        </is>
+      </c>
+      <c r="F40" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="G40" s="27">
+      <c r="G40" s="22">
         <f>C40+F40</f>
         <v/>
       </c>
-      <c r="H40" s="27">
+      <c r="H40" s="22">
         <f>G40/110%</f>
         <v/>
       </c>
@@ -13510,31 +13574,31 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>DS3678 SR</t>
-        </is>
-      </c>
-      <c r="C41" s="27">
-        <f>'지브라-스캐너'!F14</f>
+          <t>RS6100</t>
+        </is>
+      </c>
+      <c r="C41" s="22">
+        <f>'지브라-스캐너'!F27</f>
         <v/>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>인터페이스</t>
+          <t>연결방식</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>HD버전+USB케이블</t>
-        </is>
-      </c>
-      <c r="F41" s="27" t="n">
-        <v>220000</v>
-      </c>
-      <c r="G41" s="27">
+          <t>링트리거</t>
+        </is>
+      </c>
+      <c r="F41" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G41" s="22">
         <f>C41+F41</f>
         <v/>
       </c>
-      <c r="H41" s="27">
+      <c r="H41" s="22">
         <f>G41/110%</f>
         <v/>
       </c>
@@ -13545,31 +13609,31 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>DS3678 SR</t>
-        </is>
-      </c>
-      <c r="C42" s="27">
-        <f>'지브라-스캐너'!F14</f>
+          <t>FS10</t>
+        </is>
+      </c>
+      <c r="C42" s="22">
+        <f>'지브라-스캐너'!F28</f>
         <v/>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>인터페이스</t>
+          <t>본체</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>SR버전+RS232C케이블</t>
-        </is>
-      </c>
-      <c r="F42" s="27" t="n">
-        <v>33000</v>
-      </c>
-      <c r="G42" s="27">
+          <t>본체</t>
+        </is>
+      </c>
+      <c r="F42" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G42" s="22">
         <f>C42+F42</f>
         <v/>
       </c>
-      <c r="H42" s="27">
+      <c r="H42" s="22">
         <f>G42/110%</f>
         <v/>
       </c>
@@ -13580,31 +13644,31 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>DS3678 SR</t>
-        </is>
-      </c>
-      <c r="C43" s="27">
-        <f>'지브라-스캐너'!F14</f>
+          <t>FS20</t>
+        </is>
+      </c>
+      <c r="C43" s="22">
+        <f>'지브라-스캐너'!F29</f>
         <v/>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>인터페이스</t>
+          <t>본체</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>HD버전+RS232C케이블</t>
-        </is>
-      </c>
-      <c r="F43" s="27" t="n">
-        <v>275000</v>
-      </c>
-      <c r="G43" s="27">
+          <t>본체</t>
+        </is>
+      </c>
+      <c r="F43" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G43" s="22">
         <f>C43+F43</f>
         <v/>
       </c>
-      <c r="H43" s="27">
+      <c r="H43" s="22">
         <f>G43/110%</f>
         <v/>
       </c>
@@ -13615,31 +13679,31 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>DS4608 XD</t>
-        </is>
-      </c>
-      <c r="C44" s="27">
-        <f>'지브라-스캐너'!F15</f>
+          <t>FS40</t>
+        </is>
+      </c>
+      <c r="C44" s="22">
+        <f>'지브라-스캐너'!F30</f>
         <v/>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>인터페이스 / 악세사리</t>
+          <t>본체</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>정품직선형USB / 선택안함</t>
-        </is>
-      </c>
-      <c r="F44" s="27" t="n">
-        <v>18000</v>
-      </c>
-      <c r="G44" s="27">
+          <t>본체</t>
+        </is>
+      </c>
+      <c r="F44" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G44" s="22">
         <f>C44+F44</f>
         <v/>
       </c>
-      <c r="H44" s="27">
+      <c r="H44" s="22">
         <f>G44/110%</f>
         <v/>
       </c>
@@ -13650,1362 +13714,32 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>DS4608 XD</t>
-        </is>
-      </c>
-      <c r="C45" s="27">
-        <f>'지브라-스캐너'!F15</f>
+          <t>FS70</t>
+        </is>
+      </c>
+      <c r="C45" s="22">
+        <f>'지브라-스캐너'!F31</f>
         <v/>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>인터페이스 / 악세사리</t>
+          <t>본체</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>정품직선형USB / 스탠드거치대</t>
-        </is>
-      </c>
-      <c r="F45" s="27" t="n">
-        <v>73000</v>
-      </c>
-      <c r="G45" s="27">
+          <t>본체</t>
+        </is>
+      </c>
+      <c r="F45" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G45" s="22">
         <f>C45+F45</f>
         <v/>
       </c>
-      <c r="H45" s="27">
+      <c r="H45" s="22">
         <f>G45/110%</f>
-        <v/>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="n">
-        <v>45</v>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>DS4608 XD</t>
-        </is>
-      </c>
-      <c r="C46" s="27">
-        <f>'지브라-스캐너'!F15</f>
-        <v/>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>인터페이스 / 악세사리</t>
-        </is>
-      </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>RS232C / 선택안함</t>
-        </is>
-      </c>
-      <c r="F46" s="27" t="n">
-        <v>24200</v>
-      </c>
-      <c r="G46" s="27">
-        <f>C46+F46</f>
-        <v/>
-      </c>
-      <c r="H46" s="27">
-        <f>G46/110%</f>
-        <v/>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="n">
-        <v>46</v>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>DS4608 XD</t>
-        </is>
-      </c>
-      <c r="C47" s="27">
-        <f>'지브라-스캐너'!F15</f>
-        <v/>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>인터페이스 / 악세사리</t>
-        </is>
-      </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>RS232C / 스탠드거치대</t>
-        </is>
-      </c>
-      <c r="F47" s="27" t="n">
-        <v>79200</v>
-      </c>
-      <c r="G47" s="27">
-        <f>C47+F47</f>
-        <v/>
-      </c>
-      <c r="H47" s="27">
-        <f>G47/110%</f>
-        <v/>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="n">
-        <v>47</v>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>DS4608 XD</t>
-        </is>
-      </c>
-      <c r="C48" s="27">
-        <f>'지브라-스캐너'!F15</f>
-        <v/>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>인터페이스 / 악세사리</t>
-        </is>
-      </c>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>코일형USB / 선택안함</t>
-        </is>
-      </c>
-      <c r="F48" s="27" t="n">
-        <v>18000</v>
-      </c>
-      <c r="G48" s="27">
-        <f>C48+F48</f>
-        <v/>
-      </c>
-      <c r="H48" s="27">
-        <f>G48/110%</f>
-        <v/>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="n">
-        <v>48</v>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>DS4608 XD</t>
-        </is>
-      </c>
-      <c r="C49" s="27">
-        <f>'지브라-스캐너'!F15</f>
-        <v/>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>인터페이스 / 악세사리</t>
-        </is>
-      </c>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>코일형USB / 스탠드거치대</t>
-        </is>
-      </c>
-      <c r="F49" s="27" t="n">
-        <v>73000</v>
-      </c>
-      <c r="G49" s="27">
-        <f>C49+F49</f>
-        <v/>
-      </c>
-      <c r="H49" s="27">
-        <f>G49/110%</f>
-        <v/>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="n">
-        <v>49</v>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>DS4608 XD</t>
-        </is>
-      </c>
-      <c r="C50" s="27">
-        <f>'지브라-스캐너'!F15</f>
-        <v/>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>인터페이스 / 악세사리</t>
-        </is>
-      </c>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>본체만(케이블없음) / 선택안함</t>
-        </is>
-      </c>
-      <c r="F50" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="G50" s="27">
-        <f>C50+F50</f>
-        <v/>
-      </c>
-      <c r="H50" s="27">
-        <f>G50/110%</f>
-        <v/>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="n">
-        <v>50</v>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>DS4608 XD</t>
-        </is>
-      </c>
-      <c r="C51" s="27">
-        <f>'지브라-스캐너'!F15</f>
-        <v/>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>인터페이스 / 악세사리</t>
-        </is>
-      </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>본체만(케이블없음) / 스탠드거치대</t>
-        </is>
-      </c>
-      <c r="F51" s="27" t="n">
-        <v>55000</v>
-      </c>
-      <c r="G51" s="27">
-        <f>C51+F51</f>
-        <v/>
-      </c>
-      <c r="H51" s="27">
-        <f>G51/110%</f>
-        <v/>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="n">
-        <v>51</v>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>DS8288</t>
-        </is>
-      </c>
-      <c r="C52" s="27">
-        <f>'지브라-스캐너'!F16</f>
-        <v/>
-      </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>인터페이스</t>
-        </is>
-      </c>
-      <c r="E52" t="inlineStr">
-        <is>
-          <t>RS232C</t>
-        </is>
-      </c>
-      <c r="F52" s="27" t="n">
-        <v>24200</v>
-      </c>
-      <c r="G52" s="27">
-        <f>C52+F52</f>
-        <v/>
-      </c>
-      <c r="H52" s="27">
-        <f>G52/110%</f>
-        <v/>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="n">
-        <v>52</v>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>DS8288</t>
-        </is>
-      </c>
-      <c r="C53" s="27">
-        <f>'지브라-스캐너'!F16</f>
-        <v/>
-      </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>인터페이스</t>
-        </is>
-      </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>USB</t>
-        </is>
-      </c>
-      <c r="F53" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="G53" s="27">
-        <f>C53+F53</f>
-        <v/>
-      </c>
-      <c r="H53" s="27">
-        <f>G53/110%</f>
-        <v/>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="n">
-        <v>53</v>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>DS8208</t>
-        </is>
-      </c>
-      <c r="C54" s="27">
-        <f>'지브라-스캐너'!F17</f>
-        <v/>
-      </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>인터페이스</t>
-        </is>
-      </c>
-      <c r="E54" t="inlineStr">
-        <is>
-          <t>RS232C</t>
-        </is>
-      </c>
-      <c r="F54" s="27" t="n">
-        <v>24200</v>
-      </c>
-      <c r="G54" s="27">
-        <f>C54+F54</f>
-        <v/>
-      </c>
-      <c r="H54" s="27">
-        <f>G54/110%</f>
-        <v/>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="n">
-        <v>54</v>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>DS8208</t>
-        </is>
-      </c>
-      <c r="C55" s="27">
-        <f>'지브라-스캐너'!F17</f>
-        <v/>
-      </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>인터페이스</t>
-        </is>
-      </c>
-      <c r="E55" t="inlineStr">
-        <is>
-          <t>USB</t>
-        </is>
-      </c>
-      <c r="F55" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="G55" s="27">
-        <f>C55+F55</f>
-        <v/>
-      </c>
-      <c r="H55" s="27">
-        <f>G55/110%</f>
-        <v/>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="n">
-        <v>55</v>
-      </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>DS3608 ER</t>
-        </is>
-      </c>
-      <c r="C56" s="27">
-        <f>'지브라-스캐너'!F18</f>
-        <v/>
-      </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>인터페이스</t>
-        </is>
-      </c>
-      <c r="E56" t="inlineStr">
-        <is>
-          <t>USB</t>
-        </is>
-      </c>
-      <c r="F56" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="G56" s="27">
-        <f>C56+F56</f>
-        <v/>
-      </c>
-      <c r="H56" s="27">
-        <f>G56/110%</f>
-        <v/>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="n">
-        <v>56</v>
-      </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>LI3608 ER</t>
-        </is>
-      </c>
-      <c r="C57" s="27">
-        <f>'지브라-스캐너'!F19</f>
-        <v/>
-      </c>
-      <c r="D57" t="inlineStr">
-        <is>
-          <t>인터페이스</t>
-        </is>
-      </c>
-      <c r="E57" t="inlineStr">
-        <is>
-          <t>USB</t>
-        </is>
-      </c>
-      <c r="F57" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="G57" s="27">
-        <f>C57+F57</f>
-        <v/>
-      </c>
-      <c r="H57" s="27">
-        <f>G57/110%</f>
-        <v/>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="n">
-        <v>57</v>
-      </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>DS3678 XR</t>
-        </is>
-      </c>
-      <c r="C58" s="27">
-        <f>'지브라-스캐너'!F20</f>
-        <v/>
-      </c>
-      <c r="D58" t="inlineStr">
-        <is>
-          <t>인터페이스</t>
-        </is>
-      </c>
-      <c r="E58" t="inlineStr">
-        <is>
-          <t>USB</t>
-        </is>
-      </c>
-      <c r="F58" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="G58" s="27">
-        <f>C58+F58</f>
-        <v/>
-      </c>
-      <c r="H58" s="27">
-        <f>G58/110%</f>
-        <v/>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="n">
-        <v>58</v>
-      </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>DS3678 XR</t>
-        </is>
-      </c>
-      <c r="C59" s="27">
-        <f>'지브라-스캐너'!F20</f>
-        <v/>
-      </c>
-      <c r="D59" t="inlineStr">
-        <is>
-          <t>인터페이스</t>
-        </is>
-      </c>
-      <c r="E59" t="inlineStr">
-        <is>
-          <t>RS232C</t>
-        </is>
-      </c>
-      <c r="F59" s="27" t="n">
-        <v>24200</v>
-      </c>
-      <c r="G59" s="27">
-        <f>C59+F59</f>
-        <v/>
-      </c>
-      <c r="H59" s="27">
-        <f>G59/110%</f>
-        <v/>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="n">
-        <v>59</v>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>DS5502</t>
-        </is>
-      </c>
-      <c r="C60" s="27">
-        <f>'지브라-스캐너'!F21</f>
-        <v/>
-      </c>
-      <c r="D60" t="inlineStr">
-        <is>
-          <t>인터페이스</t>
-        </is>
-      </c>
-      <c r="E60" t="inlineStr">
-        <is>
-          <t>RS232C</t>
-        </is>
-      </c>
-      <c r="F60" s="27" t="n">
-        <v>49500</v>
-      </c>
-      <c r="G60" s="27">
-        <f>C60+F60</f>
-        <v/>
-      </c>
-      <c r="H60" s="27">
-        <f>G60/110%</f>
-        <v/>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="n">
-        <v>60</v>
-      </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>DS5502</t>
-        </is>
-      </c>
-      <c r="C61" s="27">
-        <f>'지브라-스캐너'!F21</f>
-        <v/>
-      </c>
-      <c r="D61" t="inlineStr">
-        <is>
-          <t>인터페이스</t>
-        </is>
-      </c>
-      <c r="E61" t="inlineStr">
-        <is>
-          <t>USB</t>
-        </is>
-      </c>
-      <c r="F61" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="G61" s="27">
-        <f>C61+F61</f>
-        <v/>
-      </c>
-      <c r="H61" s="27">
-        <f>G61/110%</f>
-        <v/>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="n">
-        <v>61</v>
-      </c>
-      <c r="B62" t="inlineStr">
-        <is>
-          <t>DS4678</t>
-        </is>
-      </c>
-      <c r="C62" s="27">
-        <f>'지브라-스캐너'!F22</f>
-        <v/>
-      </c>
-      <c r="D62" t="inlineStr">
-        <is>
-          <t>인터페이스</t>
-        </is>
-      </c>
-      <c r="E62" t="inlineStr">
-        <is>
-          <t>본체+크래들만(케이블없음)</t>
-        </is>
-      </c>
-      <c r="F62" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="G62" s="27">
-        <f>C62+F62</f>
-        <v/>
-      </c>
-      <c r="H62" s="27">
-        <f>G62/110%</f>
-        <v/>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="n">
-        <v>62</v>
-      </c>
-      <c r="B63" t="inlineStr">
-        <is>
-          <t>DS4678</t>
-        </is>
-      </c>
-      <c r="C63" s="27">
-        <f>'지브라-스캐너'!F22</f>
-        <v/>
-      </c>
-      <c r="D63" t="inlineStr">
-        <is>
-          <t>인터페이스</t>
-        </is>
-      </c>
-      <c r="E63" t="inlineStr">
-        <is>
-          <t>정품직선형USB</t>
-        </is>
-      </c>
-      <c r="F63" s="27" t="n">
-        <v>18000</v>
-      </c>
-      <c r="G63" s="27">
-        <f>C63+F63</f>
-        <v/>
-      </c>
-      <c r="H63" s="27">
-        <f>G63/110%</f>
-        <v/>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" t="n">
-        <v>63</v>
-      </c>
-      <c r="B64" t="inlineStr">
-        <is>
-          <t>DS4678</t>
-        </is>
-      </c>
-      <c r="C64" s="27">
-        <f>'지브라-스캐너'!F22</f>
-        <v/>
-      </c>
-      <c r="D64" t="inlineStr">
-        <is>
-          <t>인터페이스</t>
-        </is>
-      </c>
-      <c r="E64" t="inlineStr">
-        <is>
-          <t>코일형USB</t>
-        </is>
-      </c>
-      <c r="F64" s="27" t="n">
-        <v>18000</v>
-      </c>
-      <c r="G64" s="27">
-        <f>C64+F64</f>
-        <v/>
-      </c>
-      <c r="H64" s="27">
-        <f>G64/110%</f>
-        <v/>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" t="n">
-        <v>64</v>
-      </c>
-      <c r="B65" t="inlineStr">
-        <is>
-          <t>DS4678</t>
-        </is>
-      </c>
-      <c r="C65" s="27">
-        <f>'지브라-스캐너'!F22</f>
-        <v/>
-      </c>
-      <c r="D65" t="inlineStr">
-        <is>
-          <t>인터페이스</t>
-        </is>
-      </c>
-      <c r="E65" t="inlineStr">
-        <is>
-          <t>RS232C</t>
-        </is>
-      </c>
-      <c r="F65" s="27" t="n">
-        <v>24200</v>
-      </c>
-      <c r="G65" s="27">
-        <f>C65+F65</f>
-        <v/>
-      </c>
-      <c r="H65" s="27">
-        <f>G65/110%</f>
-        <v/>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" t="n">
-        <v>65</v>
-      </c>
-      <c r="B66" t="inlineStr">
-        <is>
-          <t>SP72</t>
-        </is>
-      </c>
-      <c r="C66" s="27">
-        <f>'지브라-스캐너'!F23</f>
-        <v/>
-      </c>
-      <c r="D66" t="inlineStr">
-        <is>
-          <t>인터페이스</t>
-        </is>
-      </c>
-      <c r="E66" t="inlineStr">
-        <is>
-          <t>USB</t>
-        </is>
-      </c>
-      <c r="F66" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="G66" s="27">
-        <f>C66+F66</f>
-        <v/>
-      </c>
-      <c r="H66" s="27">
-        <f>G66/110%</f>
-        <v/>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" t="n">
-        <v>66</v>
-      </c>
-      <c r="B67" t="inlineStr">
-        <is>
-          <t>DS9308</t>
-        </is>
-      </c>
-      <c r="C67" s="27">
-        <f>'지브라-스캐너'!F24</f>
-        <v/>
-      </c>
-      <c r="D67" t="inlineStr">
-        <is>
-          <t>인터페이스</t>
-        </is>
-      </c>
-      <c r="E67" t="inlineStr">
-        <is>
-          <t>직선형USB케이블</t>
-        </is>
-      </c>
-      <c r="F67" s="27" t="n">
-        <v>18000</v>
-      </c>
-      <c r="G67" s="27">
-        <f>C67+F67</f>
-        <v/>
-      </c>
-      <c r="H67" s="27">
-        <f>G67/110%</f>
-        <v/>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" t="n">
-        <v>67</v>
-      </c>
-      <c r="B68" t="inlineStr">
-        <is>
-          <t>DS9308</t>
-        </is>
-      </c>
-      <c r="C68" s="27">
-        <f>'지브라-스캐너'!F24</f>
-        <v/>
-      </c>
-      <c r="D68" t="inlineStr">
-        <is>
-          <t>인터페이스</t>
-        </is>
-      </c>
-      <c r="E68" t="inlineStr">
-        <is>
-          <t>RS232C</t>
-        </is>
-      </c>
-      <c r="F68" s="27" t="n">
-        <v>24200</v>
-      </c>
-      <c r="G68" s="27">
-        <f>C68+F68</f>
-        <v/>
-      </c>
-      <c r="H68" s="27">
-        <f>G68/110%</f>
-        <v/>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" t="n">
-        <v>68</v>
-      </c>
-      <c r="B69" t="inlineStr">
-        <is>
-          <t>DS9308</t>
-        </is>
-      </c>
-      <c r="C69" s="27">
-        <f>'지브라-스캐너'!F24</f>
-        <v/>
-      </c>
-      <c r="D69" t="inlineStr">
-        <is>
-          <t>인터페이스</t>
-        </is>
-      </c>
-      <c r="E69" t="inlineStr">
-        <is>
-          <t>코일형USB</t>
-        </is>
-      </c>
-      <c r="F69" s="27" t="n">
-        <v>18000</v>
-      </c>
-      <c r="G69" s="27">
-        <f>C69+F69</f>
-        <v/>
-      </c>
-      <c r="H69" s="27">
-        <f>G69/110%</f>
-        <v/>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" t="n">
-        <v>69</v>
-      </c>
-      <c r="B70" t="inlineStr">
-        <is>
-          <t>DS9308</t>
-        </is>
-      </c>
-      <c r="C70" s="27">
-        <f>'지브라-스캐너'!F24</f>
-        <v/>
-      </c>
-      <c r="D70" t="inlineStr">
-        <is>
-          <t>인터페이스</t>
-        </is>
-      </c>
-      <c r="E70" t="inlineStr">
-        <is>
-          <t>본체만(케이블없음)</t>
-        </is>
-      </c>
-      <c r="F70" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="G70" s="27">
-        <f>C70+F70</f>
-        <v/>
-      </c>
-      <c r="H70" s="27">
-        <f>G70/110%</f>
-        <v/>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" t="n">
-        <v>70</v>
-      </c>
-      <c r="B71" t="inlineStr">
-        <is>
-          <t>DS8178</t>
-        </is>
-      </c>
-      <c r="C71" s="27">
-        <f>'지브라-스캐너'!F25</f>
-        <v/>
-      </c>
-      <c r="D71" t="inlineStr">
-        <is>
-          <t>인터페이스</t>
-        </is>
-      </c>
-      <c r="E71" t="inlineStr">
-        <is>
-          <t>정품직선형USB</t>
-        </is>
-      </c>
-      <c r="F71" s="27" t="n">
-        <v>18000</v>
-      </c>
-      <c r="G71" s="27">
-        <f>C71+F71</f>
-        <v/>
-      </c>
-      <c r="H71" s="27">
-        <f>G71/110%</f>
-        <v/>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" t="n">
-        <v>71</v>
-      </c>
-      <c r="B72" t="inlineStr">
-        <is>
-          <t>DS8178</t>
-        </is>
-      </c>
-      <c r="C72" s="27">
-        <f>'지브라-스캐너'!F25</f>
-        <v/>
-      </c>
-      <c r="D72" t="inlineStr">
-        <is>
-          <t>인터페이스</t>
-        </is>
-      </c>
-      <c r="E72" t="inlineStr">
-        <is>
-          <t>RS232C</t>
-        </is>
-      </c>
-      <c r="F72" s="27" t="n">
-        <v>24200</v>
-      </c>
-      <c r="G72" s="27">
-        <f>C72+F72</f>
-        <v/>
-      </c>
-      <c r="H72" s="27">
-        <f>G72/110%</f>
-        <v/>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" t="n">
-        <v>72</v>
-      </c>
-      <c r="B73" t="inlineStr">
-        <is>
-          <t>DS8178</t>
-        </is>
-      </c>
-      <c r="C73" s="27">
-        <f>'지브라-스캐너'!F25</f>
-        <v/>
-      </c>
-      <c r="D73" t="inlineStr">
-        <is>
-          <t>인터페이스</t>
-        </is>
-      </c>
-      <c r="E73" t="inlineStr">
-        <is>
-          <t>코일형USB</t>
-        </is>
-      </c>
-      <c r="F73" s="27" t="n">
-        <v>18000</v>
-      </c>
-      <c r="G73" s="27">
-        <f>C73+F73</f>
-        <v/>
-      </c>
-      <c r="H73" s="27">
-        <f>G73/110%</f>
-        <v/>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" t="n">
-        <v>73</v>
-      </c>
-      <c r="B74" t="inlineStr">
-        <is>
-          <t>DS8178</t>
-        </is>
-      </c>
-      <c r="C74" s="27">
-        <f>'지브라-스캐너'!F25</f>
-        <v/>
-      </c>
-      <c r="D74" t="inlineStr">
-        <is>
-          <t>인터페이스</t>
-        </is>
-      </c>
-      <c r="E74" t="inlineStr">
-        <is>
-          <t>본체+크래들만(케이블없음)</t>
-        </is>
-      </c>
-      <c r="F74" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="G74" s="27">
-        <f>C74+F74</f>
-        <v/>
-      </c>
-      <c r="H74" s="27">
-        <f>G74/110%</f>
-        <v/>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" t="n">
-        <v>74</v>
-      </c>
-      <c r="B75" t="inlineStr">
-        <is>
-          <t>LI4278</t>
-        </is>
-      </c>
-      <c r="C75" s="27">
-        <f>'지브라-스캐너'!F26</f>
-        <v/>
-      </c>
-      <c r="D75" t="inlineStr">
-        <is>
-          <t>인터페이스</t>
-        </is>
-      </c>
-      <c r="E75" t="inlineStr">
-        <is>
-          <t>정품직선형USB</t>
-        </is>
-      </c>
-      <c r="F75" s="27" t="n">
-        <v>18000</v>
-      </c>
-      <c r="G75" s="27">
-        <f>C75+F75</f>
-        <v/>
-      </c>
-      <c r="H75" s="27">
-        <f>G75/110%</f>
-        <v/>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" t="n">
-        <v>75</v>
-      </c>
-      <c r="B76" t="inlineStr">
-        <is>
-          <t>LI4278</t>
-        </is>
-      </c>
-      <c r="C76" s="27">
-        <f>'지브라-스캐너'!F26</f>
-        <v/>
-      </c>
-      <c r="D76" t="inlineStr">
-        <is>
-          <t>인터페이스</t>
-        </is>
-      </c>
-      <c r="E76" t="inlineStr">
-        <is>
-          <t>RS232C</t>
-        </is>
-      </c>
-      <c r="F76" s="27" t="n">
-        <v>24200</v>
-      </c>
-      <c r="G76" s="27">
-        <f>C76+F76</f>
-        <v/>
-      </c>
-      <c r="H76" s="27">
-        <f>G76/110%</f>
-        <v/>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" t="n">
-        <v>76</v>
-      </c>
-      <c r="B77" t="inlineStr">
-        <is>
-          <t>LI4278</t>
-        </is>
-      </c>
-      <c r="C77" s="27">
-        <f>'지브라-스캐너'!F26</f>
-        <v/>
-      </c>
-      <c r="D77" t="inlineStr">
-        <is>
-          <t>인터페이스</t>
-        </is>
-      </c>
-      <c r="E77" t="inlineStr">
-        <is>
-          <t>코일형USB</t>
-        </is>
-      </c>
-      <c r="F77" s="27" t="n">
-        <v>18000</v>
-      </c>
-      <c r="G77" s="27">
-        <f>C77+F77</f>
-        <v/>
-      </c>
-      <c r="H77" s="27">
-        <f>G77/110%</f>
-        <v/>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" t="n">
-        <v>77</v>
-      </c>
-      <c r="B78" t="inlineStr">
-        <is>
-          <t>LI4278</t>
-        </is>
-      </c>
-      <c r="C78" s="27">
-        <f>'지브라-스캐너'!F26</f>
-        <v/>
-      </c>
-      <c r="D78" t="inlineStr">
-        <is>
-          <t>인터페이스</t>
-        </is>
-      </c>
-      <c r="E78" t="inlineStr">
-        <is>
-          <t>본체+크래들만(케이블없음)</t>
-        </is>
-      </c>
-      <c r="F78" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="G78" s="27">
-        <f>C78+F78</f>
-        <v/>
-      </c>
-      <c r="H78" s="27">
-        <f>G78/110%</f>
-        <v/>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" t="n">
-        <v>78</v>
-      </c>
-      <c r="B79" t="inlineStr">
-        <is>
-          <t>RS6100</t>
-        </is>
-      </c>
-      <c r="C79" s="27">
-        <f>'지브라-스캐너'!F27</f>
-        <v/>
-      </c>
-      <c r="D79" t="inlineStr">
-        <is>
-          <t>연결방식</t>
-        </is>
-      </c>
-      <c r="E79" t="inlineStr">
-        <is>
-          <t>링트리거</t>
-        </is>
-      </c>
-      <c r="F79" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="G79" s="27">
-        <f>C79+F79</f>
-        <v/>
-      </c>
-      <c r="H79" s="27">
-        <f>G79/110%</f>
-        <v/>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" t="n">
-        <v>79</v>
-      </c>
-      <c r="B80" t="inlineStr">
-        <is>
-          <t>FS10</t>
-        </is>
-      </c>
-      <c r="C80" s="27">
-        <f>'지브라-스캐너'!F28</f>
-        <v/>
-      </c>
-      <c r="D80" t="inlineStr">
-        <is>
-          <t>본체</t>
-        </is>
-      </c>
-      <c r="E80" t="inlineStr">
-        <is>
-          <t>본체</t>
-        </is>
-      </c>
-      <c r="F80" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="G80" s="27">
-        <f>C80+F80</f>
-        <v/>
-      </c>
-      <c r="H80" s="27">
-        <f>G80/110%</f>
-        <v/>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" t="n">
-        <v>80</v>
-      </c>
-      <c r="B81" t="inlineStr">
-        <is>
-          <t>FS20</t>
-        </is>
-      </c>
-      <c r="C81" s="27">
-        <f>'지브라-스캐너'!F29</f>
-        <v/>
-      </c>
-      <c r="D81" t="inlineStr">
-        <is>
-          <t>본체</t>
-        </is>
-      </c>
-      <c r="E81" t="inlineStr">
-        <is>
-          <t>본체</t>
-        </is>
-      </c>
-      <c r="F81" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="G81" s="27">
-        <f>C81+F81</f>
-        <v/>
-      </c>
-      <c r="H81" s="27">
-        <f>G81/110%</f>
-        <v/>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" t="n">
-        <v>81</v>
-      </c>
-      <c r="B82" t="inlineStr">
-        <is>
-          <t>FS40</t>
-        </is>
-      </c>
-      <c r="C82" s="27">
-        <f>'지브라-스캐너'!F30</f>
-        <v/>
-      </c>
-      <c r="D82" t="inlineStr">
-        <is>
-          <t>본체</t>
-        </is>
-      </c>
-      <c r="E82" t="inlineStr">
-        <is>
-          <t>본체</t>
-        </is>
-      </c>
-      <c r="F82" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="G82" s="27">
-        <f>C82+F82</f>
-        <v/>
-      </c>
-      <c r="H82" s="27">
-        <f>G82/110%</f>
-        <v/>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" t="n">
-        <v>82</v>
-      </c>
-      <c r="B83" t="inlineStr">
-        <is>
-          <t>FS70</t>
-        </is>
-      </c>
-      <c r="C83" s="27">
-        <f>'지브라-스캐너'!F31</f>
-        <v/>
-      </c>
-      <c r="D83" t="inlineStr">
-        <is>
-          <t>본체</t>
-        </is>
-      </c>
-      <c r="E83" t="inlineStr">
-        <is>
-          <t>본체</t>
-        </is>
-      </c>
-      <c r="F83" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="G83" s="27">
-        <f>C83+F83</f>
-        <v/>
-      </c>
-      <c r="H83" s="27">
-        <f>G83/110%</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Mark DS457 HD as discontinued
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0164u4m2HzVL7yDN6jZnxUBp
</commit_message>
<xml_diff>
--- a/output/지브라_스캐너_옵션추가.xlsx
+++ b/output/지브라_스캐너_옵션추가.xlsx
@@ -10403,14 +10403,19 @@
         <f>1-(D12/K12)</f>
         <v/>
       </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>단종</t>
+        </is>
+      </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>옵션 정보 없음(상품 엑셀에 미포함)</t>
+          <t>-</t>
         </is>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>확인필요</t>
+          <t>-</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add competitor price comparison columns on a USB-included basis
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0164u4m2HzVL7yDN6jZnxUBp
</commit_message>
<xml_diff>
--- a/output/지브라_스캐너_옵션추가.xlsx
+++ b/output/지브라_스캐너_옵션추가.xlsx
@@ -236,7 +236,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="35">
+  <fills count="36">
     <fill>
       <patternFill/>
     </fill>
@@ -426,6 +426,11 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -705,7 +710,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -771,6 +776,11 @@
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="35" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="164" fontId="25" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment vertical="center"/>
     </xf>
@@ -9697,7 +9707,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R31"/>
+  <dimension ref="A1:X31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="16.375" customWidth="1" style="16" min="2" max="2"/>
@@ -9711,6 +9721,12 @@
     <col width="48" customWidth="1" style="16" min="16" max="16"/>
     <col width="20" customWidth="1" style="16" min="17" max="17"/>
     <col width="22" customWidth="1" style="16" min="18" max="18"/>
+    <col width="16" customWidth="1" style="16" min="19" max="19"/>
+    <col width="14" customWidth="1" style="16" min="20" max="20"/>
+    <col width="20" customWidth="1" style="16" min="21" max="21"/>
+    <col width="24" customWidth="1" style="16" min="22" max="22"/>
+    <col width="16" customWidth="1" style="16" min="23" max="23"/>
+    <col width="18" customWidth="1" style="16" min="24" max="24"/>
   </cols>
   <sheetData>
     <row r="1" ht="18.75" customHeight="1" s="16">
@@ -9796,6 +9812,36 @@
           <t>USB포함가(18,000원 기준)</t>
         </is>
       </c>
+      <c r="S1" s="4" t="inlineStr">
+        <is>
+          <t>타업체명</t>
+        </is>
+      </c>
+      <c r="T1" s="4" t="inlineStr">
+        <is>
+          <t>타업체 판매가</t>
+        </is>
+      </c>
+      <c r="U1" s="4" t="inlineStr">
+        <is>
+          <t>타업체 케이블포함(O/X)</t>
+        </is>
+      </c>
+      <c r="V1" s="4" t="inlineStr">
+        <is>
+          <t>타업체 케이블가(모르면 비움)</t>
+        </is>
+      </c>
+      <c r="W1" s="4" t="inlineStr">
+        <is>
+          <t>타업체 USB포함가</t>
+        </is>
+      </c>
+      <c r="X1" s="4" t="inlineStr">
+        <is>
+          <t>가격차(우리-타업체)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="n">
@@ -9835,6 +9881,18 @@
         <f>IF(Q2="X",F2+18000,F2)</f>
         <v/>
       </c>
+      <c r="S2" s="23" t="n"/>
+      <c r="T2" s="24" t="n"/>
+      <c r="U2" s="25" t="n"/>
+      <c r="V2" s="24" t="n"/>
+      <c r="W2" s="22">
+        <f>IF(T2="","",IF(U2="O",T2,T2+IF(V2="",18000,V2)))</f>
+        <v/>
+      </c>
+      <c r="X2" s="22">
+        <f>IF(OR(W2="",R2=""),"",R2-W2)</f>
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="n">
@@ -9866,7 +9924,7 @@
         <f>J3/110%</f>
         <v/>
       </c>
-      <c r="L3" s="23" t="inlineStr">
+      <c r="L3" s="26" t="inlineStr">
         <is>
           <t>제벡스코리아</t>
         </is>
@@ -9892,6 +9950,18 @@
       </c>
       <c r="R3" s="22">
         <f>IF(Q3="X",F3+18000,F3)</f>
+        <v/>
+      </c>
+      <c r="S3" s="23" t="n"/>
+      <c r="T3" s="24" t="n"/>
+      <c r="U3" s="25" t="n"/>
+      <c r="V3" s="24" t="n"/>
+      <c r="W3" s="22">
+        <f>IF(T3="","",IF(U3="O",T3,T3+IF(V3="",18000,V3)))</f>
+        <v/>
+      </c>
+      <c r="X3" s="22">
+        <f>IF(OR(W3="",R3=""),"",R3-W3)</f>
         <v/>
       </c>
     </row>
@@ -9925,7 +9995,7 @@
         <f>J4/110%</f>
         <v/>
       </c>
-      <c r="L4" s="23" t="inlineStr">
+      <c r="L4" s="26" t="inlineStr">
         <is>
           <t>마켓굿초이스</t>
         </is>
@@ -9955,6 +10025,18 @@
         <f>IF(Q4="X",F4+18000,F4)</f>
         <v/>
       </c>
+      <c r="S4" s="23" t="n"/>
+      <c r="T4" s="24" t="n"/>
+      <c r="U4" s="25" t="n"/>
+      <c r="V4" s="24" t="n"/>
+      <c r="W4" s="22">
+        <f>IF(T4="","",IF(U4="O",T4,T4+IF(V4="",18000,V4)))</f>
+        <v/>
+      </c>
+      <c r="X4" s="22">
+        <f>IF(OR(W4="",R4=""),"",R4-W4)</f>
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="n">
@@ -9986,7 +10068,7 @@
         <f>J5/110%</f>
         <v/>
       </c>
-      <c r="L5" s="23" t="inlineStr">
+      <c r="L5" s="26" t="inlineStr">
         <is>
           <t>바코드다판다</t>
         </is>
@@ -10012,6 +10094,18 @@
       </c>
       <c r="R5" s="22">
         <f>IF(Q5="X",F5+18000,F5)</f>
+        <v/>
+      </c>
+      <c r="S5" s="23" t="n"/>
+      <c r="T5" s="24" t="n"/>
+      <c r="U5" s="25" t="n"/>
+      <c r="V5" s="24" t="n"/>
+      <c r="W5" s="22">
+        <f>IF(T5="","",IF(U5="O",T5,T5+IF(V5="",18000,V5)))</f>
+        <v/>
+      </c>
+      <c r="X5" s="22">
+        <f>IF(OR(W5="",R5=""),"",R5-W5)</f>
         <v/>
       </c>
     </row>
@@ -10045,7 +10139,7 @@
         <f>J6/110%</f>
         <v/>
       </c>
-      <c r="L6" s="23" t="inlineStr">
+      <c r="L6" s="26" t="inlineStr">
         <is>
           <t>에이치에스스토어(usb제외)</t>
         </is>
@@ -10075,6 +10169,18 @@
         <f>IF(Q6="X",F6+18000,F6)</f>
         <v/>
       </c>
+      <c r="S6" s="23" t="n"/>
+      <c r="T6" s="24" t="n"/>
+      <c r="U6" s="25" t="n"/>
+      <c r="V6" s="24" t="n"/>
+      <c r="W6" s="22">
+        <f>IF(T6="","",IF(U6="O",T6,T6+IF(V6="",18000,V6)))</f>
+        <v/>
+      </c>
+      <c r="X6" s="22">
+        <f>IF(OR(W6="",R6=""),"",R6-W6)</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="n">
@@ -10103,7 +10209,7 @@
         <f>J7/110%</f>
         <v/>
       </c>
-      <c r="L7" s="23" t="inlineStr">
+      <c r="L7" s="26" t="inlineStr">
         <is>
           <t>컴엔더</t>
         </is>
@@ -10128,6 +10234,18 @@
       </c>
       <c r="R7" s="22">
         <f>IF(Q7="X",F7+18000,F7)</f>
+        <v/>
+      </c>
+      <c r="S7" s="23" t="n"/>
+      <c r="T7" s="24" t="n"/>
+      <c r="U7" s="25" t="n"/>
+      <c r="V7" s="24" t="n"/>
+      <c r="W7" s="22">
+        <f>IF(T7="","",IF(U7="O",T7,T7+IF(V7="",18000,V7)))</f>
+        <v/>
+      </c>
+      <c r="X7" s="22">
+        <f>IF(OR(W7="",R7=""),"",R7-W7)</f>
         <v/>
       </c>
     </row>
@@ -10161,7 +10279,7 @@
         <f>J8/110%</f>
         <v/>
       </c>
-      <c r="L8" s="23" t="inlineStr">
+      <c r="L8" s="26" t="inlineStr">
         <is>
           <t>유니정보</t>
         </is>
@@ -10186,6 +10304,18 @@
       </c>
       <c r="R8" s="22">
         <f>IF(Q8="X",F8+18000,F8)</f>
+        <v/>
+      </c>
+      <c r="S8" s="23" t="n"/>
+      <c r="T8" s="24" t="n"/>
+      <c r="U8" s="25" t="n"/>
+      <c r="V8" s="24" t="n"/>
+      <c r="W8" s="22">
+        <f>IF(T8="","",IF(U8="O",T8,T8+IF(V8="",18000,V8)))</f>
+        <v/>
+      </c>
+      <c r="X8" s="22">
+        <f>IF(OR(W8="",R8=""),"",R8-W8)</f>
         <v/>
       </c>
     </row>
@@ -10219,7 +10349,7 @@
         <f>J9/110%</f>
         <v/>
       </c>
-      <c r="L9" s="23" t="inlineStr">
+      <c r="L9" s="26" t="inlineStr">
         <is>
           <t>더원시스</t>
         </is>
@@ -10244,6 +10374,18 @@
       </c>
       <c r="R9" s="22">
         <f>IF(Q9="X",F9+18000,F9)</f>
+        <v/>
+      </c>
+      <c r="S9" s="23" t="n"/>
+      <c r="T9" s="24" t="n"/>
+      <c r="U9" s="25" t="n"/>
+      <c r="V9" s="24" t="n"/>
+      <c r="W9" s="22">
+        <f>IF(T9="","",IF(U9="O",T9,T9+IF(V9="",18000,V9)))</f>
+        <v/>
+      </c>
+      <c r="X9" s="22">
+        <f>IF(OR(W9="",R9=""),"",R9-W9)</f>
         <v/>
       </c>
     </row>
@@ -10274,7 +10416,7 @@
         <f>J10/110%</f>
         <v/>
       </c>
-      <c r="L10" s="23" t="inlineStr">
+      <c r="L10" s="26" t="inlineStr">
         <is>
           <t>착한라벨</t>
         </is>
@@ -10299,6 +10441,18 @@
       </c>
       <c r="R10" s="22">
         <f>IF(Q10="X",F10+18000,F10)</f>
+        <v/>
+      </c>
+      <c r="S10" s="23" t="n"/>
+      <c r="T10" s="24" t="n"/>
+      <c r="U10" s="25" t="n"/>
+      <c r="V10" s="24" t="n"/>
+      <c r="W10" s="22">
+        <f>IF(T10="","",IF(U10="O",T10,T10+IF(V10="",18000,V10)))</f>
+        <v/>
+      </c>
+      <c r="X10" s="22">
+        <f>IF(OR(W10="",R10=""),"",R10-W10)</f>
         <v/>
       </c>
     </row>
@@ -10332,7 +10486,7 @@
         <f>J11/110%</f>
         <v/>
       </c>
-      <c r="L11" s="24" t="inlineStr">
+      <c r="L11" s="27" t="inlineStr">
         <is>
           <t>디앤에스테크(USB미포함)</t>
         </is>
@@ -10357,6 +10511,18 @@
       </c>
       <c r="R11" s="22">
         <f>IF(Q11="X",F11+18000,F11)</f>
+        <v/>
+      </c>
+      <c r="S11" s="23" t="n"/>
+      <c r="T11" s="24" t="n"/>
+      <c r="U11" s="25" t="n"/>
+      <c r="V11" s="24" t="n"/>
+      <c r="W11" s="22">
+        <f>IF(T11="","",IF(U11="O",T11,T11+IF(V11="",18000,V11)))</f>
+        <v/>
+      </c>
+      <c r="X11" s="22">
+        <f>IF(OR(W11="",R11=""),"",R11-W11)</f>
         <v/>
       </c>
     </row>
@@ -10390,7 +10556,7 @@
         <f>J12/110%</f>
         <v/>
       </c>
-      <c r="L12" s="23" t="inlineStr">
+      <c r="L12" s="26" t="inlineStr">
         <is>
           <t>유니정보</t>
         </is>
@@ -10417,6 +10583,18 @@
         <is>
           <t>-</t>
         </is>
+      </c>
+      <c r="S12" s="23" t="n"/>
+      <c r="T12" s="24" t="n"/>
+      <c r="U12" s="25" t="n"/>
+      <c r="V12" s="24" t="n"/>
+      <c r="W12" s="22">
+        <f>IF(T12="","",IF(U12="O",T12,T12+IF(V12="",18000,V12)))</f>
+        <v/>
+      </c>
+      <c r="X12" s="22">
+        <f>IF(OR(W12="",R12=""),"",R12-W12)</f>
+        <v/>
       </c>
     </row>
     <row r="13">
@@ -10449,7 +10627,7 @@
         <f>J13/110%</f>
         <v/>
       </c>
-      <c r="L13" s="23" t="inlineStr">
+      <c r="L13" s="26" t="inlineStr">
         <is>
           <t>코스모스몰</t>
         </is>
@@ -10471,6 +10649,18 @@
         <is>
           <t>-</t>
         </is>
+      </c>
+      <c r="S13" s="23" t="n"/>
+      <c r="T13" s="24" t="n"/>
+      <c r="U13" s="25" t="n"/>
+      <c r="V13" s="24" t="n"/>
+      <c r="W13" s="22">
+        <f>IF(T13="","",IF(U13="O",T13,T13+IF(V13="",18000,V13)))</f>
+        <v/>
+      </c>
+      <c r="X13" s="22">
+        <f>IF(OR(W13="",R13=""),"",R13-W13)</f>
+        <v/>
       </c>
     </row>
     <row r="14">
@@ -10503,7 +10693,7 @@
         <f>J14/110%</f>
         <v/>
       </c>
-      <c r="L14" s="23" t="inlineStr">
+      <c r="L14" s="26" t="inlineStr">
         <is>
           <t>더원시스</t>
         </is>
@@ -10533,6 +10723,18 @@
         <f>IF(Q14="X",F14+18000,F14)</f>
         <v/>
       </c>
+      <c r="S14" s="23" t="n"/>
+      <c r="T14" s="24" t="n"/>
+      <c r="U14" s="25" t="n"/>
+      <c r="V14" s="24" t="n"/>
+      <c r="W14" s="22">
+        <f>IF(T14="","",IF(U14="O",T14,T14+IF(V14="",18000,V14)))</f>
+        <v/>
+      </c>
+      <c r="X14" s="22">
+        <f>IF(OR(W14="",R14=""),"",R14-W14)</f>
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="0" t="n">
@@ -10564,7 +10766,7 @@
         <f>J15/110%</f>
         <v/>
       </c>
-      <c r="L15" s="23" t="inlineStr">
+      <c r="L15" s="26" t="inlineStr">
         <is>
           <t>더원시스</t>
         </is>
@@ -10594,6 +10796,18 @@
         <f>IF(Q15="X",F15+18000,F15)</f>
         <v/>
       </c>
+      <c r="S15" s="23" t="n"/>
+      <c r="T15" s="24" t="n"/>
+      <c r="U15" s="25" t="n"/>
+      <c r="V15" s="24" t="n"/>
+      <c r="W15" s="22">
+        <f>IF(T15="","",IF(U15="O",T15,T15+IF(V15="",18000,V15)))</f>
+        <v/>
+      </c>
+      <c r="X15" s="22">
+        <f>IF(OR(W15="",R15=""),"",R15-W15)</f>
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="0" t="n">
@@ -10625,7 +10839,7 @@
         <f>J16/110%</f>
         <v/>
       </c>
-      <c r="L16" s="23" t="inlineStr">
+      <c r="L16" s="26" t="inlineStr">
         <is>
           <t>코스모스몰</t>
         </is>
@@ -10650,6 +10864,18 @@
       </c>
       <c r="R16" s="22">
         <f>IF(Q16="X",F16+18000,F16)</f>
+        <v/>
+      </c>
+      <c r="S16" s="23" t="n"/>
+      <c r="T16" s="24" t="n"/>
+      <c r="U16" s="25" t="n"/>
+      <c r="V16" s="24" t="n"/>
+      <c r="W16" s="22">
+        <f>IF(T16="","",IF(U16="O",T16,T16+IF(V16="",18000,V16)))</f>
+        <v/>
+      </c>
+      <c r="X16" s="22">
+        <f>IF(OR(W16="",R16=""),"",R16-W16)</f>
         <v/>
       </c>
     </row>
@@ -10680,7 +10906,7 @@
         <f>J17/110%</f>
         <v/>
       </c>
-      <c r="L17" s="23" t="inlineStr">
+      <c r="L17" s="26" t="inlineStr">
         <is>
           <t>코스모스몰</t>
         </is>
@@ -10705,6 +10931,18 @@
       </c>
       <c r="R17" s="22">
         <f>IF(Q17="X",F17+18000,F17)</f>
+        <v/>
+      </c>
+      <c r="S17" s="23" t="n"/>
+      <c r="T17" s="24" t="n"/>
+      <c r="U17" s="25" t="n"/>
+      <c r="V17" s="24" t="n"/>
+      <c r="W17" s="22">
+        <f>IF(T17="","",IF(U17="O",T17,T17+IF(V17="",18000,V17)))</f>
+        <v/>
+      </c>
+      <c r="X17" s="22">
+        <f>IF(OR(W17="",R17=""),"",R17-W17)</f>
         <v/>
       </c>
     </row>
@@ -10738,7 +10976,7 @@
         <f>J18/110%</f>
         <v/>
       </c>
-      <c r="L18" s="23" t="inlineStr">
+      <c r="L18" s="26" t="inlineStr">
         <is>
           <t>바코드랩</t>
         </is>
@@ -10763,6 +11001,18 @@
       </c>
       <c r="R18" s="22">
         <f>IF(Q18="X",F18+18000,F18)</f>
+        <v/>
+      </c>
+      <c r="S18" s="23" t="n"/>
+      <c r="T18" s="24" t="n"/>
+      <c r="U18" s="25" t="n"/>
+      <c r="V18" s="24" t="n"/>
+      <c r="W18" s="22">
+        <f>IF(T18="","",IF(U18="O",T18,T18+IF(V18="",18000,V18)))</f>
+        <v/>
+      </c>
+      <c r="X18" s="22">
+        <f>IF(OR(W18="",R18=""),"",R18-W18)</f>
         <v/>
       </c>
     </row>
@@ -10796,7 +11046,7 @@
         <f>J19/110%</f>
         <v/>
       </c>
-      <c r="L19" s="23" t="inlineStr">
+      <c r="L19" s="26" t="inlineStr">
         <is>
           <t>바코드랩</t>
         </is>
@@ -10821,6 +11071,18 @@
       </c>
       <c r="R19" s="22">
         <f>IF(Q19="X",F19+18000,F19)</f>
+        <v/>
+      </c>
+      <c r="S19" s="23" t="n"/>
+      <c r="T19" s="24" t="n"/>
+      <c r="U19" s="25" t="n"/>
+      <c r="V19" s="24" t="n"/>
+      <c r="W19" s="22">
+        <f>IF(T19="","",IF(U19="O",T19,T19+IF(V19="",18000,V19)))</f>
+        <v/>
+      </c>
+      <c r="X19" s="22">
+        <f>IF(OR(W19="",R19=""),"",R19-W19)</f>
         <v/>
       </c>
     </row>
@@ -10851,7 +11113,7 @@
         <f>J20/110%</f>
         <v/>
       </c>
-      <c r="L20" s="23" t="inlineStr">
+      <c r="L20" s="26" t="inlineStr">
         <is>
           <t>코스모스몰</t>
         </is>
@@ -10876,6 +11138,18 @@
       </c>
       <c r="R20" s="22">
         <f>IF(Q20="X",F20+18000,F20)</f>
+        <v/>
+      </c>
+      <c r="S20" s="23" t="n"/>
+      <c r="T20" s="24" t="n"/>
+      <c r="U20" s="25" t="n"/>
+      <c r="V20" s="24" t="n"/>
+      <c r="W20" s="22">
+        <f>IF(T20="","",IF(U20="O",T20,T20+IF(V20="",18000,V20)))</f>
+        <v/>
+      </c>
+      <c r="X20" s="22">
+        <f>IF(OR(W20="",R20=""),"",R20-W20)</f>
         <v/>
       </c>
     </row>
@@ -10906,7 +11180,7 @@
         <f>J21/110%</f>
         <v/>
       </c>
-      <c r="L21" s="23" t="inlineStr">
+      <c r="L21" s="26" t="inlineStr">
         <is>
           <t>유니정보,착한라벨,우주사무기</t>
         </is>
@@ -10931,6 +11205,18 @@
       </c>
       <c r="R21" s="22">
         <f>IF(Q21="X",F21+18000,F21)</f>
+        <v/>
+      </c>
+      <c r="S21" s="23" t="n"/>
+      <c r="T21" s="24" t="n"/>
+      <c r="U21" s="25" t="n"/>
+      <c r="V21" s="24" t="n"/>
+      <c r="W21" s="22">
+        <f>IF(T21="","",IF(U21="O",T21,T21+IF(V21="",18000,V21)))</f>
+        <v/>
+      </c>
+      <c r="X21" s="22">
+        <f>IF(OR(W21="",R21=""),"",R21-W21)</f>
         <v/>
       </c>
     </row>
@@ -10964,7 +11250,7 @@
         <f>J22/110%</f>
         <v/>
       </c>
-      <c r="L22" s="23" t="inlineStr">
+      <c r="L22" s="26" t="inlineStr">
         <is>
           <t>코스모스전문몰</t>
         </is>
@@ -10990,6 +11276,18 @@
       </c>
       <c r="R22" s="22">
         <f>IF(Q22="X",F22+18000,F22)</f>
+        <v/>
+      </c>
+      <c r="S22" s="23" t="n"/>
+      <c r="T22" s="24" t="n"/>
+      <c r="U22" s="25" t="n"/>
+      <c r="V22" s="24" t="n"/>
+      <c r="W22" s="22">
+        <f>IF(T22="","",IF(U22="O",T22,T22+IF(V22="",18000,V22)))</f>
+        <v/>
+      </c>
+      <c r="X22" s="22">
+        <f>IF(OR(W22="",R22=""),"",R22-W22)</f>
         <v/>
       </c>
     </row>
@@ -11023,7 +11321,7 @@
         <f>J23/110%</f>
         <v/>
       </c>
-      <c r="L23" s="23" t="inlineStr">
+      <c r="L23" s="26" t="inlineStr">
         <is>
           <t>코스모스몰,더원시스</t>
         </is>
@@ -11048,6 +11346,18 @@
       </c>
       <c r="R23" s="22">
         <f>IF(Q23="X",F23+18000,F23)</f>
+        <v/>
+      </c>
+      <c r="S23" s="23" t="n"/>
+      <c r="T23" s="24" t="n"/>
+      <c r="U23" s="25" t="n"/>
+      <c r="V23" s="24" t="n"/>
+      <c r="W23" s="22">
+        <f>IF(T23="","",IF(U23="O",T23,T23+IF(V23="",18000,V23)))</f>
+        <v/>
+      </c>
+      <c r="X23" s="22">
+        <f>IF(OR(W23="",R23=""),"",R23-W23)</f>
         <v/>
       </c>
     </row>
@@ -11074,7 +11384,7 @@
       </c>
       <c r="J24" s="19" t="n"/>
       <c r="K24" s="17" t="n"/>
-      <c r="L24" s="23" t="n"/>
+      <c r="L24" s="26" t="n"/>
       <c r="M24" s="3" t="n"/>
       <c r="N24" s="3" t="n"/>
       <c r="O24" t="inlineStr">
@@ -11097,6 +11407,18 @@
         <f>IF(Q24="X",F24+18000,F24)</f>
         <v/>
       </c>
+      <c r="S24" s="23" t="n"/>
+      <c r="T24" s="24" t="n"/>
+      <c r="U24" s="25" t="n"/>
+      <c r="V24" s="24" t="n"/>
+      <c r="W24" s="22">
+        <f>IF(T24="","",IF(U24="O",T24,T24+IF(V24="",18000,V24)))</f>
+        <v/>
+      </c>
+      <c r="X24" s="22">
+        <f>IF(OR(W24="",R24=""),"",R24-W24)</f>
+        <v/>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="0" t="n">
@@ -11121,7 +11443,7 @@
       </c>
       <c r="J25" s="19" t="n"/>
       <c r="K25" s="17" t="n"/>
-      <c r="L25" s="23" t="n"/>
+      <c r="L25" s="26" t="n"/>
       <c r="M25" s="3" t="n"/>
       <c r="N25" s="3" t="n"/>
       <c r="O25" t="inlineStr">
@@ -11144,6 +11466,18 @@
         <f>IF(Q25="X",F25+18000,F25)</f>
         <v/>
       </c>
+      <c r="S25" s="23" t="n"/>
+      <c r="T25" s="24" t="n"/>
+      <c r="U25" s="25" t="n"/>
+      <c r="V25" s="24" t="n"/>
+      <c r="W25" s="22">
+        <f>IF(T25="","",IF(U25="O",T25,T25+IF(V25="",18000,V25)))</f>
+        <v/>
+      </c>
+      <c r="X25" s="22">
+        <f>IF(OR(W25="",R25=""),"",R25-W25)</f>
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="0" t="n">
@@ -11168,7 +11502,7 @@
       </c>
       <c r="J26" s="19" t="n"/>
       <c r="K26" s="17" t="n"/>
-      <c r="L26" s="23" t="n"/>
+      <c r="L26" s="26" t="n"/>
       <c r="M26" s="3" t="n"/>
       <c r="N26" s="3" t="n"/>
       <c r="O26" t="inlineStr">
@@ -11191,6 +11525,18 @@
         <f>IF(Q26="X",F26+18000,F26)</f>
         <v/>
       </c>
+      <c r="S26" s="23" t="n"/>
+      <c r="T26" s="24" t="n"/>
+      <c r="U26" s="25" t="n"/>
+      <c r="V26" s="24" t="n"/>
+      <c r="W26" s="22">
+        <f>IF(T26="","",IF(U26="O",T26,T26+IF(V26="",18000,V26)))</f>
+        <v/>
+      </c>
+      <c r="X26" s="22">
+        <f>IF(OR(W26="",R26=""),"",R26-W26)</f>
+        <v/>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="0" t="n">
@@ -11215,7 +11561,7 @@
       </c>
       <c r="J27" s="19" t="n"/>
       <c r="K27" s="17" t="n"/>
-      <c r="L27" s="23" t="n"/>
+      <c r="L27" s="26" t="n"/>
       <c r="M27" s="3" t="n"/>
       <c r="N27" s="3" t="n"/>
       <c r="O27" t="inlineStr">
@@ -11233,6 +11579,18 @@
           <t>-</t>
         </is>
       </c>
+      <c r="S27" s="23" t="n"/>
+      <c r="T27" s="24" t="n"/>
+      <c r="U27" s="25" t="n"/>
+      <c r="V27" s="24" t="n"/>
+      <c r="W27" s="22">
+        <f>IF(T27="","",IF(U27="O",T27,T27+IF(V27="",18000,V27)))</f>
+        <v/>
+      </c>
+      <c r="X27" s="22">
+        <f>IF(OR(W27="",R27=""),"",R27-W27)</f>
+        <v/>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="0" t="n">
@@ -11257,7 +11615,7 @@
       </c>
       <c r="J28" s="19" t="n"/>
       <c r="K28" s="17" t="n"/>
-      <c r="L28" s="23" t="n"/>
+      <c r="L28" s="26" t="n"/>
       <c r="M28" s="3" t="n"/>
       <c r="N28" s="3" t="n"/>
       <c r="O28" t="inlineStr">
@@ -11275,6 +11633,18 @@
           <t>-</t>
         </is>
       </c>
+      <c r="S28" s="23" t="n"/>
+      <c r="T28" s="24" t="n"/>
+      <c r="U28" s="25" t="n"/>
+      <c r="V28" s="24" t="n"/>
+      <c r="W28" s="22">
+        <f>IF(T28="","",IF(U28="O",T28,T28+IF(V28="",18000,V28)))</f>
+        <v/>
+      </c>
+      <c r="X28" s="22">
+        <f>IF(OR(W28="",R28=""),"",R28-W28)</f>
+        <v/>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="0" t="n">
@@ -11299,7 +11669,7 @@
       </c>
       <c r="J29" s="19" t="n"/>
       <c r="K29" s="17" t="n"/>
-      <c r="L29" s="23" t="n"/>
+      <c r="L29" s="26" t="n"/>
       <c r="M29" s="3" t="n"/>
       <c r="N29" s="3" t="n"/>
       <c r="O29" t="inlineStr">
@@ -11317,6 +11687,18 @@
           <t>-</t>
         </is>
       </c>
+      <c r="S29" s="23" t="n"/>
+      <c r="T29" s="24" t="n"/>
+      <c r="U29" s="25" t="n"/>
+      <c r="V29" s="24" t="n"/>
+      <c r="W29" s="22">
+        <f>IF(T29="","",IF(U29="O",T29,T29+IF(V29="",18000,V29)))</f>
+        <v/>
+      </c>
+      <c r="X29" s="22">
+        <f>IF(OR(W29="",R29=""),"",R29-W29)</f>
+        <v/>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="0" t="n">
@@ -11341,7 +11723,7 @@
       </c>
       <c r="J30" s="19" t="n"/>
       <c r="K30" s="17" t="n"/>
-      <c r="L30" s="23" t="n"/>
+      <c r="L30" s="26" t="n"/>
       <c r="M30" s="3" t="n"/>
       <c r="N30" s="3" t="n"/>
       <c r="O30" t="inlineStr">
@@ -11359,6 +11741,18 @@
           <t>-</t>
         </is>
       </c>
+      <c r="S30" s="23" t="n"/>
+      <c r="T30" s="24" t="n"/>
+      <c r="U30" s="25" t="n"/>
+      <c r="V30" s="24" t="n"/>
+      <c r="W30" s="22">
+        <f>IF(T30="","",IF(U30="O",T30,T30+IF(V30="",18000,V30)))</f>
+        <v/>
+      </c>
+      <c r="X30" s="22">
+        <f>IF(OR(W30="",R30=""),"",R30-W30)</f>
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="0" t="n">
@@ -11383,7 +11777,7 @@
       </c>
       <c r="J31" s="19" t="n"/>
       <c r="K31" s="17" t="n"/>
-      <c r="L31" s="23" t="n"/>
+      <c r="L31" s="26" t="n"/>
       <c r="M31" s="3" t="n"/>
       <c r="N31" s="3" t="n"/>
       <c r="O31" t="inlineStr">
@@ -11401,8 +11795,25 @@
           <t>-</t>
         </is>
       </c>
+      <c r="S31" s="23" t="n"/>
+      <c r="T31" s="24" t="n"/>
+      <c r="U31" s="25" t="n"/>
+      <c r="V31" s="24" t="n"/>
+      <c r="W31" s="22">
+        <f>IF(T31="","",IF(U31="O",T31,T31+IF(V31="",18000,V31)))</f>
+        <v/>
+      </c>
+      <c r="X31" s="22">
+        <f>IF(OR(W31="",R31=""),"",R31-W31)</f>
+        <v/>
+      </c>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="U2:U31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"O,X"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
@@ -11626,35 +12037,35 @@
           <t xml:space="preserve"> 키패드(핸드헬드)</t>
         </is>
       </c>
-      <c r="D4" s="25" t="n">
+      <c r="D4" s="28" t="n">
         <v>1840000</v>
       </c>
-      <c r="E4" s="25">
+      <c r="E4" s="28">
         <f>D4*1.1</f>
         <v/>
       </c>
-      <c r="F4" s="25" t="n">
+      <c r="F4" s="28" t="n">
         <v>2640000</v>
       </c>
-      <c r="G4" s="25">
+      <c r="G4" s="28">
         <f>F4/110%</f>
         <v/>
       </c>
-      <c r="H4" s="26" t="n">
+      <c r="H4" s="29" t="n">
         <v>2500000</v>
       </c>
-      <c r="I4" s="26">
+      <c r="I4" s="29">
         <f>ROUND(H4*1.1/0.95,-1)</f>
         <v/>
       </c>
-      <c r="J4" s="25" t="n">
+      <c r="J4" s="28" t="n">
         <v>2640000</v>
       </c>
-      <c r="K4" s="25">
+      <c r="K4" s="28">
         <f>J4/1.1</f>
         <v/>
       </c>
-      <c r="L4" s="25" t="inlineStr">
+      <c r="L4" s="28" t="inlineStr">
         <is>
           <t>코스모스몰</t>
         </is>
@@ -11841,32 +12252,32 @@
           <t xml:space="preserve"> 프리미엄풀터치</t>
         </is>
       </c>
-      <c r="D8" s="25" t="n">
+      <c r="D8" s="28" t="n">
         <v>2500000</v>
       </c>
-      <c r="E8" s="25">
+      <c r="E8" s="28">
         <f>D8*1.1</f>
         <v/>
       </c>
-      <c r="F8" s="25" t="n">
+      <c r="F8" s="28" t="n">
         <v>2640000</v>
       </c>
-      <c r="G8" s="26" t="n"/>
-      <c r="H8" s="26" t="n">
+      <c r="G8" s="29" t="n"/>
+      <c r="H8" s="29" t="n">
         <v>3000000</v>
       </c>
-      <c r="I8" s="26">
+      <c r="I8" s="29">
         <f>ROUND(H8*1.1/0.95,-1)</f>
         <v/>
       </c>
-      <c r="J8" s="25" t="n">
+      <c r="J8" s="28" t="n">
         <v>2577960</v>
       </c>
-      <c r="K8" s="25">
+      <c r="K8" s="28">
         <f>J8/1.1</f>
         <v/>
       </c>
-      <c r="L8" s="25" t="inlineStr">
+      <c r="L8" s="28" t="inlineStr">
         <is>
           <t>솔바텍지마켓</t>
         </is>
@@ -11945,30 +12356,30 @@
           <t xml:space="preserve"> 키패드(핸드헬드)</t>
         </is>
       </c>
-      <c r="D10" s="25" t="n">
+      <c r="D10" s="28" t="n">
         <v>1490000</v>
       </c>
-      <c r="E10" s="25">
+      <c r="E10" s="28">
         <f>D10*1.1</f>
         <v/>
       </c>
-      <c r="F10" s="25" t="n">
+      <c r="F10" s="28" t="n">
         <v>2750000</v>
       </c>
-      <c r="G10" s="25">
+      <c r="G10" s="28">
         <f>F10/110%</f>
         <v/>
       </c>
-      <c r="H10" s="25" t="n"/>
-      <c r="I10" s="25" t="n"/>
-      <c r="J10" s="25" t="n">
+      <c r="H10" s="28" t="n"/>
+      <c r="I10" s="28" t="n"/>
+      <c r="J10" s="28" t="n">
         <v>2750000</v>
       </c>
-      <c r="K10" s="25">
+      <c r="K10" s="28">
         <f>J10/1.1</f>
         <v/>
       </c>
-      <c r="L10" s="25" t="inlineStr">
+      <c r="L10" s="28" t="inlineStr">
         <is>
           <t>코스모스몰,더원시스</t>
         </is>
@@ -12139,7 +12550,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="I18" s="27" t="n"/>
+      <c r="I18" s="30" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Add USB-included cost and margin columns (cable cost 9,000 KRW)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0164u4m2HzVL7yDN6jZnxUBp
</commit_message>
<xml_diff>
--- a/output/지브라_스캐너_옵션추가.xlsx
+++ b/output/지브라_스캐너_옵션추가.xlsx
@@ -710,7 +710,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -781,6 +781,7 @@
     <xf numFmtId="0" fontId="0" fillId="35" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="25" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment vertical="center"/>
     </xf>
@@ -9707,7 +9708,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X31"/>
+  <dimension ref="A1:AA31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="16.375" customWidth="1" style="16" min="2" max="2"/>
@@ -9727,6 +9728,9 @@
     <col width="24" customWidth="1" style="16" min="22" max="22"/>
     <col width="16" customWidth="1" style="16" min="23" max="23"/>
     <col width="18" customWidth="1" style="16" min="24" max="24"/>
+    <col width="20" customWidth="1" style="16" min="25" max="25"/>
+    <col width="20" customWidth="1" style="16" min="26" max="26"/>
+    <col width="18" customWidth="1" style="16" min="27" max="27"/>
   </cols>
   <sheetData>
     <row r="1" ht="18.75" customHeight="1" s="16">
@@ -9840,6 +9844,21 @@
       <c r="X1" s="4" t="inlineStr">
         <is>
           <t>가격차(우리-타업체)</t>
+        </is>
+      </c>
+      <c r="Y1" s="4" t="inlineStr">
+        <is>
+          <t>USB포함 매입가(VAT별도)</t>
+        </is>
+      </c>
+      <c r="Z1" s="4" t="inlineStr">
+        <is>
+          <t>현재 마진율(USB포함 기준)</t>
+        </is>
+      </c>
+      <c r="AA1" s="4" t="inlineStr">
+        <is>
+          <t>타업체가 기준 마진율</t>
         </is>
       </c>
     </row>
@@ -9893,6 +9912,18 @@
         <f>IF(OR(W2="",R2=""),"",R2-W2)</f>
         <v/>
       </c>
+      <c r="Y2" s="22">
+        <f>IF(OR(D2="",R2=""),"",IF(Q2="X",D2+9000,D2))</f>
+        <v/>
+      </c>
+      <c r="Z2" s="26">
+        <f>IF(Y2="","",1-Y2/(R2/110%))</f>
+        <v/>
+      </c>
+      <c r="AA2" s="26">
+        <f>IF(OR(Y2="",W2=""),"",1-Y2/(W2/110%))</f>
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="n">
@@ -9924,7 +9955,7 @@
         <f>J3/110%</f>
         <v/>
       </c>
-      <c r="L3" s="26" t="inlineStr">
+      <c r="L3" s="27" t="inlineStr">
         <is>
           <t>제벡스코리아</t>
         </is>
@@ -9964,6 +9995,18 @@
         <f>IF(OR(W3="",R3=""),"",R3-W3)</f>
         <v/>
       </c>
+      <c r="Y3" s="22">
+        <f>IF(OR(D3="",R3=""),"",IF(Q3="X",D3+9000,D3))</f>
+        <v/>
+      </c>
+      <c r="Z3" s="26">
+        <f>IF(Y3="","",1-Y3/(R3/110%))</f>
+        <v/>
+      </c>
+      <c r="AA3" s="26">
+        <f>IF(OR(Y3="",W3=""),"",1-Y3/(W3/110%))</f>
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="n">
@@ -9995,7 +10038,7 @@
         <f>J4/110%</f>
         <v/>
       </c>
-      <c r="L4" s="26" t="inlineStr">
+      <c r="L4" s="27" t="inlineStr">
         <is>
           <t>마켓굿초이스</t>
         </is>
@@ -10037,6 +10080,18 @@
         <f>IF(OR(W4="",R4=""),"",R4-W4)</f>
         <v/>
       </c>
+      <c r="Y4" s="22">
+        <f>IF(OR(D4="",R4=""),"",IF(Q4="X",D4+9000,D4))</f>
+        <v/>
+      </c>
+      <c r="Z4" s="26">
+        <f>IF(Y4="","",1-Y4/(R4/110%))</f>
+        <v/>
+      </c>
+      <c r="AA4" s="26">
+        <f>IF(OR(Y4="",W4=""),"",1-Y4/(W4/110%))</f>
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="n">
@@ -10068,7 +10123,7 @@
         <f>J5/110%</f>
         <v/>
       </c>
-      <c r="L5" s="26" t="inlineStr">
+      <c r="L5" s="27" t="inlineStr">
         <is>
           <t>바코드다판다</t>
         </is>
@@ -10108,6 +10163,18 @@
         <f>IF(OR(W5="",R5=""),"",R5-W5)</f>
         <v/>
       </c>
+      <c r="Y5" s="22">
+        <f>IF(OR(D5="",R5=""),"",IF(Q5="X",D5+9000,D5))</f>
+        <v/>
+      </c>
+      <c r="Z5" s="26">
+        <f>IF(Y5="","",1-Y5/(R5/110%))</f>
+        <v/>
+      </c>
+      <c r="AA5" s="26">
+        <f>IF(OR(Y5="",W5=""),"",1-Y5/(W5/110%))</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="n">
@@ -10139,7 +10206,7 @@
         <f>J6/110%</f>
         <v/>
       </c>
-      <c r="L6" s="26" t="inlineStr">
+      <c r="L6" s="27" t="inlineStr">
         <is>
           <t>에이치에스스토어(usb제외)</t>
         </is>
@@ -10181,6 +10248,18 @@
         <f>IF(OR(W6="",R6=""),"",R6-W6)</f>
         <v/>
       </c>
+      <c r="Y6" s="22">
+        <f>IF(OR(D6="",R6=""),"",IF(Q6="X",D6+9000,D6))</f>
+        <v/>
+      </c>
+      <c r="Z6" s="26">
+        <f>IF(Y6="","",1-Y6/(R6/110%))</f>
+        <v/>
+      </c>
+      <c r="AA6" s="26">
+        <f>IF(OR(Y6="",W6=""),"",1-Y6/(W6/110%))</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="n">
@@ -10209,7 +10288,7 @@
         <f>J7/110%</f>
         <v/>
       </c>
-      <c r="L7" s="26" t="inlineStr">
+      <c r="L7" s="27" t="inlineStr">
         <is>
           <t>컴엔더</t>
         </is>
@@ -10248,6 +10327,18 @@
         <f>IF(OR(W7="",R7=""),"",R7-W7)</f>
         <v/>
       </c>
+      <c r="Y7" s="22">
+        <f>IF(OR(D7="",R7=""),"",IF(Q7="X",D7+9000,D7))</f>
+        <v/>
+      </c>
+      <c r="Z7" s="26">
+        <f>IF(Y7="","",1-Y7/(R7/110%))</f>
+        <v/>
+      </c>
+      <c r="AA7" s="26">
+        <f>IF(OR(Y7="",W7=""),"",1-Y7/(W7/110%))</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="n">
@@ -10279,7 +10370,7 @@
         <f>J8/110%</f>
         <v/>
       </c>
-      <c r="L8" s="26" t="inlineStr">
+      <c r="L8" s="27" t="inlineStr">
         <is>
           <t>유니정보</t>
         </is>
@@ -10318,6 +10409,18 @@
         <f>IF(OR(W8="",R8=""),"",R8-W8)</f>
         <v/>
       </c>
+      <c r="Y8" s="22">
+        <f>IF(OR(D8="",R8=""),"",IF(Q8="X",D8+9000,D8))</f>
+        <v/>
+      </c>
+      <c r="Z8" s="26">
+        <f>IF(Y8="","",1-Y8/(R8/110%))</f>
+        <v/>
+      </c>
+      <c r="AA8" s="26">
+        <f>IF(OR(Y8="",W8=""),"",1-Y8/(W8/110%))</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="n">
@@ -10349,7 +10452,7 @@
         <f>J9/110%</f>
         <v/>
       </c>
-      <c r="L9" s="26" t="inlineStr">
+      <c r="L9" s="27" t="inlineStr">
         <is>
           <t>더원시스</t>
         </is>
@@ -10388,6 +10491,18 @@
         <f>IF(OR(W9="",R9=""),"",R9-W9)</f>
         <v/>
       </c>
+      <c r="Y9" s="22">
+        <f>IF(OR(D9="",R9=""),"",IF(Q9="X",D9+9000,D9))</f>
+        <v/>
+      </c>
+      <c r="Z9" s="26">
+        <f>IF(Y9="","",1-Y9/(R9/110%))</f>
+        <v/>
+      </c>
+      <c r="AA9" s="26">
+        <f>IF(OR(Y9="",W9=""),"",1-Y9/(W9/110%))</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="n">
@@ -10416,7 +10531,7 @@
         <f>J10/110%</f>
         <v/>
       </c>
-      <c r="L10" s="26" t="inlineStr">
+      <c r="L10" s="27" t="inlineStr">
         <is>
           <t>착한라벨</t>
         </is>
@@ -10455,6 +10570,18 @@
         <f>IF(OR(W10="",R10=""),"",R10-W10)</f>
         <v/>
       </c>
+      <c r="Y10" s="22">
+        <f>IF(OR(D10="",R10=""),"",IF(Q10="X",D10+9000,D10))</f>
+        <v/>
+      </c>
+      <c r="Z10" s="26">
+        <f>IF(Y10="","",1-Y10/(R10/110%))</f>
+        <v/>
+      </c>
+      <c r="AA10" s="26">
+        <f>IF(OR(Y10="",W10=""),"",1-Y10/(W10/110%))</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="n">
@@ -10486,7 +10613,7 @@
         <f>J11/110%</f>
         <v/>
       </c>
-      <c r="L11" s="27" t="inlineStr">
+      <c r="L11" s="28" t="inlineStr">
         <is>
           <t>디앤에스테크(USB미포함)</t>
         </is>
@@ -10525,6 +10652,18 @@
         <f>IF(OR(W11="",R11=""),"",R11-W11)</f>
         <v/>
       </c>
+      <c r="Y11" s="22">
+        <f>IF(OR(D11="",R11=""),"",IF(Q11="X",D11+9000,D11))</f>
+        <v/>
+      </c>
+      <c r="Z11" s="26">
+        <f>IF(Y11="","",1-Y11/(R11/110%))</f>
+        <v/>
+      </c>
+      <c r="AA11" s="26">
+        <f>IF(OR(Y11="",W11=""),"",1-Y11/(W11/110%))</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="0" t="n">
@@ -10556,7 +10695,7 @@
         <f>J12/110%</f>
         <v/>
       </c>
-      <c r="L12" s="26" t="inlineStr">
+      <c r="L12" s="27" t="inlineStr">
         <is>
           <t>유니정보</t>
         </is>
@@ -10596,6 +10735,18 @@
         <f>IF(OR(W12="",R12=""),"",R12-W12)</f>
         <v/>
       </c>
+      <c r="Y12" s="22">
+        <f>IF(OR(D12="",R12=""),"",IF(Q12="X",D12+9000,D12))</f>
+        <v/>
+      </c>
+      <c r="Z12" s="26">
+        <f>IF(Y12="","",1-Y12/(R12/110%))</f>
+        <v/>
+      </c>
+      <c r="AA12" s="26">
+        <f>IF(OR(Y12="",W12=""),"",1-Y12/(W12/110%))</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="0" t="n">
@@ -10627,7 +10778,7 @@
         <f>J13/110%</f>
         <v/>
       </c>
-      <c r="L13" s="26" t="inlineStr">
+      <c r="L13" s="27" t="inlineStr">
         <is>
           <t>코스모스몰</t>
         </is>
@@ -10662,6 +10813,18 @@
         <f>IF(OR(W13="",R13=""),"",R13-W13)</f>
         <v/>
       </c>
+      <c r="Y13" s="22">
+        <f>IF(OR(D13="",R13=""),"",IF(Q13="X",D13+9000,D13))</f>
+        <v/>
+      </c>
+      <c r="Z13" s="26">
+        <f>IF(Y13="","",1-Y13/(R13/110%))</f>
+        <v/>
+      </c>
+      <c r="AA13" s="26">
+        <f>IF(OR(Y13="",W13=""),"",1-Y13/(W13/110%))</f>
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="0" t="n">
@@ -10693,7 +10856,7 @@
         <f>J14/110%</f>
         <v/>
       </c>
-      <c r="L14" s="26" t="inlineStr">
+      <c r="L14" s="27" t="inlineStr">
         <is>
           <t>더원시스</t>
         </is>
@@ -10735,6 +10898,18 @@
         <f>IF(OR(W14="",R14=""),"",R14-W14)</f>
         <v/>
       </c>
+      <c r="Y14" s="22">
+        <f>IF(OR(D14="",R14=""),"",IF(Q14="X",D14+9000,D14))</f>
+        <v/>
+      </c>
+      <c r="Z14" s="26">
+        <f>IF(Y14="","",1-Y14/(R14/110%))</f>
+        <v/>
+      </c>
+      <c r="AA14" s="26">
+        <f>IF(OR(Y14="",W14=""),"",1-Y14/(W14/110%))</f>
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="0" t="n">
@@ -10766,7 +10941,7 @@
         <f>J15/110%</f>
         <v/>
       </c>
-      <c r="L15" s="26" t="inlineStr">
+      <c r="L15" s="27" t="inlineStr">
         <is>
           <t>더원시스</t>
         </is>
@@ -10808,6 +10983,18 @@
         <f>IF(OR(W15="",R15=""),"",R15-W15)</f>
         <v/>
       </c>
+      <c r="Y15" s="22">
+        <f>IF(OR(D15="",R15=""),"",IF(Q15="X",D15+9000,D15))</f>
+        <v/>
+      </c>
+      <c r="Z15" s="26">
+        <f>IF(Y15="","",1-Y15/(R15/110%))</f>
+        <v/>
+      </c>
+      <c r="AA15" s="26">
+        <f>IF(OR(Y15="",W15=""),"",1-Y15/(W15/110%))</f>
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="0" t="n">
@@ -10839,7 +11026,7 @@
         <f>J16/110%</f>
         <v/>
       </c>
-      <c r="L16" s="26" t="inlineStr">
+      <c r="L16" s="27" t="inlineStr">
         <is>
           <t>코스모스몰</t>
         </is>
@@ -10878,6 +11065,18 @@
         <f>IF(OR(W16="",R16=""),"",R16-W16)</f>
         <v/>
       </c>
+      <c r="Y16" s="22">
+        <f>IF(OR(D16="",R16=""),"",IF(Q16="X",D16+9000,D16))</f>
+        <v/>
+      </c>
+      <c r="Z16" s="26">
+        <f>IF(Y16="","",1-Y16/(R16/110%))</f>
+        <v/>
+      </c>
+      <c r="AA16" s="26">
+        <f>IF(OR(Y16="",W16=""),"",1-Y16/(W16/110%))</f>
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="0" t="n">
@@ -10906,7 +11105,7 @@
         <f>J17/110%</f>
         <v/>
       </c>
-      <c r="L17" s="26" t="inlineStr">
+      <c r="L17" s="27" t="inlineStr">
         <is>
           <t>코스모스몰</t>
         </is>
@@ -10945,6 +11144,18 @@
         <f>IF(OR(W17="",R17=""),"",R17-W17)</f>
         <v/>
       </c>
+      <c r="Y17" s="22">
+        <f>IF(OR(D17="",R17=""),"",IF(Q17="X",D17+9000,D17))</f>
+        <v/>
+      </c>
+      <c r="Z17" s="26">
+        <f>IF(Y17="","",1-Y17/(R17/110%))</f>
+        <v/>
+      </c>
+      <c r="AA17" s="26">
+        <f>IF(OR(Y17="",W17=""),"",1-Y17/(W17/110%))</f>
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="0" t="n">
@@ -10976,7 +11187,7 @@
         <f>J18/110%</f>
         <v/>
       </c>
-      <c r="L18" s="26" t="inlineStr">
+      <c r="L18" s="27" t="inlineStr">
         <is>
           <t>바코드랩</t>
         </is>
@@ -11015,6 +11226,18 @@
         <f>IF(OR(W18="",R18=""),"",R18-W18)</f>
         <v/>
       </c>
+      <c r="Y18" s="22">
+        <f>IF(OR(D18="",R18=""),"",IF(Q18="X",D18+9000,D18))</f>
+        <v/>
+      </c>
+      <c r="Z18" s="26">
+        <f>IF(Y18="","",1-Y18/(R18/110%))</f>
+        <v/>
+      </c>
+      <c r="AA18" s="26">
+        <f>IF(OR(Y18="",W18=""),"",1-Y18/(W18/110%))</f>
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="0" t="n">
@@ -11046,7 +11269,7 @@
         <f>J19/110%</f>
         <v/>
       </c>
-      <c r="L19" s="26" t="inlineStr">
+      <c r="L19" s="27" t="inlineStr">
         <is>
           <t>바코드랩</t>
         </is>
@@ -11085,6 +11308,18 @@
         <f>IF(OR(W19="",R19=""),"",R19-W19)</f>
         <v/>
       </c>
+      <c r="Y19" s="22">
+        <f>IF(OR(D19="",R19=""),"",IF(Q19="X",D19+9000,D19))</f>
+        <v/>
+      </c>
+      <c r="Z19" s="26">
+        <f>IF(Y19="","",1-Y19/(R19/110%))</f>
+        <v/>
+      </c>
+      <c r="AA19" s="26">
+        <f>IF(OR(Y19="",W19=""),"",1-Y19/(W19/110%))</f>
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="0" t="n">
@@ -11113,7 +11348,7 @@
         <f>J20/110%</f>
         <v/>
       </c>
-      <c r="L20" s="26" t="inlineStr">
+      <c r="L20" s="27" t="inlineStr">
         <is>
           <t>코스모스몰</t>
         </is>
@@ -11152,6 +11387,18 @@
         <f>IF(OR(W20="",R20=""),"",R20-W20)</f>
         <v/>
       </c>
+      <c r="Y20" s="22">
+        <f>IF(OR(D20="",R20=""),"",IF(Q20="X",D20+9000,D20))</f>
+        <v/>
+      </c>
+      <c r="Z20" s="26">
+        <f>IF(Y20="","",1-Y20/(R20/110%))</f>
+        <v/>
+      </c>
+      <c r="AA20" s="26">
+        <f>IF(OR(Y20="",W20=""),"",1-Y20/(W20/110%))</f>
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="0" t="n">
@@ -11180,7 +11427,7 @@
         <f>J21/110%</f>
         <v/>
       </c>
-      <c r="L21" s="26" t="inlineStr">
+      <c r="L21" s="27" t="inlineStr">
         <is>
           <t>유니정보,착한라벨,우주사무기</t>
         </is>
@@ -11219,6 +11466,18 @@
         <f>IF(OR(W21="",R21=""),"",R21-W21)</f>
         <v/>
       </c>
+      <c r="Y21" s="22">
+        <f>IF(OR(D21="",R21=""),"",IF(Q21="X",D21+9000,D21))</f>
+        <v/>
+      </c>
+      <c r="Z21" s="26">
+        <f>IF(Y21="","",1-Y21/(R21/110%))</f>
+        <v/>
+      </c>
+      <c r="AA21" s="26">
+        <f>IF(OR(Y21="",W21=""),"",1-Y21/(W21/110%))</f>
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="0" t="n">
@@ -11250,7 +11509,7 @@
         <f>J22/110%</f>
         <v/>
       </c>
-      <c r="L22" s="26" t="inlineStr">
+      <c r="L22" s="27" t="inlineStr">
         <is>
           <t>코스모스전문몰</t>
         </is>
@@ -11290,6 +11549,18 @@
         <f>IF(OR(W22="",R22=""),"",R22-W22)</f>
         <v/>
       </c>
+      <c r="Y22" s="22">
+        <f>IF(OR(D22="",R22=""),"",IF(Q22="X",D22+9000,D22))</f>
+        <v/>
+      </c>
+      <c r="Z22" s="26">
+        <f>IF(Y22="","",1-Y22/(R22/110%))</f>
+        <v/>
+      </c>
+      <c r="AA22" s="26">
+        <f>IF(OR(Y22="",W22=""),"",1-Y22/(W22/110%))</f>
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="0" t="n">
@@ -11321,7 +11592,7 @@
         <f>J23/110%</f>
         <v/>
       </c>
-      <c r="L23" s="26" t="inlineStr">
+      <c r="L23" s="27" t="inlineStr">
         <is>
           <t>코스모스몰,더원시스</t>
         </is>
@@ -11360,6 +11631,18 @@
         <f>IF(OR(W23="",R23=""),"",R23-W23)</f>
         <v/>
       </c>
+      <c r="Y23" s="22">
+        <f>IF(OR(D23="",R23=""),"",IF(Q23="X",D23+9000,D23))</f>
+        <v/>
+      </c>
+      <c r="Z23" s="26">
+        <f>IF(Y23="","",1-Y23/(R23/110%))</f>
+        <v/>
+      </c>
+      <c r="AA23" s="26">
+        <f>IF(OR(Y23="",W23=""),"",1-Y23/(W23/110%))</f>
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="0" t="n">
@@ -11384,7 +11667,7 @@
       </c>
       <c r="J24" s="19" t="n"/>
       <c r="K24" s="17" t="n"/>
-      <c r="L24" s="26" t="n"/>
+      <c r="L24" s="27" t="n"/>
       <c r="M24" s="3" t="n"/>
       <c r="N24" s="3" t="n"/>
       <c r="O24" t="inlineStr">
@@ -11419,6 +11702,18 @@
         <f>IF(OR(W24="",R24=""),"",R24-W24)</f>
         <v/>
       </c>
+      <c r="Y24" s="22">
+        <f>IF(OR(D24="",R24=""),"",IF(Q24="X",D24+9000,D24))</f>
+        <v/>
+      </c>
+      <c r="Z24" s="26">
+        <f>IF(Y24="","",1-Y24/(R24/110%))</f>
+        <v/>
+      </c>
+      <c r="AA24" s="26">
+        <f>IF(OR(Y24="",W24=""),"",1-Y24/(W24/110%))</f>
+        <v/>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="0" t="n">
@@ -11443,7 +11738,7 @@
       </c>
       <c r="J25" s="19" t="n"/>
       <c r="K25" s="17" t="n"/>
-      <c r="L25" s="26" t="n"/>
+      <c r="L25" s="27" t="n"/>
       <c r="M25" s="3" t="n"/>
       <c r="N25" s="3" t="n"/>
       <c r="O25" t="inlineStr">
@@ -11478,6 +11773,18 @@
         <f>IF(OR(W25="",R25=""),"",R25-W25)</f>
         <v/>
       </c>
+      <c r="Y25" s="22">
+        <f>IF(OR(D25="",R25=""),"",IF(Q25="X",D25+9000,D25))</f>
+        <v/>
+      </c>
+      <c r="Z25" s="26">
+        <f>IF(Y25="","",1-Y25/(R25/110%))</f>
+        <v/>
+      </c>
+      <c r="AA25" s="26">
+        <f>IF(OR(Y25="",W25=""),"",1-Y25/(W25/110%))</f>
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="0" t="n">
@@ -11502,7 +11809,7 @@
       </c>
       <c r="J26" s="19" t="n"/>
       <c r="K26" s="17" t="n"/>
-      <c r="L26" s="26" t="n"/>
+      <c r="L26" s="27" t="n"/>
       <c r="M26" s="3" t="n"/>
       <c r="N26" s="3" t="n"/>
       <c r="O26" t="inlineStr">
@@ -11537,6 +11844,18 @@
         <f>IF(OR(W26="",R26=""),"",R26-W26)</f>
         <v/>
       </c>
+      <c r="Y26" s="22">
+        <f>IF(OR(D26="",R26=""),"",IF(Q26="X",D26+9000,D26))</f>
+        <v/>
+      </c>
+      <c r="Z26" s="26">
+        <f>IF(Y26="","",1-Y26/(R26/110%))</f>
+        <v/>
+      </c>
+      <c r="AA26" s="26">
+        <f>IF(OR(Y26="",W26=""),"",1-Y26/(W26/110%))</f>
+        <v/>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="0" t="n">
@@ -11561,7 +11880,7 @@
       </c>
       <c r="J27" s="19" t="n"/>
       <c r="K27" s="17" t="n"/>
-      <c r="L27" s="26" t="n"/>
+      <c r="L27" s="27" t="n"/>
       <c r="M27" s="3" t="n"/>
       <c r="N27" s="3" t="n"/>
       <c r="O27" t="inlineStr">
@@ -11591,6 +11910,18 @@
         <f>IF(OR(W27="",R27=""),"",R27-W27)</f>
         <v/>
       </c>
+      <c r="Y27" s="22">
+        <f>IF(OR(D27="",R27=""),"",IF(Q27="X",D27+9000,D27))</f>
+        <v/>
+      </c>
+      <c r="Z27" s="26">
+        <f>IF(Y27="","",1-Y27/(R27/110%))</f>
+        <v/>
+      </c>
+      <c r="AA27" s="26">
+        <f>IF(OR(Y27="",W27=""),"",1-Y27/(W27/110%))</f>
+        <v/>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="0" t="n">
@@ -11615,7 +11946,7 @@
       </c>
       <c r="J28" s="19" t="n"/>
       <c r="K28" s="17" t="n"/>
-      <c r="L28" s="26" t="n"/>
+      <c r="L28" s="27" t="n"/>
       <c r="M28" s="3" t="n"/>
       <c r="N28" s="3" t="n"/>
       <c r="O28" t="inlineStr">
@@ -11645,6 +11976,18 @@
         <f>IF(OR(W28="",R28=""),"",R28-W28)</f>
         <v/>
       </c>
+      <c r="Y28" s="22">
+        <f>IF(OR(D28="",R28=""),"",IF(Q28="X",D28+9000,D28))</f>
+        <v/>
+      </c>
+      <c r="Z28" s="26">
+        <f>IF(Y28="","",1-Y28/(R28/110%))</f>
+        <v/>
+      </c>
+      <c r="AA28" s="26">
+        <f>IF(OR(Y28="",W28=""),"",1-Y28/(W28/110%))</f>
+        <v/>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="0" t="n">
@@ -11669,7 +12012,7 @@
       </c>
       <c r="J29" s="19" t="n"/>
       <c r="K29" s="17" t="n"/>
-      <c r="L29" s="26" t="n"/>
+      <c r="L29" s="27" t="n"/>
       <c r="M29" s="3" t="n"/>
       <c r="N29" s="3" t="n"/>
       <c r="O29" t="inlineStr">
@@ -11699,6 +12042,18 @@
         <f>IF(OR(W29="",R29=""),"",R29-W29)</f>
         <v/>
       </c>
+      <c r="Y29" s="22">
+        <f>IF(OR(D29="",R29=""),"",IF(Q29="X",D29+9000,D29))</f>
+        <v/>
+      </c>
+      <c r="Z29" s="26">
+        <f>IF(Y29="","",1-Y29/(R29/110%))</f>
+        <v/>
+      </c>
+      <c r="AA29" s="26">
+        <f>IF(OR(Y29="",W29=""),"",1-Y29/(W29/110%))</f>
+        <v/>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="0" t="n">
@@ -11723,7 +12078,7 @@
       </c>
       <c r="J30" s="19" t="n"/>
       <c r="K30" s="17" t="n"/>
-      <c r="L30" s="26" t="n"/>
+      <c r="L30" s="27" t="n"/>
       <c r="M30" s="3" t="n"/>
       <c r="N30" s="3" t="n"/>
       <c r="O30" t="inlineStr">
@@ -11753,6 +12108,18 @@
         <f>IF(OR(W30="",R30=""),"",R30-W30)</f>
         <v/>
       </c>
+      <c r="Y30" s="22">
+        <f>IF(OR(D30="",R30=""),"",IF(Q30="X",D30+9000,D30))</f>
+        <v/>
+      </c>
+      <c r="Z30" s="26">
+        <f>IF(Y30="","",1-Y30/(R30/110%))</f>
+        <v/>
+      </c>
+      <c r="AA30" s="26">
+        <f>IF(OR(Y30="",W30=""),"",1-Y30/(W30/110%))</f>
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="0" t="n">
@@ -11777,7 +12144,7 @@
       </c>
       <c r="J31" s="19" t="n"/>
       <c r="K31" s="17" t="n"/>
-      <c r="L31" s="26" t="n"/>
+      <c r="L31" s="27" t="n"/>
       <c r="M31" s="3" t="n"/>
       <c r="N31" s="3" t="n"/>
       <c r="O31" t="inlineStr">
@@ -11805,6 +12172,18 @@
       </c>
       <c r="X31" s="22">
         <f>IF(OR(W31="",R31=""),"",R31-W31)</f>
+        <v/>
+      </c>
+      <c r="Y31" s="22">
+        <f>IF(OR(D31="",R31=""),"",IF(Q31="X",D31+9000,D31))</f>
+        <v/>
+      </c>
+      <c r="Z31" s="26">
+        <f>IF(Y31="","",1-Y31/(R31/110%))</f>
+        <v/>
+      </c>
+      <c r="AA31" s="26">
+        <f>IF(OR(Y31="",W31=""),"",1-Y31/(W31/110%))</f>
         <v/>
       </c>
     </row>
@@ -12037,35 +12416,35 @@
           <t xml:space="preserve"> 키패드(핸드헬드)</t>
         </is>
       </c>
-      <c r="D4" s="28" t="n">
+      <c r="D4" s="29" t="n">
         <v>1840000</v>
       </c>
-      <c r="E4" s="28">
+      <c r="E4" s="29">
         <f>D4*1.1</f>
         <v/>
       </c>
-      <c r="F4" s="28" t="n">
+      <c r="F4" s="29" t="n">
         <v>2640000</v>
       </c>
-      <c r="G4" s="28">
+      <c r="G4" s="29">
         <f>F4/110%</f>
         <v/>
       </c>
-      <c r="H4" s="29" t="n">
+      <c r="H4" s="30" t="n">
         <v>2500000</v>
       </c>
-      <c r="I4" s="29">
+      <c r="I4" s="30">
         <f>ROUND(H4*1.1/0.95,-1)</f>
         <v/>
       </c>
-      <c r="J4" s="28" t="n">
+      <c r="J4" s="29" t="n">
         <v>2640000</v>
       </c>
-      <c r="K4" s="28">
+      <c r="K4" s="29">
         <f>J4/1.1</f>
         <v/>
       </c>
-      <c r="L4" s="28" t="inlineStr">
+      <c r="L4" s="29" t="inlineStr">
         <is>
           <t>코스모스몰</t>
         </is>
@@ -12252,32 +12631,32 @@
           <t xml:space="preserve"> 프리미엄풀터치</t>
         </is>
       </c>
-      <c r="D8" s="28" t="n">
+      <c r="D8" s="29" t="n">
         <v>2500000</v>
       </c>
-      <c r="E8" s="28">
+      <c r="E8" s="29">
         <f>D8*1.1</f>
         <v/>
       </c>
-      <c r="F8" s="28" t="n">
+      <c r="F8" s="29" t="n">
         <v>2640000</v>
       </c>
-      <c r="G8" s="29" t="n"/>
-      <c r="H8" s="29" t="n">
+      <c r="G8" s="30" t="n"/>
+      <c r="H8" s="30" t="n">
         <v>3000000</v>
       </c>
-      <c r="I8" s="29">
+      <c r="I8" s="30">
         <f>ROUND(H8*1.1/0.95,-1)</f>
         <v/>
       </c>
-      <c r="J8" s="28" t="n">
+      <c r="J8" s="29" t="n">
         <v>2577960</v>
       </c>
-      <c r="K8" s="28">
+      <c r="K8" s="29">
         <f>J8/1.1</f>
         <v/>
       </c>
-      <c r="L8" s="28" t="inlineStr">
+      <c r="L8" s="29" t="inlineStr">
         <is>
           <t>솔바텍지마켓</t>
         </is>
@@ -12356,30 +12735,30 @@
           <t xml:space="preserve"> 키패드(핸드헬드)</t>
         </is>
       </c>
-      <c r="D10" s="28" t="n">
+      <c r="D10" s="29" t="n">
         <v>1490000</v>
       </c>
-      <c r="E10" s="28">
+      <c r="E10" s="29">
         <f>D10*1.1</f>
         <v/>
       </c>
-      <c r="F10" s="28" t="n">
+      <c r="F10" s="29" t="n">
         <v>2750000</v>
       </c>
-      <c r="G10" s="28">
+      <c r="G10" s="29">
         <f>F10/110%</f>
         <v/>
       </c>
-      <c r="H10" s="28" t="n"/>
-      <c r="I10" s="28" t="n"/>
-      <c r="J10" s="28" t="n">
+      <c r="H10" s="29" t="n"/>
+      <c r="I10" s="29" t="n"/>
+      <c r="J10" s="29" t="n">
         <v>2750000</v>
       </c>
-      <c r="K10" s="28">
+      <c r="K10" s="29">
         <f>J10/1.1</f>
         <v/>
       </c>
-      <c r="L10" s="28" t="inlineStr">
+      <c r="L10" s="29" t="inlineStr">
         <is>
           <t>코스모스몰,더원시스</t>
         </is>
@@ -12550,7 +12929,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="I18" s="30" t="n"/>
+      <c r="I18" s="31" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Use simple arithmetic formulas instead of IF in the Zebra scanner sheet
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0164u4m2HzVL7yDN6jZnxUBp
</commit_message>
<xml_diff>
--- a/output/지브라_스캐너_옵션추가.xlsx
+++ b/output/지브라_스캐너_옵션추가.xlsx
@@ -9725,7 +9725,7 @@
     <col width="16" customWidth="1" style="16" min="19" max="19"/>
     <col width="14" customWidth="1" style="16" min="20" max="20"/>
     <col width="20" customWidth="1" style="16" min="21" max="21"/>
-    <col width="24" customWidth="1" style="16" min="22" max="22"/>
+    <col width="30" customWidth="1" style="16" min="22" max="22"/>
     <col width="16" customWidth="1" style="16" min="23" max="23"/>
     <col width="18" customWidth="1" style="16" min="24" max="24"/>
     <col width="20" customWidth="1" style="16" min="25" max="25"/>
@@ -9833,7 +9833,7 @@
       </c>
       <c r="V1" s="4" t="inlineStr">
         <is>
-          <t>타업체 케이블가(모르면 비움)</t>
+          <t>타업체 케이블가(포함이면 0, 모르면 18000)</t>
         </is>
       </c>
       <c r="W1" s="4" t="inlineStr">
@@ -9897,7 +9897,7 @@
         </is>
       </c>
       <c r="R2" s="22">
-        <f>IF(Q2="X",F2+18000,F2)</f>
+        <f>F2+18000</f>
         <v/>
       </c>
       <c r="S2" s="23" t="n"/>
@@ -9905,23 +9905,23 @@
       <c r="U2" s="25" t="n"/>
       <c r="V2" s="24" t="n"/>
       <c r="W2" s="22">
-        <f>IF(T2="","",IF(U2="O",T2,T2+IF(V2="",18000,V2)))</f>
+        <f>T2+V2</f>
         <v/>
       </c>
       <c r="X2" s="22">
-        <f>IF(OR(W2="",R2=""),"",R2-W2)</f>
+        <f>R2-W2</f>
         <v/>
       </c>
       <c r="Y2" s="22">
-        <f>IF(OR(D2="",R2=""),"",IF(Q2="X",D2+9000,D2))</f>
+        <f>D2+9000</f>
         <v/>
       </c>
       <c r="Z2" s="26">
-        <f>IF(Y2="","",1-Y2/(R2/110%))</f>
+        <f>1-(Y2/(R2/110%))</f>
         <v/>
       </c>
       <c r="AA2" s="26">
-        <f>IF(OR(Y2="",W2=""),"",1-Y2/(W2/110%))</f>
+        <f>1-(Y2/(W2/110%))</f>
         <v/>
       </c>
     </row>
@@ -9980,7 +9980,7 @@
         </is>
       </c>
       <c r="R3" s="22">
-        <f>IF(Q3="X",F3+18000,F3)</f>
+        <f>F3+18000</f>
         <v/>
       </c>
       <c r="S3" s="23" t="n"/>
@@ -9988,23 +9988,23 @@
       <c r="U3" s="25" t="n"/>
       <c r="V3" s="24" t="n"/>
       <c r="W3" s="22">
-        <f>IF(T3="","",IF(U3="O",T3,T3+IF(V3="",18000,V3)))</f>
+        <f>T3+V3</f>
         <v/>
       </c>
       <c r="X3" s="22">
-        <f>IF(OR(W3="",R3=""),"",R3-W3)</f>
+        <f>R3-W3</f>
         <v/>
       </c>
       <c r="Y3" s="22">
-        <f>IF(OR(D3="",R3=""),"",IF(Q3="X",D3+9000,D3))</f>
+        <f>D3+9000</f>
         <v/>
       </c>
       <c r="Z3" s="26">
-        <f>IF(Y3="","",1-Y3/(R3/110%))</f>
+        <f>1-(Y3/(R3/110%))</f>
         <v/>
       </c>
       <c r="AA3" s="26">
-        <f>IF(OR(Y3="",W3=""),"",1-Y3/(W3/110%))</f>
+        <f>1-(Y3/(W3/110%))</f>
         <v/>
       </c>
     </row>
@@ -10065,7 +10065,7 @@
         </is>
       </c>
       <c r="R4" s="22">
-        <f>IF(Q4="X",F4+18000,F4)</f>
+        <f>F4+18000</f>
         <v/>
       </c>
       <c r="S4" s="23" t="n"/>
@@ -10073,23 +10073,23 @@
       <c r="U4" s="25" t="n"/>
       <c r="V4" s="24" t="n"/>
       <c r="W4" s="22">
-        <f>IF(T4="","",IF(U4="O",T4,T4+IF(V4="",18000,V4)))</f>
+        <f>T4+V4</f>
         <v/>
       </c>
       <c r="X4" s="22">
-        <f>IF(OR(W4="",R4=""),"",R4-W4)</f>
+        <f>R4-W4</f>
         <v/>
       </c>
       <c r="Y4" s="22">
-        <f>IF(OR(D4="",R4=""),"",IF(Q4="X",D4+9000,D4))</f>
+        <f>D4+9000</f>
         <v/>
       </c>
       <c r="Z4" s="26">
-        <f>IF(Y4="","",1-Y4/(R4/110%))</f>
+        <f>1-(Y4/(R4/110%))</f>
         <v/>
       </c>
       <c r="AA4" s="26">
-        <f>IF(OR(Y4="",W4=""),"",1-Y4/(W4/110%))</f>
+        <f>1-(Y4/(W4/110%))</f>
         <v/>
       </c>
     </row>
@@ -10148,7 +10148,7 @@
         </is>
       </c>
       <c r="R5" s="22">
-        <f>IF(Q5="X",F5+18000,F5)</f>
+        <f>F5+18000</f>
         <v/>
       </c>
       <c r="S5" s="23" t="n"/>
@@ -10156,23 +10156,23 @@
       <c r="U5" s="25" t="n"/>
       <c r="V5" s="24" t="n"/>
       <c r="W5" s="22">
-        <f>IF(T5="","",IF(U5="O",T5,T5+IF(V5="",18000,V5)))</f>
+        <f>T5+V5</f>
         <v/>
       </c>
       <c r="X5" s="22">
-        <f>IF(OR(W5="",R5=""),"",R5-W5)</f>
+        <f>R5-W5</f>
         <v/>
       </c>
       <c r="Y5" s="22">
-        <f>IF(OR(D5="",R5=""),"",IF(Q5="X",D5+9000,D5))</f>
+        <f>D5+9000</f>
         <v/>
       </c>
       <c r="Z5" s="26">
-        <f>IF(Y5="","",1-Y5/(R5/110%))</f>
+        <f>1-(Y5/(R5/110%))</f>
         <v/>
       </c>
       <c r="AA5" s="26">
-        <f>IF(OR(Y5="",W5=""),"",1-Y5/(W5/110%))</f>
+        <f>1-(Y5/(W5/110%))</f>
         <v/>
       </c>
     </row>
@@ -10233,7 +10233,7 @@
         </is>
       </c>
       <c r="R6" s="22">
-        <f>IF(Q6="X",F6+18000,F6)</f>
+        <f>F6+18000</f>
         <v/>
       </c>
       <c r="S6" s="23" t="n"/>
@@ -10241,23 +10241,23 @@
       <c r="U6" s="25" t="n"/>
       <c r="V6" s="24" t="n"/>
       <c r="W6" s="22">
-        <f>IF(T6="","",IF(U6="O",T6,T6+IF(V6="",18000,V6)))</f>
+        <f>T6+V6</f>
         <v/>
       </c>
       <c r="X6" s="22">
-        <f>IF(OR(W6="",R6=""),"",R6-W6)</f>
+        <f>R6-W6</f>
         <v/>
       </c>
       <c r="Y6" s="22">
-        <f>IF(OR(D6="",R6=""),"",IF(Q6="X",D6+9000,D6))</f>
+        <f>D6+9000</f>
         <v/>
       </c>
       <c r="Z6" s="26">
-        <f>IF(Y6="","",1-Y6/(R6/110%))</f>
+        <f>1-(Y6/(R6/110%))</f>
         <v/>
       </c>
       <c r="AA6" s="26">
-        <f>IF(OR(Y6="",W6=""),"",1-Y6/(W6/110%))</f>
+        <f>1-(Y6/(W6/110%))</f>
         <v/>
       </c>
     </row>
@@ -10312,7 +10312,7 @@
         </is>
       </c>
       <c r="R7" s="22">
-        <f>IF(Q7="X",F7+18000,F7)</f>
+        <f>F7+18000</f>
         <v/>
       </c>
       <c r="S7" s="23" t="n"/>
@@ -10320,23 +10320,23 @@
       <c r="U7" s="25" t="n"/>
       <c r="V7" s="24" t="n"/>
       <c r="W7" s="22">
-        <f>IF(T7="","",IF(U7="O",T7,T7+IF(V7="",18000,V7)))</f>
+        <f>T7+V7</f>
         <v/>
       </c>
       <c r="X7" s="22">
-        <f>IF(OR(W7="",R7=""),"",R7-W7)</f>
+        <f>R7-W7</f>
         <v/>
       </c>
       <c r="Y7" s="22">
-        <f>IF(OR(D7="",R7=""),"",IF(Q7="X",D7+9000,D7))</f>
+        <f>D7+9000</f>
         <v/>
       </c>
       <c r="Z7" s="26">
-        <f>IF(Y7="","",1-Y7/(R7/110%))</f>
+        <f>1-(Y7/(R7/110%))</f>
         <v/>
       </c>
       <c r="AA7" s="26">
-        <f>IF(OR(Y7="",W7=""),"",1-Y7/(W7/110%))</f>
+        <f>1-(Y7/(W7/110%))</f>
         <v/>
       </c>
     </row>
@@ -10394,7 +10394,7 @@
         </is>
       </c>
       <c r="R8" s="22">
-        <f>IF(Q8="X",F8+18000,F8)</f>
+        <f>F8</f>
         <v/>
       </c>
       <c r="S8" s="23" t="n"/>
@@ -10402,23 +10402,23 @@
       <c r="U8" s="25" t="n"/>
       <c r="V8" s="24" t="n"/>
       <c r="W8" s="22">
-        <f>IF(T8="","",IF(U8="O",T8,T8+IF(V8="",18000,V8)))</f>
+        <f>T8+V8</f>
         <v/>
       </c>
       <c r="X8" s="22">
-        <f>IF(OR(W8="",R8=""),"",R8-W8)</f>
+        <f>R8-W8</f>
         <v/>
       </c>
       <c r="Y8" s="22">
-        <f>IF(OR(D8="",R8=""),"",IF(Q8="X",D8+9000,D8))</f>
+        <f>D8</f>
         <v/>
       </c>
       <c r="Z8" s="26">
-        <f>IF(Y8="","",1-Y8/(R8/110%))</f>
+        <f>1-(Y8/(R8/110%))</f>
         <v/>
       </c>
       <c r="AA8" s="26">
-        <f>IF(OR(Y8="",W8=""),"",1-Y8/(W8/110%))</f>
+        <f>1-(Y8/(W8/110%))</f>
         <v/>
       </c>
     </row>
@@ -10476,7 +10476,7 @@
         </is>
       </c>
       <c r="R9" s="22">
-        <f>IF(Q9="X",F9+18000,F9)</f>
+        <f>F9</f>
         <v/>
       </c>
       <c r="S9" s="23" t="n"/>
@@ -10484,23 +10484,23 @@
       <c r="U9" s="25" t="n"/>
       <c r="V9" s="24" t="n"/>
       <c r="W9" s="22">
-        <f>IF(T9="","",IF(U9="O",T9,T9+IF(V9="",18000,V9)))</f>
+        <f>T9+V9</f>
         <v/>
       </c>
       <c r="X9" s="22">
-        <f>IF(OR(W9="",R9=""),"",R9-W9)</f>
+        <f>R9-W9</f>
         <v/>
       </c>
       <c r="Y9" s="22">
-        <f>IF(OR(D9="",R9=""),"",IF(Q9="X",D9+9000,D9))</f>
+        <f>D9</f>
         <v/>
       </c>
       <c r="Z9" s="26">
-        <f>IF(Y9="","",1-Y9/(R9/110%))</f>
+        <f>1-(Y9/(R9/110%))</f>
         <v/>
       </c>
       <c r="AA9" s="26">
-        <f>IF(OR(Y9="",W9=""),"",1-Y9/(W9/110%))</f>
+        <f>1-(Y9/(W9/110%))</f>
         <v/>
       </c>
     </row>
@@ -10555,7 +10555,7 @@
         </is>
       </c>
       <c r="R10" s="22">
-        <f>IF(Q10="X",F10+18000,F10)</f>
+        <f>F10</f>
         <v/>
       </c>
       <c r="S10" s="23" t="n"/>
@@ -10563,23 +10563,23 @@
       <c r="U10" s="25" t="n"/>
       <c r="V10" s="24" t="n"/>
       <c r="W10" s="22">
-        <f>IF(T10="","",IF(U10="O",T10,T10+IF(V10="",18000,V10)))</f>
+        <f>T10+V10</f>
         <v/>
       </c>
       <c r="X10" s="22">
-        <f>IF(OR(W10="",R10=""),"",R10-W10)</f>
+        <f>R10-W10</f>
         <v/>
       </c>
       <c r="Y10" s="22">
-        <f>IF(OR(D10="",R10=""),"",IF(Q10="X",D10+9000,D10))</f>
+        <f>D10</f>
         <v/>
       </c>
       <c r="Z10" s="26">
-        <f>IF(Y10="","",1-Y10/(R10/110%))</f>
+        <f>1-(Y10/(R10/110%))</f>
         <v/>
       </c>
       <c r="AA10" s="26">
-        <f>IF(OR(Y10="",W10=""),"",1-Y10/(W10/110%))</f>
+        <f>1-(Y10/(W10/110%))</f>
         <v/>
       </c>
     </row>
@@ -10637,7 +10637,7 @@
         </is>
       </c>
       <c r="R11" s="22">
-        <f>IF(Q11="X",F11+18000,F11)</f>
+        <f>F11+18000</f>
         <v/>
       </c>
       <c r="S11" s="23" t="n"/>
@@ -10645,23 +10645,23 @@
       <c r="U11" s="25" t="n"/>
       <c r="V11" s="24" t="n"/>
       <c r="W11" s="22">
-        <f>IF(T11="","",IF(U11="O",T11,T11+IF(V11="",18000,V11)))</f>
+        <f>T11+V11</f>
         <v/>
       </c>
       <c r="X11" s="22">
-        <f>IF(OR(W11="",R11=""),"",R11-W11)</f>
+        <f>R11-W11</f>
         <v/>
       </c>
       <c r="Y11" s="22">
-        <f>IF(OR(D11="",R11=""),"",IF(Q11="X",D11+9000,D11))</f>
+        <f>D11+9000</f>
         <v/>
       </c>
       <c r="Z11" s="26">
-        <f>IF(Y11="","",1-Y11/(R11/110%))</f>
+        <f>1-(Y11/(R11/110%))</f>
         <v/>
       </c>
       <c r="AA11" s="26">
-        <f>IF(OR(Y11="",W11=""),"",1-Y11/(W11/110%))</f>
+        <f>1-(Y11/(W11/110%))</f>
         <v/>
       </c>
     </row>
@@ -10727,26 +10727,8 @@
       <c r="T12" s="24" t="n"/>
       <c r="U12" s="25" t="n"/>
       <c r="V12" s="24" t="n"/>
-      <c r="W12" s="22">
-        <f>IF(T12="","",IF(U12="O",T12,T12+IF(V12="",18000,V12)))</f>
-        <v/>
-      </c>
-      <c r="X12" s="22">
-        <f>IF(OR(W12="",R12=""),"",R12-W12)</f>
-        <v/>
-      </c>
-      <c r="Y12" s="22">
-        <f>IF(OR(D12="",R12=""),"",IF(Q12="X",D12+9000,D12))</f>
-        <v/>
-      </c>
-      <c r="Z12" s="26">
-        <f>IF(Y12="","",1-Y12/(R12/110%))</f>
-        <v/>
-      </c>
-      <c r="AA12" s="26">
-        <f>IF(OR(Y12="",W12=""),"",1-Y12/(W12/110%))</f>
-        <v/>
-      </c>
+      <c r="W12" s="22" t="n"/>
+      <c r="X12" s="22" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="0" t="n">
@@ -10805,26 +10787,8 @@
       <c r="T13" s="24" t="n"/>
       <c r="U13" s="25" t="n"/>
       <c r="V13" s="24" t="n"/>
-      <c r="W13" s="22">
-        <f>IF(T13="","",IF(U13="O",T13,T13+IF(V13="",18000,V13)))</f>
-        <v/>
-      </c>
-      <c r="X13" s="22">
-        <f>IF(OR(W13="",R13=""),"",R13-W13)</f>
-        <v/>
-      </c>
-      <c r="Y13" s="22">
-        <f>IF(OR(D13="",R13=""),"",IF(Q13="X",D13+9000,D13))</f>
-        <v/>
-      </c>
-      <c r="Z13" s="26">
-        <f>IF(Y13="","",1-Y13/(R13/110%))</f>
-        <v/>
-      </c>
-      <c r="AA13" s="26">
-        <f>IF(OR(Y13="",W13=""),"",1-Y13/(W13/110%))</f>
-        <v/>
-      </c>
+      <c r="W13" s="22" t="n"/>
+      <c r="X13" s="22" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="0" t="n">
@@ -10883,7 +10847,7 @@
         </is>
       </c>
       <c r="R14" s="22">
-        <f>IF(Q14="X",F14+18000,F14)</f>
+        <f>F14</f>
         <v/>
       </c>
       <c r="S14" s="23" t="n"/>
@@ -10891,23 +10855,23 @@
       <c r="U14" s="25" t="n"/>
       <c r="V14" s="24" t="n"/>
       <c r="W14" s="22">
-        <f>IF(T14="","",IF(U14="O",T14,T14+IF(V14="",18000,V14)))</f>
+        <f>T14+V14</f>
         <v/>
       </c>
       <c r="X14" s="22">
-        <f>IF(OR(W14="",R14=""),"",R14-W14)</f>
+        <f>R14-W14</f>
         <v/>
       </c>
       <c r="Y14" s="22">
-        <f>IF(OR(D14="",R14=""),"",IF(Q14="X",D14+9000,D14))</f>
+        <f>D14</f>
         <v/>
       </c>
       <c r="Z14" s="26">
-        <f>IF(Y14="","",1-Y14/(R14/110%))</f>
+        <f>1-(Y14/(R14/110%))</f>
         <v/>
       </c>
       <c r="AA14" s="26">
-        <f>IF(OR(Y14="",W14=""),"",1-Y14/(W14/110%))</f>
+        <f>1-(Y14/(W14/110%))</f>
         <v/>
       </c>
     </row>
@@ -10968,7 +10932,7 @@
         </is>
       </c>
       <c r="R15" s="22">
-        <f>IF(Q15="X",F15+18000,F15)</f>
+        <f>F15+18000</f>
         <v/>
       </c>
       <c r="S15" s="23" t="n"/>
@@ -10976,23 +10940,23 @@
       <c r="U15" s="25" t="n"/>
       <c r="V15" s="24" t="n"/>
       <c r="W15" s="22">
-        <f>IF(T15="","",IF(U15="O",T15,T15+IF(V15="",18000,V15)))</f>
+        <f>T15+V15</f>
         <v/>
       </c>
       <c r="X15" s="22">
-        <f>IF(OR(W15="",R15=""),"",R15-W15)</f>
+        <f>R15-W15</f>
         <v/>
       </c>
       <c r="Y15" s="22">
-        <f>IF(OR(D15="",R15=""),"",IF(Q15="X",D15+9000,D15))</f>
+        <f>D15+9000</f>
         <v/>
       </c>
       <c r="Z15" s="26">
-        <f>IF(Y15="","",1-Y15/(R15/110%))</f>
+        <f>1-(Y15/(R15/110%))</f>
         <v/>
       </c>
       <c r="AA15" s="26">
-        <f>IF(OR(Y15="",W15=""),"",1-Y15/(W15/110%))</f>
+        <f>1-(Y15/(W15/110%))</f>
         <v/>
       </c>
     </row>
@@ -11050,7 +11014,7 @@
         </is>
       </c>
       <c r="R16" s="22">
-        <f>IF(Q16="X",F16+18000,F16)</f>
+        <f>F16</f>
         <v/>
       </c>
       <c r="S16" s="23" t="n"/>
@@ -11058,23 +11022,23 @@
       <c r="U16" s="25" t="n"/>
       <c r="V16" s="24" t="n"/>
       <c r="W16" s="22">
-        <f>IF(T16="","",IF(U16="O",T16,T16+IF(V16="",18000,V16)))</f>
+        <f>T16+V16</f>
         <v/>
       </c>
       <c r="X16" s="22">
-        <f>IF(OR(W16="",R16=""),"",R16-W16)</f>
+        <f>R16-W16</f>
         <v/>
       </c>
       <c r="Y16" s="22">
-        <f>IF(OR(D16="",R16=""),"",IF(Q16="X",D16+9000,D16))</f>
+        <f>D16</f>
         <v/>
       </c>
       <c r="Z16" s="26">
-        <f>IF(Y16="","",1-Y16/(R16/110%))</f>
+        <f>1-(Y16/(R16/110%))</f>
         <v/>
       </c>
       <c r="AA16" s="26">
-        <f>IF(OR(Y16="",W16=""),"",1-Y16/(W16/110%))</f>
+        <f>1-(Y16/(W16/110%))</f>
         <v/>
       </c>
     </row>
@@ -11129,7 +11093,7 @@
         </is>
       </c>
       <c r="R17" s="22">
-        <f>IF(Q17="X",F17+18000,F17)</f>
+        <f>F17</f>
         <v/>
       </c>
       <c r="S17" s="23" t="n"/>
@@ -11137,23 +11101,23 @@
       <c r="U17" s="25" t="n"/>
       <c r="V17" s="24" t="n"/>
       <c r="W17" s="22">
-        <f>IF(T17="","",IF(U17="O",T17,T17+IF(V17="",18000,V17)))</f>
+        <f>T17+V17</f>
         <v/>
       </c>
       <c r="X17" s="22">
-        <f>IF(OR(W17="",R17=""),"",R17-W17)</f>
+        <f>R17-W17</f>
         <v/>
       </c>
       <c r="Y17" s="22">
-        <f>IF(OR(D17="",R17=""),"",IF(Q17="X",D17+9000,D17))</f>
+        <f>D17</f>
         <v/>
       </c>
       <c r="Z17" s="26">
-        <f>IF(Y17="","",1-Y17/(R17/110%))</f>
+        <f>1-(Y17/(R17/110%))</f>
         <v/>
       </c>
       <c r="AA17" s="26">
-        <f>IF(OR(Y17="",W17=""),"",1-Y17/(W17/110%))</f>
+        <f>1-(Y17/(W17/110%))</f>
         <v/>
       </c>
     </row>
@@ -11211,7 +11175,7 @@
         </is>
       </c>
       <c r="R18" s="22">
-        <f>IF(Q18="X",F18+18000,F18)</f>
+        <f>F18</f>
         <v/>
       </c>
       <c r="S18" s="23" t="n"/>
@@ -11219,23 +11183,23 @@
       <c r="U18" s="25" t="n"/>
       <c r="V18" s="24" t="n"/>
       <c r="W18" s="22">
-        <f>IF(T18="","",IF(U18="O",T18,T18+IF(V18="",18000,V18)))</f>
+        <f>T18+V18</f>
         <v/>
       </c>
       <c r="X18" s="22">
-        <f>IF(OR(W18="",R18=""),"",R18-W18)</f>
+        <f>R18-W18</f>
         <v/>
       </c>
       <c r="Y18" s="22">
-        <f>IF(OR(D18="",R18=""),"",IF(Q18="X",D18+9000,D18))</f>
+        <f>D18</f>
         <v/>
       </c>
       <c r="Z18" s="26">
-        <f>IF(Y18="","",1-Y18/(R18/110%))</f>
+        <f>1-(Y18/(R18/110%))</f>
         <v/>
       </c>
       <c r="AA18" s="26">
-        <f>IF(OR(Y18="",W18=""),"",1-Y18/(W18/110%))</f>
+        <f>1-(Y18/(W18/110%))</f>
         <v/>
       </c>
     </row>
@@ -11293,7 +11257,7 @@
         </is>
       </c>
       <c r="R19" s="22">
-        <f>IF(Q19="X",F19+18000,F19)</f>
+        <f>F19</f>
         <v/>
       </c>
       <c r="S19" s="23" t="n"/>
@@ -11301,23 +11265,23 @@
       <c r="U19" s="25" t="n"/>
       <c r="V19" s="24" t="n"/>
       <c r="W19" s="22">
-        <f>IF(T19="","",IF(U19="O",T19,T19+IF(V19="",18000,V19)))</f>
+        <f>T19+V19</f>
         <v/>
       </c>
       <c r="X19" s="22">
-        <f>IF(OR(W19="",R19=""),"",R19-W19)</f>
+        <f>R19-W19</f>
         <v/>
       </c>
       <c r="Y19" s="22">
-        <f>IF(OR(D19="",R19=""),"",IF(Q19="X",D19+9000,D19))</f>
+        <f>D19</f>
         <v/>
       </c>
       <c r="Z19" s="26">
-        <f>IF(Y19="","",1-Y19/(R19/110%))</f>
+        <f>1-(Y19/(R19/110%))</f>
         <v/>
       </c>
       <c r="AA19" s="26">
-        <f>IF(OR(Y19="",W19=""),"",1-Y19/(W19/110%))</f>
+        <f>1-(Y19/(W19/110%))</f>
         <v/>
       </c>
     </row>
@@ -11372,7 +11336,7 @@
         </is>
       </c>
       <c r="R20" s="22">
-        <f>IF(Q20="X",F20+18000,F20)</f>
+        <f>F20</f>
         <v/>
       </c>
       <c r="S20" s="23" t="n"/>
@@ -11380,23 +11344,23 @@
       <c r="U20" s="25" t="n"/>
       <c r="V20" s="24" t="n"/>
       <c r="W20" s="22">
-        <f>IF(T20="","",IF(U20="O",T20,T20+IF(V20="",18000,V20)))</f>
+        <f>T20+V20</f>
         <v/>
       </c>
       <c r="X20" s="22">
-        <f>IF(OR(W20="",R20=""),"",R20-W20)</f>
+        <f>R20-W20</f>
         <v/>
       </c>
       <c r="Y20" s="22">
-        <f>IF(OR(D20="",R20=""),"",IF(Q20="X",D20+9000,D20))</f>
+        <f>D20</f>
         <v/>
       </c>
       <c r="Z20" s="26">
-        <f>IF(Y20="","",1-Y20/(R20/110%))</f>
+        <f>1-(Y20/(R20/110%))</f>
         <v/>
       </c>
       <c r="AA20" s="26">
-        <f>IF(OR(Y20="",W20=""),"",1-Y20/(W20/110%))</f>
+        <f>1-(Y20/(W20/110%))</f>
         <v/>
       </c>
     </row>
@@ -11451,7 +11415,7 @@
         </is>
       </c>
       <c r="R21" s="22">
-        <f>IF(Q21="X",F21+18000,F21)</f>
+        <f>F21</f>
         <v/>
       </c>
       <c r="S21" s="23" t="n"/>
@@ -11459,23 +11423,23 @@
       <c r="U21" s="25" t="n"/>
       <c r="V21" s="24" t="n"/>
       <c r="W21" s="22">
-        <f>IF(T21="","",IF(U21="O",T21,T21+IF(V21="",18000,V21)))</f>
+        <f>T21+V21</f>
         <v/>
       </c>
       <c r="X21" s="22">
-        <f>IF(OR(W21="",R21=""),"",R21-W21)</f>
+        <f>R21-W21</f>
         <v/>
       </c>
       <c r="Y21" s="22">
-        <f>IF(OR(D21="",R21=""),"",IF(Q21="X",D21+9000,D21))</f>
+        <f>D21</f>
         <v/>
       </c>
       <c r="Z21" s="26">
-        <f>IF(Y21="","",1-Y21/(R21/110%))</f>
+        <f>1-(Y21/(R21/110%))</f>
         <v/>
       </c>
       <c r="AA21" s="26">
-        <f>IF(OR(Y21="",W21=""),"",1-Y21/(W21/110%))</f>
+        <f>1-(Y21/(W21/110%))</f>
         <v/>
       </c>
     </row>
@@ -11534,7 +11498,7 @@
         </is>
       </c>
       <c r="R22" s="22">
-        <f>IF(Q22="X",F22+18000,F22)</f>
+        <f>F22+18000</f>
         <v/>
       </c>
       <c r="S22" s="23" t="n"/>
@@ -11542,23 +11506,23 @@
       <c r="U22" s="25" t="n"/>
       <c r="V22" s="24" t="n"/>
       <c r="W22" s="22">
-        <f>IF(T22="","",IF(U22="O",T22,T22+IF(V22="",18000,V22)))</f>
+        <f>T22+V22</f>
         <v/>
       </c>
       <c r="X22" s="22">
-        <f>IF(OR(W22="",R22=""),"",R22-W22)</f>
+        <f>R22-W22</f>
         <v/>
       </c>
       <c r="Y22" s="22">
-        <f>IF(OR(D22="",R22=""),"",IF(Q22="X",D22+9000,D22))</f>
+        <f>D22+9000</f>
         <v/>
       </c>
       <c r="Z22" s="26">
-        <f>IF(Y22="","",1-Y22/(R22/110%))</f>
+        <f>1-(Y22/(R22/110%))</f>
         <v/>
       </c>
       <c r="AA22" s="26">
-        <f>IF(OR(Y22="",W22=""),"",1-Y22/(W22/110%))</f>
+        <f>1-(Y22/(W22/110%))</f>
         <v/>
       </c>
     </row>
@@ -11616,7 +11580,7 @@
         </is>
       </c>
       <c r="R23" s="22">
-        <f>IF(Q23="X",F23+18000,F23)</f>
+        <f>F23</f>
         <v/>
       </c>
       <c r="S23" s="23" t="n"/>
@@ -11624,23 +11588,23 @@
       <c r="U23" s="25" t="n"/>
       <c r="V23" s="24" t="n"/>
       <c r="W23" s="22">
-        <f>IF(T23="","",IF(U23="O",T23,T23+IF(V23="",18000,V23)))</f>
+        <f>T23+V23</f>
         <v/>
       </c>
       <c r="X23" s="22">
-        <f>IF(OR(W23="",R23=""),"",R23-W23)</f>
+        <f>R23-W23</f>
         <v/>
       </c>
       <c r="Y23" s="22">
-        <f>IF(OR(D23="",R23=""),"",IF(Q23="X",D23+9000,D23))</f>
+        <f>D23</f>
         <v/>
       </c>
       <c r="Z23" s="26">
-        <f>IF(Y23="","",1-Y23/(R23/110%))</f>
+        <f>1-(Y23/(R23/110%))</f>
         <v/>
       </c>
       <c r="AA23" s="26">
-        <f>IF(OR(Y23="",W23=""),"",1-Y23/(W23/110%))</f>
+        <f>1-(Y23/(W23/110%))</f>
         <v/>
       </c>
     </row>
@@ -11687,7 +11651,7 @@
         </is>
       </c>
       <c r="R24" s="22">
-        <f>IF(Q24="X",F24+18000,F24)</f>
+        <f>F24+18000</f>
         <v/>
       </c>
       <c r="S24" s="23" t="n"/>
@@ -11695,23 +11659,23 @@
       <c r="U24" s="25" t="n"/>
       <c r="V24" s="24" t="n"/>
       <c r="W24" s="22">
-        <f>IF(T24="","",IF(U24="O",T24,T24+IF(V24="",18000,V24)))</f>
+        <f>T24+V24</f>
         <v/>
       </c>
       <c r="X24" s="22">
-        <f>IF(OR(W24="",R24=""),"",R24-W24)</f>
+        <f>R24-W24</f>
         <v/>
       </c>
       <c r="Y24" s="22">
-        <f>IF(OR(D24="",R24=""),"",IF(Q24="X",D24+9000,D24))</f>
+        <f>D24+9000</f>
         <v/>
       </c>
       <c r="Z24" s="26">
-        <f>IF(Y24="","",1-Y24/(R24/110%))</f>
+        <f>1-(Y24/(R24/110%))</f>
         <v/>
       </c>
       <c r="AA24" s="26">
-        <f>IF(OR(Y24="",W24=""),"",1-Y24/(W24/110%))</f>
+        <f>1-(Y24/(W24/110%))</f>
         <v/>
       </c>
     </row>
@@ -11758,7 +11722,7 @@
         </is>
       </c>
       <c r="R25" s="22">
-        <f>IF(Q25="X",F25+18000,F25)</f>
+        <f>F25+18000</f>
         <v/>
       </c>
       <c r="S25" s="23" t="n"/>
@@ -11766,23 +11730,23 @@
       <c r="U25" s="25" t="n"/>
       <c r="V25" s="24" t="n"/>
       <c r="W25" s="22">
-        <f>IF(T25="","",IF(U25="O",T25,T25+IF(V25="",18000,V25)))</f>
+        <f>T25+V25</f>
         <v/>
       </c>
       <c r="X25" s="22">
-        <f>IF(OR(W25="",R25=""),"",R25-W25)</f>
+        <f>R25-W25</f>
         <v/>
       </c>
       <c r="Y25" s="22">
-        <f>IF(OR(D25="",R25=""),"",IF(Q25="X",D25+9000,D25))</f>
+        <f>D25+9000</f>
         <v/>
       </c>
       <c r="Z25" s="26">
-        <f>IF(Y25="","",1-Y25/(R25/110%))</f>
+        <f>1-(Y25/(R25/110%))</f>
         <v/>
       </c>
       <c r="AA25" s="26">
-        <f>IF(OR(Y25="",W25=""),"",1-Y25/(W25/110%))</f>
+        <f>1-(Y25/(W25/110%))</f>
         <v/>
       </c>
     </row>
@@ -11829,7 +11793,7 @@
         </is>
       </c>
       <c r="R26" s="22">
-        <f>IF(Q26="X",F26+18000,F26)</f>
+        <f>F26+18000</f>
         <v/>
       </c>
       <c r="S26" s="23" t="n"/>
@@ -11837,23 +11801,23 @@
       <c r="U26" s="25" t="n"/>
       <c r="V26" s="24" t="n"/>
       <c r="W26" s="22">
-        <f>IF(T26="","",IF(U26="O",T26,T26+IF(V26="",18000,V26)))</f>
+        <f>T26+V26</f>
         <v/>
       </c>
       <c r="X26" s="22">
-        <f>IF(OR(W26="",R26=""),"",R26-W26)</f>
+        <f>R26-W26</f>
         <v/>
       </c>
       <c r="Y26" s="22">
-        <f>IF(OR(D26="",R26=""),"",IF(Q26="X",D26+9000,D26))</f>
+        <f>D26+9000</f>
         <v/>
       </c>
       <c r="Z26" s="26">
-        <f>IF(Y26="","",1-Y26/(R26/110%))</f>
+        <f>1-(Y26/(R26/110%))</f>
         <v/>
       </c>
       <c r="AA26" s="26">
-        <f>IF(OR(Y26="",W26=""),"",1-Y26/(W26/110%))</f>
+        <f>1-(Y26/(W26/110%))</f>
         <v/>
       </c>
     </row>
@@ -11902,26 +11866,8 @@
       <c r="T27" s="24" t="n"/>
       <c r="U27" s="25" t="n"/>
       <c r="V27" s="24" t="n"/>
-      <c r="W27" s="22">
-        <f>IF(T27="","",IF(U27="O",T27,T27+IF(V27="",18000,V27)))</f>
-        <v/>
-      </c>
-      <c r="X27" s="22">
-        <f>IF(OR(W27="",R27=""),"",R27-W27)</f>
-        <v/>
-      </c>
-      <c r="Y27" s="22">
-        <f>IF(OR(D27="",R27=""),"",IF(Q27="X",D27+9000,D27))</f>
-        <v/>
-      </c>
-      <c r="Z27" s="26">
-        <f>IF(Y27="","",1-Y27/(R27/110%))</f>
-        <v/>
-      </c>
-      <c r="AA27" s="26">
-        <f>IF(OR(Y27="",W27=""),"",1-Y27/(W27/110%))</f>
-        <v/>
-      </c>
+      <c r="W27" s="22" t="n"/>
+      <c r="X27" s="22" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="0" t="n">
@@ -11968,26 +11914,8 @@
       <c r="T28" s="24" t="n"/>
       <c r="U28" s="25" t="n"/>
       <c r="V28" s="24" t="n"/>
-      <c r="W28" s="22">
-        <f>IF(T28="","",IF(U28="O",T28,T28+IF(V28="",18000,V28)))</f>
-        <v/>
-      </c>
-      <c r="X28" s="22">
-        <f>IF(OR(W28="",R28=""),"",R28-W28)</f>
-        <v/>
-      </c>
-      <c r="Y28" s="22">
-        <f>IF(OR(D28="",R28=""),"",IF(Q28="X",D28+9000,D28))</f>
-        <v/>
-      </c>
-      <c r="Z28" s="26">
-        <f>IF(Y28="","",1-Y28/(R28/110%))</f>
-        <v/>
-      </c>
-      <c r="AA28" s="26">
-        <f>IF(OR(Y28="",W28=""),"",1-Y28/(W28/110%))</f>
-        <v/>
-      </c>
+      <c r="W28" s="22" t="n"/>
+      <c r="X28" s="22" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="0" t="n">
@@ -12034,26 +11962,8 @@
       <c r="T29" s="24" t="n"/>
       <c r="U29" s="25" t="n"/>
       <c r="V29" s="24" t="n"/>
-      <c r="W29" s="22">
-        <f>IF(T29="","",IF(U29="O",T29,T29+IF(V29="",18000,V29)))</f>
-        <v/>
-      </c>
-      <c r="X29" s="22">
-        <f>IF(OR(W29="",R29=""),"",R29-W29)</f>
-        <v/>
-      </c>
-      <c r="Y29" s="22">
-        <f>IF(OR(D29="",R29=""),"",IF(Q29="X",D29+9000,D29))</f>
-        <v/>
-      </c>
-      <c r="Z29" s="26">
-        <f>IF(Y29="","",1-Y29/(R29/110%))</f>
-        <v/>
-      </c>
-      <c r="AA29" s="26">
-        <f>IF(OR(Y29="",W29=""),"",1-Y29/(W29/110%))</f>
-        <v/>
-      </c>
+      <c r="W29" s="22" t="n"/>
+      <c r="X29" s="22" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="0" t="n">
@@ -12100,26 +12010,8 @@
       <c r="T30" s="24" t="n"/>
       <c r="U30" s="25" t="n"/>
       <c r="V30" s="24" t="n"/>
-      <c r="W30" s="22">
-        <f>IF(T30="","",IF(U30="O",T30,T30+IF(V30="",18000,V30)))</f>
-        <v/>
-      </c>
-      <c r="X30" s="22">
-        <f>IF(OR(W30="",R30=""),"",R30-W30)</f>
-        <v/>
-      </c>
-      <c r="Y30" s="22">
-        <f>IF(OR(D30="",R30=""),"",IF(Q30="X",D30+9000,D30))</f>
-        <v/>
-      </c>
-      <c r="Z30" s="26">
-        <f>IF(Y30="","",1-Y30/(R30/110%))</f>
-        <v/>
-      </c>
-      <c r="AA30" s="26">
-        <f>IF(OR(Y30="",W30=""),"",1-Y30/(W30/110%))</f>
-        <v/>
-      </c>
+      <c r="W30" s="22" t="n"/>
+      <c r="X30" s="22" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="0" t="n">
@@ -12166,26 +12058,8 @@
       <c r="T31" s="24" t="n"/>
       <c r="U31" s="25" t="n"/>
       <c r="V31" s="24" t="n"/>
-      <c r="W31" s="22">
-        <f>IF(T31="","",IF(U31="O",T31,T31+IF(V31="",18000,V31)))</f>
-        <v/>
-      </c>
-      <c r="X31" s="22">
-        <f>IF(OR(W31="",R31=""),"",R31-W31)</f>
-        <v/>
-      </c>
-      <c r="Y31" s="22">
-        <f>IF(OR(D31="",R31=""),"",IF(Q31="X",D31+9000,D31))</f>
-        <v/>
-      </c>
-      <c r="Z31" s="26">
-        <f>IF(Y31="","",1-Y31/(R31/110%))</f>
-        <v/>
-      </c>
-      <c r="AA31" s="26">
-        <f>IF(OR(Y31="",W31=""),"",1-Y31/(W31/110%))</f>
-        <v/>
-      </c>
+      <c r="W31" s="22" t="n"/>
+      <c r="X31" s="22" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="1">

</xml_diff>

<commit_message>
Fill margin formulas for DS9308, DS8178, LI4278
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0164u4m2HzVL7yDN6jZnxUBp
</commit_message>
<xml_diff>
--- a/output/지브라_스캐너_옵션추가.xlsx
+++ b/output/지브라_스캐너_옵션추가.xlsx
@@ -10923,8 +10923,14 @@
           <t>에이치앤아이디지탈</t>
         </is>
       </c>
-      <c r="M24" s="3" t="n"/>
-      <c r="N24" s="3" t="n"/>
+      <c r="M24" s="3">
+        <f>1-(D24/G24)</f>
+        <v/>
+      </c>
+      <c r="N24" s="3">
+        <f>1-(D24/K24)</f>
+        <v/>
+      </c>
       <c r="P24" s="16" t="inlineStr">
         <is>
           <t>RS232C (+24,200원)
@@ -10994,8 +11000,14 @@
           <t>착한라벨</t>
         </is>
       </c>
-      <c r="M25" s="3" t="n"/>
-      <c r="N25" s="3" t="n"/>
+      <c r="M25" s="3">
+        <f>1-(D25/G25)</f>
+        <v/>
+      </c>
+      <c r="N25" s="3">
+        <f>1-(D25/K25)</f>
+        <v/>
+      </c>
       <c r="P25" s="16" t="inlineStr">
         <is>
           <t>RS232C (+24,200원)
@@ -11065,8 +11077,14 @@
           <t>더원시스</t>
         </is>
       </c>
-      <c r="M26" s="3" t="n"/>
-      <c r="N26" s="3" t="n"/>
+      <c r="M26" s="3">
+        <f>1-(D26/G26)</f>
+        <v/>
+      </c>
+      <c r="N26" s="3">
+        <f>1-(D26/K26)</f>
+        <v/>
+      </c>
       <c r="P26" s="16" t="inlineStr">
         <is>
           <t>RS232C (+24,200원)

</xml_diff>